<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-13)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -1284,6 +1284,16 @@
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
         </is>
       </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Hero Motors Ltd</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/hero-motors-ipo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-14)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AR8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,32 +699,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lumino Industries Limited</t>
+          <t>Nopaperforms Solutions Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>UDRHP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Diversified Industrials</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -733,31 +728,31 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>202.6</v>
+        <v>115.65</v>
       </c>
       <c r="R2" t="n">
-        <v>0.05</v>
+        <v>25.24</v>
       </c>
       <c r="S2" t="n">
-        <v>160</v>
+        <v>1</v>
       </c>
       <c r="T2" t="n">
-        <v>28.42</v>
+        <v>408.67</v>
       </c>
       <c r="U2" t="n">
-        <v>7.66</v>
+        <v>0.83</v>
+      </c>
+      <c r="V2" t="n">
+        <v>6.58</v>
       </c>
       <c r="W2" t="n">
-        <v>24.61</v>
-      </c>
-      <c r="X2" t="n">
-        <v>25.75</v>
+        <v>33.12</v>
       </c>
       <c r="AA2" t="n">
-        <v>48.7</v>
+        <v>48</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -766,7 +761,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -777,56 +772,19 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lumino-industries-limited-prospectus_104288.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/nopaperforms-solutions-limited-udrhp-1_104427.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Lumino%20Industries%20Limited%20-%20Abridged%20Prospectus_p.pdf</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>Lumino Industries Ltd.</t>
-        </is>
-      </c>
-      <c r="AI2" t="n">
-        <v>3286</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>21.93</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>71.97</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>50.48</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>33.18</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>130.83</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>27.7</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>34.15</v>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/lumino-industries-ltd</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/NOPAPERFORMS%20SOLUTIONS%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nopaperforms Solutions Limited</t>
+          <t>M K C Agro Fresh Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -836,7 +794,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -846,7 +804,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -855,31 +818,37 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q3" t="n">
-        <v>115.65</v>
+        <v>521.53</v>
       </c>
       <c r="R3" t="n">
-        <v>25.24</v>
+        <v>6.38</v>
       </c>
       <c r="S3" t="n">
-        <v>1</v>
+        <v>22.11</v>
       </c>
       <c r="T3" t="n">
-        <v>408.67</v>
+        <v>14.09</v>
       </c>
       <c r="U3" t="n">
-        <v>0.83</v>
+        <v>4.24</v>
       </c>
       <c r="V3" t="n">
-        <v>6.58</v>
+        <v>7.49</v>
       </c>
       <c r="W3" t="n">
-        <v>33.12</v>
+        <v>15.92</v>
+      </c>
+      <c r="X3" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1.47</v>
       </c>
       <c r="AA3" t="n">
-        <v>48</v>
+        <v>30.8</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -888,7 +857,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -899,44 +868,44 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/nopaperforms-solutions-limited-udrhp-1_104427.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/m-k-c-agro-fresh-limited-drhp_104430.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/NOPAPERFORMS%20SOLUTIONS%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/M%20K%20C%20AGRO%20FRESH%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M K C Agro Fresh Limited</t>
+          <t>Torrent Gas Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>UDRHP</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Oil &amp; Gas</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -944,47 +913,35 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="N4" t="n">
-        <v>10</v>
+      <c r="L4" t="n">
+        <v>335000000</v>
       </c>
       <c r="Q4" t="n">
-        <v>521.53</v>
+        <v>1396.78</v>
       </c>
       <c r="R4" t="n">
-        <v>6.38</v>
+        <v>-76.45999999999999</v>
       </c>
       <c r="S4" t="n">
-        <v>22.11</v>
+        <v>55.68</v>
       </c>
       <c r="T4" t="n">
-        <v>14.09</v>
+        <v>-80.18000000000001</v>
       </c>
       <c r="U4" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="V4" t="n">
-        <v>7.49</v>
-      </c>
-      <c r="W4" t="n">
-        <v>15.92</v>
-      </c>
-      <c r="X4" t="n">
-        <v>9.880000000000001</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>1.47</v>
+        <v>3.99</v>
       </c>
       <c r="AA4" t="n">
-        <v>30.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -995,29 +952,29 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/m-k-c-agro-fresh-limited-drhp_104430.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/M%20K%20C%20AGRO%20FRESH%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Torrent Gas Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1027,43 +984,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>335000000</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>1396.78</v>
-      </c>
-      <c r="R5" t="n">
-        <v>-76.45999999999999</v>
-      </c>
-      <c r="S5" t="n">
-        <v>55.68</v>
-      </c>
-      <c r="T5" t="n">
-        <v>-80.18000000000001</v>
-      </c>
-      <c r="U5" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>8.199999999999999</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1073,25 +999,20 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>Glass Wall Systems (India) Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1101,12 +1022,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1121,7 +1042,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -1132,29 +1053,29 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Glass Wall Systems (India) Limited</t>
+          <t>Incred Holdings Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Corrigendum</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1169,7 +1090,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1180,19 +1101,19 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Incred Holdings Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1207,7 +1128,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1228,68 +1154,15 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Hero Motors Limited</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Corrigendum</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
         </is>
       </c>
-      <c r="AH9" t="inlineStr">
+      <c r="AH8" t="inlineStr">
         <is>
           <t>Hero Motors Ltd</t>
         </is>
       </c>
-      <c r="AR9" t="inlineStr">
+      <c r="AR8" t="inlineStr">
         <is>
           <t>https://groww.in/ipo/hero-motors-ipo</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-15)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR8"/>
+  <dimension ref="A1:AR13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -964,22 +964,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>Kanohar Electricals Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -1005,19 +1005,41 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Kanohar Electricals Ltd.</t>
+        </is>
+      </c>
+      <c r="AM5" t="n">
+        <v>61.38</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>122.61</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>81.56999999999999</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Glass Wall Systems (India) Limited</t>
+          <t>Rentomojo Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1053,29 +1075,51 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Rentomojo Ltd</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>30.79</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>46.72</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>53.78</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/rentomojo-ipo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Incred Holdings Limited</t>
+          <t>Steamhouse India Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1090,7 +1134,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1101,24 +1145,46 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Steamhouse India Ltd</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>28.61</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>12</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/steamhouse-india-ipo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>German Green Steel and Power Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1128,12 +1194,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Automobiles</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1154,17 +1220,313 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>Hero Motors Ltd</t>
-        </is>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/hero-motors-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-addendum-ii-to-drhp_104480.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Runwal Enterprises Limited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Prasol Chemicals Limited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/prasol-chemicals-limited-prospectus_104479.html</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Prasol Chemicals Ltd</t>
+        </is>
+      </c>
+      <c r="AM10" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/prasol-chemicals-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Glass Wall Systems (India) Limited</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Incred Holdings Limited</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Pranav Constructions Limited</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/pranav-constructions-limited-prospectus_104488.html</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Pranav Constructions Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ13" t="n">
+        <v>28.91</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>49.03</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>120.16</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>258.71</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>207.93</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>42</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/pranav-constructions-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-16)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR13"/>
+  <dimension ref="A1:AR14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -880,91 +880,77 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Torrent Gas Limited</t>
+          <t>Veegaland Developers Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>335000000</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>1396.78</v>
-      </c>
-      <c r="R4" t="n">
-        <v>-76.45999999999999</v>
-      </c>
-      <c r="S4" t="n">
-        <v>55.68</v>
-      </c>
-      <c r="T4" t="n">
-        <v>-80.18000000000001</v>
-      </c>
-      <c r="U4" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>8.199999999999999</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Veegaland Developers Ltd</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>17.76</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/veegaland-developers-ipo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Limited</t>
+          <t>Maharashtra Oil Extractions Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -974,18 +960,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>34.92</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -999,42 +1001,47 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Ltd.</t>
-        </is>
-      </c>
-      <c r="AM5" t="n">
-        <v>61.38</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>122.61</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>81.56999999999999</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>17.74</v>
+          <t>Maharashtra Corporation Ltd.</t>
+        </is>
+      </c>
+      <c r="AI5" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>16.62</v>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
+          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rentomojo Limited</t>
+          <t>Kanohar Electricals Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1075,41 +1082,44 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>Rentomojo Ltd</t>
+          <t>Kanohar Electricals</t>
         </is>
       </c>
       <c r="AM6" t="n">
-        <v>30.79</v>
+        <v>61.38</v>
       </c>
       <c r="AN6" t="n">
-        <v>46.72</v>
+        <v>122.61</v>
       </c>
       <c r="AO6" t="n">
-        <v>53.78</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="AP6" t="n">
-        <v>11.91</v>
+        <v>17.74</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>8.470000000000001</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/rentomojo-ipo</t>
+          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Steamhouse India Limited</t>
+          <t>Rentomojo Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1145,61 +1155,56 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>Steamhouse India Ltd</t>
+          <t>Rentomojo Ltd</t>
         </is>
       </c>
       <c r="AM7" t="n">
-        <v>13.63</v>
+        <v>30.79</v>
       </c>
       <c r="AN7" t="n">
-        <v>5.26</v>
+        <v>46.72</v>
       </c>
       <c r="AO7" t="n">
-        <v>28.61</v>
+        <v>53.78</v>
       </c>
       <c r="AP7" t="n">
-        <v>12</v>
+        <v>11.91</v>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/steamhouse-india-ipo</t>
+          <t>https://groww.in/ipo/rentomojo-ipo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>German Green Steel and Power Limited</t>
+          <t>Steamhouse India Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Metals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1209,7 +1214,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -1220,19 +1225,41 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-addendum-ii-to-drhp_104480.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>Steamhouse India Ltd</t>
+        </is>
+      </c>
+      <c r="AM8" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>28.61</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>12</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/steamhouse-india-ipo</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>German Green Steel and Power Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1247,7 +1274,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Metals</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1268,14 +1300,14 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-addendum-ii-to-drhp_104480.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Prasol Chemicals Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1285,22 +1317,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Chemicals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1310,7 +1337,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -1321,36 +1348,14 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/prasol-chemicals-limited-prospectus_104479.html</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>Prasol Chemicals Ltd</t>
-        </is>
-      </c>
-      <c r="AM10" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>5.63</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/prasol-chemicals-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Glass Wall Systems (India) Limited</t>
+          <t>Prasol Chemicals Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1370,7 +1375,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -1391,29 +1401,63 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/prasol-chemicals-limited-prospectus_104479.html</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>Prasol Chemicals Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ11" t="n">
+        <v>18.53</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>92.06999999999999</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>-9.76</v>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/prasol-chemicals-ltd</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Incred Holdings Limited</t>
+          <t>Glass Wall Systems (India) Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1428,7 +1472,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
@@ -1439,14 +1483,30 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>Glass Wall Systems (India) Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ12" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/glass-wall-systems-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pranav Constructions Limited</t>
+          <t>Incred Holdings Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1456,22 +1516,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Corrigendum</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Construction</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -1481,7 +1536,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
@@ -1492,39 +1547,95 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pranav Constructions Limited</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr">
+        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/pranav-constructions-limited-prospectus_104488.html</t>
         </is>
       </c>
-      <c r="AH13" t="inlineStr">
+      <c r="AH14" t="inlineStr">
         <is>
           <t>Pranav Constructions Ltd.</t>
         </is>
       </c>
-      <c r="AJ13" t="n">
+      <c r="AI14" t="n">
+        <v>1460</v>
+      </c>
+      <c r="AJ14" t="n">
         <v>28.91</v>
       </c>
-      <c r="AK13" t="n">
+      <c r="AK14" t="n">
         <v>1.08</v>
       </c>
-      <c r="AL13" t="n">
+      <c r="AL14" t="n">
         <v>49.03</v>
       </c>
-      <c r="AM13" t="n">
+      <c r="AM14" t="n">
         <v>120.16</v>
       </c>
-      <c r="AN13" t="n">
+      <c r="AN14" t="n">
         <v>258.71</v>
       </c>
-      <c r="AO13" t="n">
+      <c r="AO14" t="n">
         <v>207.93</v>
       </c>
-      <c r="AP13" t="n">
+      <c r="AP14" t="n">
         <v>42</v>
       </c>
-      <c r="AQ13" t="n">
+      <c r="AQ14" t="n">
         <v>33.06</v>
       </c>
-      <c r="AR13" t="inlineStr">
+      <c r="AR14" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/pranav-constructions-ltd</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-17)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR14"/>
+  <dimension ref="A1:AR16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -880,27 +880,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>Rayzon Solar Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -910,7 +915,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -921,73 +926,35 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>Veegaland Developers Ltd</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>13.37</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>17.76</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>17.98</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>8.880000000000001</v>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/veegaland-developers-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Maharashtra Oil Extractions Limited</t>
+          <t>Manika Plastech Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>34.92</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -1001,52 +968,47 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Maharashtra Corporation Ltd.</t>
-        </is>
-      </c>
-      <c r="AI5" t="n">
-        <v>19</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>-0.6</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>16.62</v>
+          <t>Manika Plastech Ltd</t>
+        </is>
+      </c>
+      <c r="AM5" t="n">
+        <v>27.91</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>62.99</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>22.31</v>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
+          <t>https://groww.in/ipo/manika-plastech-ipo</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Limited</t>
+          <t>LCC Projects Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1082,54 +1044,63 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>Kanohar Electricals</t>
-        </is>
+          <t>LCC Projects Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ6" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>100</v>
       </c>
       <c r="AM6" t="n">
-        <v>61.38</v>
+        <v>20.58</v>
       </c>
       <c r="AN6" t="n">
-        <v>122.61</v>
+        <v>7.37</v>
       </c>
       <c r="AO6" t="n">
-        <v>81.56999999999999</v>
+        <v>42.56</v>
       </c>
       <c r="AP6" t="n">
-        <v>17.74</v>
+        <v>18.48</v>
       </c>
       <c r="AQ6" t="n">
-        <v>8.470000000000001</v>
+        <v>29.45</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
+          <t>https://groww.in/stocks/lcc-projects-ltd</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rentomojo Limited</t>
+          <t>Sterlite Electric Limited – Second</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1144,7 +1115,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1155,41 +1126,19 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Rentomojo Ltd</t>
-        </is>
-      </c>
-      <c r="AM7" t="n">
-        <v>30.79</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>46.72</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>53.78</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>11.91</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/rentomojo-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Steamhouse India Limited</t>
+          <t>Veegaland Developers Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1225,46 +1174,46 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Steamhouse India Ltd</t>
+          <t>Veegaland Developers Ltd</t>
         </is>
       </c>
       <c r="AM8" t="n">
-        <v>13.63</v>
+        <v>13.37</v>
       </c>
       <c r="AN8" t="n">
-        <v>5.26</v>
+        <v>17.76</v>
       </c>
       <c r="AO8" t="n">
-        <v>28.61</v>
+        <v>17.98</v>
       </c>
       <c r="AP8" t="n">
-        <v>12</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/steamhouse-india-ipo</t>
+          <t>https://groww.in/ipo/veegaland-developers-ipo</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>German Green Steel and Power Limited</t>
+          <t>Maharashtra Oil Extractions Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1274,13 +1223,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Metals</t>
-        </is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>34.92</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1289,40 +1249,67 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-addendum-ii-to-drhp_104480.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Maharashtra Corporation Ltd.</t>
+        </is>
+      </c>
+      <c r="AI9" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>Kanohar Electricals Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1337,7 +1324,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -1348,19 +1335,56 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Kanohar Electricals Ltd.</t>
+        </is>
+      </c>
+      <c r="AI10" t="n">
+        <v>5949</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>74.65000000000001</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>61.38</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>122.61</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>81.56999999999999</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prasol Chemicals Limited</t>
+          <t>Rentomojo Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1375,12 +1399,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Chemicals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -1401,53 +1420,50 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/prasol-chemicals-limited-prospectus_104479.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Prasol Chemicals Ltd.</t>
+          <t>Rentomojo Ltd.</t>
         </is>
       </c>
       <c r="AJ11" t="n">
-        <v>18.53</v>
+        <v>35.26</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>92.06999999999999</v>
+        <v>0.79</v>
       </c>
       <c r="AM11" t="n">
-        <v>2.64</v>
+        <v>30.79</v>
       </c>
       <c r="AN11" t="n">
-        <v>5.63</v>
+        <v>46.72</v>
       </c>
       <c r="AO11" t="n">
-        <v>1.27</v>
+        <v>53.78</v>
       </c>
       <c r="AP11" t="n">
-        <v>1.52</v>
+        <v>11.91</v>
       </c>
       <c r="AQ11" t="n">
-        <v>-9.76</v>
+        <v>19.42</v>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/prasol-chemicals-ltd</t>
+          <t>https://groww.in/stocks/rentomojo-ltd</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Glass Wall Systems (India) Limited</t>
+          <t>Steamhouse India Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1483,40 +1499,58 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>Glass Wall Systems (India) Ltd.</t>
+          <t>Steamhouse India Ltd.</t>
         </is>
       </c>
       <c r="AJ12" t="n">
-        <v>32.24</v>
+        <v>22.36</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.03</v>
+        <v>1.94</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>98.69</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>28.61</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>12</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>16.67</v>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/glass-wall-systems-india-ltd</t>
+          <t>https://groww.in/stocks/steamhouse-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Incred Holdings Limited</t>
+          <t>German Green Steel and Power Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1526,7 +1560,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Metals</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -1547,39 +1586,34 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-addendum-ii-to-drhp_104480.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pranav Constructions Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Construction</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -1589,7 +1623,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
@@ -1600,44 +1634,167 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/pranav-constructions-limited-prospectus_104488.html</t>
-        </is>
-      </c>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>Pranav Constructions Ltd.</t>
-        </is>
-      </c>
-      <c r="AI14" t="n">
-        <v>1460</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>28.91</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>49.03</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>120.16</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>258.71</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>207.93</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>42</v>
-      </c>
-      <c r="AQ14" t="n">
-        <v>33.06</v>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/pranav-constructions-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Prasol Chemicals Limited</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/prasol-chemicals-limited-prospectus_104479.html</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>Prasol Chemicals Ltd.</t>
+        </is>
+      </c>
+      <c r="AI15" t="n">
+        <v>3977</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>18.53</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>75.25</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>-9.76</v>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/prasol-chemicals-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Glass Wall Systems (India) Limited</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>Glass Wall Systems (India) Ltd.</t>
+        </is>
+      </c>
+      <c r="AI16" t="n">
+        <v>1894</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>53.22</v>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/glass-wall-systems-india-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-18)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR16"/>
+  <dimension ref="A1:AR12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,17 +699,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nopaperforms Solutions Limited</t>
+          <t>Iberia Pharmaceuticals India Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -719,40 +719,45 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>115.65</v>
+        <v>96.54000000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>25.24</v>
+        <v>11.32</v>
       </c>
       <c r="S2" t="n">
-        <v>1</v>
+        <v>11.13</v>
       </c>
       <c r="T2" t="n">
-        <v>408.67</v>
+        <v>-21.54</v>
       </c>
       <c r="U2" t="n">
-        <v>0.83</v>
+        <v>11.53</v>
       </c>
       <c r="V2" t="n">
-        <v>6.58</v>
+        <v>17.56</v>
       </c>
       <c r="W2" t="n">
-        <v>33.12</v>
+        <v>24.31</v>
       </c>
       <c r="AA2" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -761,7 +766,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -772,115 +777,72 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/nopaperforms-solutions-limited-udrhp-1_104427.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iberia-pharmaceuticals-india-limited-drhp_104542.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/NOPAPERFORMS%20SOLUTIONS%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/IBERIA%20PHARMACEUTICALS%20INDIA%20LIMITED_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>M K C Agro Fresh Limited</t>
+          <t>Rayzon Solar Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>521.53</v>
-      </c>
-      <c r="R3" t="n">
-        <v>6.38</v>
-      </c>
-      <c r="S3" t="n">
-        <v>22.11</v>
-      </c>
-      <c r="T3" t="n">
-        <v>14.09</v>
-      </c>
-      <c r="U3" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="V3" t="n">
-        <v>7.49</v>
-      </c>
-      <c r="W3" t="n">
-        <v>15.92</v>
-      </c>
-      <c r="X3" t="n">
-        <v>9.880000000000001</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>30.8</v>
+          <t>Renewables</t>
+        </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/m-k-c-agro-fresh-limited-drhp_104430.html</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/M%20K%20C%20AGRO%20FRESH%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rayzon Solar Limited</t>
+          <t>Manika Plastech Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -890,22 +852,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Renewables</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -915,7 +872,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -926,14 +883,36 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Manika Plastech Ltd</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>27.91</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>62.99</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>22.31</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/manika-plastech-ipo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Manika Plastech Limited</t>
+          <t>LCC Projects Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -974,51 +953,66 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Manika Plastech Ltd</t>
-        </is>
+          <t>LCC Projects Ltd.</t>
+        </is>
+      </c>
+      <c r="AI5" t="n">
+        <v>5004</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>89.90000000000001</v>
       </c>
       <c r="AM5" t="n">
-        <v>27.91</v>
+        <v>20.58</v>
       </c>
       <c r="AN5" t="n">
-        <v>10.94</v>
+        <v>7.37</v>
       </c>
       <c r="AO5" t="n">
-        <v>62.99</v>
+        <v>42.56</v>
       </c>
       <c r="AP5" t="n">
-        <v>22.31</v>
+        <v>18.48</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>29.45</v>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/manika-plastech-ipo</t>
+          <t>https://groww.in/stocks/lcc-projects-ltd</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LCC Projects Limited</t>
+          <t>Sterlite Electric Limited – Second</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1033,7 +1027,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -1044,48 +1038,14 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>LCC Projects Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ6" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>100</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>20.58</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>7.37</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>42.56</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>18.48</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>29.45</v>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/lcc-projects-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sterlite Electric Limited – Second</t>
+          <t>Veegaland Developers Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1095,12 +1055,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1115,7 +1075,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1126,35 +1086,82 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Veegaland Developers Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ7" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>17.76</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>10</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>Maharashtra Oil Extractions Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>34.92</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
@@ -1168,42 +1175,47 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Veegaland Developers Ltd</t>
-        </is>
-      </c>
-      <c r="AM8" t="n">
-        <v>13.37</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>17.76</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>17.98</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>8.880000000000001</v>
+          <t>Maharashtra Corporation Ltd.</t>
+        </is>
+      </c>
+      <c r="AI8" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>16.62</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/veegaland-developers-ipo</t>
+          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Maharashtra Oil Extractions Limited</t>
+          <t>Kanohar Electricals Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1213,34 +1225,18 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>34.92</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1254,47 +1250,57 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>DRHP_PDF</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
-        </is>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Maharashtra Corporation Ltd.</t>
+          <t>Kanohar Electricals Ltd.</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>19</v>
+        <v>6483</v>
       </c>
       <c r="AJ9" t="n">
-        <v>-0.6</v>
+        <v>34.8</v>
       </c>
       <c r="AK9" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AL9" t="n">
-        <v>16.62</v>
+        <v>74.65000000000001</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>61.38</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>122.61</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>81.56999999999999</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>8.470000000000001</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
+          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Limited</t>
+          <t>Rentomojo Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1335,56 +1341,56 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Ltd.</t>
+          <t>Rentomojo Ltd.</t>
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>5949</v>
+        <v>5549</v>
       </c>
       <c r="AJ10" t="n">
-        <v>34.8</v>
+        <v>35.26</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.1</v>
+        <v>0.79</v>
       </c>
       <c r="AL10" t="n">
-        <v>74.65000000000001</v>
+        <v>19.74</v>
       </c>
       <c r="AM10" t="n">
-        <v>61.38</v>
+        <v>30.79</v>
       </c>
       <c r="AN10" t="n">
-        <v>122.61</v>
+        <v>46.72</v>
       </c>
       <c r="AO10" t="n">
-        <v>81.56999999999999</v>
+        <v>53.78</v>
       </c>
       <c r="AP10" t="n">
-        <v>17.74</v>
+        <v>11.91</v>
       </c>
       <c r="AQ10" t="n">
-        <v>8.470000000000001</v>
+        <v>19.42</v>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
+          <t>https://groww.in/stocks/rentomojo-ltd</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rentomojo Limited</t>
+          <t>Steamhouse India Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1420,65 +1426,76 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Rentomojo Ltd.</t>
-        </is>
+          <t>Steamhouse India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI11" t="n">
+        <v>2825</v>
       </c>
       <c r="AJ11" t="n">
-        <v>35.26</v>
+        <v>22.36</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.79</v>
+        <v>1.94</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>77.95999999999999</v>
       </c>
       <c r="AM11" t="n">
-        <v>30.79</v>
+        <v>13.63</v>
       </c>
       <c r="AN11" t="n">
-        <v>46.72</v>
+        <v>5.26</v>
       </c>
       <c r="AO11" t="n">
-        <v>53.78</v>
+        <v>28.61</v>
       </c>
       <c r="AP11" t="n">
-        <v>11.91</v>
+        <v>12</v>
       </c>
       <c r="AQ11" t="n">
-        <v>19.42</v>
+        <v>16.67</v>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/rentomojo-ltd</t>
+          <t>https://groww.in/stocks/steamhouse-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Steamhouse India Limited</t>
+          <t>German Green Steel and Power Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Metals</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -1488,7 +1505,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
@@ -1499,302 +1516,7 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
-        </is>
-      </c>
-      <c r="AH12" t="inlineStr">
-        <is>
-          <t>Steamhouse India Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ12" t="n">
-        <v>22.36</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>98.69</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>13.63</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>28.61</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>12</v>
-      </c>
-      <c r="AQ12" t="n">
-        <v>16.67</v>
-      </c>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/steamhouse-india-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>German Green Steel and Power Limited</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Metals</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr">
-        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-addendum-ii-to-drhp_104480.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Runwal Enterprises Limited</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Prasol Chemicals Limited</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Chemicals</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/prasol-chemicals-limited-prospectus_104479.html</t>
-        </is>
-      </c>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>Prasol Chemicals Ltd.</t>
-        </is>
-      </c>
-      <c r="AI15" t="n">
-        <v>3977</v>
-      </c>
-      <c r="AJ15" t="n">
-        <v>18.53</v>
-      </c>
-      <c r="AK15" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>75.25</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>5.63</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="AQ15" t="n">
-        <v>-9.76</v>
-      </c>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/prasol-chemicals-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Glass Wall Systems (India) Limited</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
-        </is>
-      </c>
-      <c r="AH16" t="inlineStr">
-        <is>
-          <t>Glass Wall Systems (India) Ltd.</t>
-        </is>
-      </c>
-      <c r="AI16" t="n">
-        <v>1894</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>32.24</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>53.22</v>
-      </c>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/glass-wall-systems-india-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-19)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Iberia Pharmaceuticals India Limited</t>
+          <t>Madhur Iron &amp; Steel India Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -719,45 +719,51 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="N2" t="n">
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>96.54000000000001</v>
+        <v>444.02</v>
       </c>
       <c r="R2" t="n">
-        <v>11.32</v>
+        <v>30.76</v>
       </c>
       <c r="S2" t="n">
-        <v>11.13</v>
+        <v>23.88</v>
       </c>
       <c r="T2" t="n">
-        <v>-21.54</v>
+        <v>31.75</v>
       </c>
       <c r="U2" t="n">
-        <v>11.53</v>
+        <v>5.38</v>
       </c>
       <c r="V2" t="n">
-        <v>17.56</v>
+        <v>11.74</v>
       </c>
       <c r="W2" t="n">
-        <v>24.31</v>
+        <v>22.54</v>
+      </c>
+      <c r="X2" t="n">
+        <v>16.22</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>1.66</v>
       </c>
       <c r="AA2" t="n">
-        <v>34</v>
+        <v>61.9</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -777,19 +783,19 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iberia-pharmaceuticals-india-limited-drhp_104542.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/madhur-iron-and-steel-india-limited-drhp_104575.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/IBERIA%20PHARMACEUTICALS%20INDIA%20LIMITED_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Madhur%20Iron%20And%20Steel%20India%20Limited%20-%20Draft%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rayzon Solar Limited</t>
+          <t>Iberia Pharmaceuticals India Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -799,7 +805,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -809,40 +815,77 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Renewables</t>
-        </is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>96.54000000000001</v>
+      </c>
+      <c r="R3" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="S3" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-21.54</v>
+      </c>
+      <c r="U3" t="n">
+        <v>11.53</v>
+      </c>
+      <c r="V3" t="n">
+        <v>17.56</v>
+      </c>
+      <c r="W3" t="n">
+        <v>24.31</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>34</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iberia-pharmaceuticals-india-limited-drhp_104542.html</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/IBERIA%20PHARMACEUTICALS%20INDIA%20LIMITED_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Manika Plastech Limited</t>
+          <t>Rayzon Solar Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -852,17 +895,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -872,7 +920,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -883,36 +931,14 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>Manika Plastech Ltd</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>27.91</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>10.94</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>62.99</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>22.31</v>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/manika-plastech-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LCC Projects Limited</t>
+          <t>Manika Plastech Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -953,66 +979,51 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>LCC Projects Ltd.</t>
-        </is>
-      </c>
-      <c r="AI5" t="n">
-        <v>5004</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>89.90000000000001</v>
+          <t>Manika Plastech Ltd</t>
+        </is>
       </c>
       <c r="AM5" t="n">
-        <v>20.58</v>
+        <v>27.91</v>
       </c>
       <c r="AN5" t="n">
-        <v>7.37</v>
+        <v>10.94</v>
       </c>
       <c r="AO5" t="n">
-        <v>42.56</v>
+        <v>62.99</v>
       </c>
       <c r="AP5" t="n">
-        <v>18.48</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>29.45</v>
+        <v>22.31</v>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/lcc-projects-ltd</t>
+          <t>https://groww.in/ipo/manika-plastech-ipo</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sterlite Electric Limited – Second</t>
+          <t>LCC Projects Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1027,7 +1038,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -1038,14 +1049,51 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>LCC Projects Ltd.</t>
+        </is>
+      </c>
+      <c r="AI6" t="n">
+        <v>5004</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>42.56</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>18.48</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>29.45</v>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/lcc-projects-ltd</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>Sterlite Electric Limited – Second</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1055,12 +1103,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1075,7 +1123,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1086,82 +1134,35 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Veegaland Developers Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ7" t="n">
-        <v>9.970000000000001</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>13.37</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>17.76</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>17.98</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>8.880000000000001</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>10</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Maharashtra Oil Extractions Limited</t>
+          <t>Veegaland Developers Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>34.92</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
@@ -1175,47 +1176,51 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>DRHP_PDF</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
-        </is>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Maharashtra Corporation Ltd.</t>
-        </is>
-      </c>
-      <c r="AI8" t="n">
-        <v>20</v>
+          <t>Veegaland Developers Ltd.</t>
+        </is>
       </c>
       <c r="AJ8" t="n">
-        <v>-0.6</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="AK8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>16.62</v>
+        <v>0.32</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>17.76</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>10</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
+          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Limited</t>
+          <t>Maharashtra Oil Extractions Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1225,18 +1230,34 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>34.92</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1250,57 +1271,47 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Ltd.</t>
+          <t>Maharashtra Corporation Ltd.</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>6483</v>
+        <v>20</v>
       </c>
       <c r="AJ9" t="n">
-        <v>34.8</v>
+        <v>-0.6</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AL9" t="n">
-        <v>74.65000000000001</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>61.38</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>122.61</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>81.56999999999999</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>17.74</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>8.470000000000001</v>
+        <v>16.62</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
+          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rentomojo Limited</t>
+          <t>Kanohar Electricals Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1341,56 +1352,56 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>Rentomojo Ltd.</t>
+          <t>Kanohar Electricals Ltd.</t>
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>5549</v>
+        <v>6483</v>
       </c>
       <c r="AJ10" t="n">
-        <v>35.26</v>
+        <v>34.8</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.79</v>
+        <v>0.1</v>
       </c>
       <c r="AL10" t="n">
-        <v>19.74</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="AM10" t="n">
-        <v>30.79</v>
+        <v>61.38</v>
       </c>
       <c r="AN10" t="n">
-        <v>46.72</v>
+        <v>122.61</v>
       </c>
       <c r="AO10" t="n">
-        <v>53.78</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="AP10" t="n">
-        <v>11.91</v>
+        <v>17.74</v>
       </c>
       <c r="AQ10" t="n">
-        <v>19.42</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/rentomojo-ltd</t>
+          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Steamhouse India Limited</t>
+          <t>Rentomojo Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1426,76 +1437,71 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Steamhouse India Ltd.</t>
+          <t>Rentomojo Ltd.</t>
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>2825</v>
+        <v>5549</v>
       </c>
       <c r="AJ11" t="n">
-        <v>22.36</v>
+        <v>35.26</v>
       </c>
       <c r="AK11" t="n">
-        <v>1.94</v>
+        <v>0.79</v>
       </c>
       <c r="AL11" t="n">
-        <v>77.95999999999999</v>
+        <v>19.74</v>
       </c>
       <c r="AM11" t="n">
-        <v>13.63</v>
+        <v>30.79</v>
       </c>
       <c r="AN11" t="n">
-        <v>5.26</v>
+        <v>46.72</v>
       </c>
       <c r="AO11" t="n">
-        <v>28.61</v>
+        <v>53.78</v>
       </c>
       <c r="AP11" t="n">
-        <v>12</v>
+        <v>11.91</v>
       </c>
       <c r="AQ11" t="n">
-        <v>16.67</v>
+        <v>19.42</v>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/steamhouse-india-ltd</t>
+          <t>https://groww.in/stocks/rentomojo-ltd</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>German Green Steel and Power Limited</t>
+          <t>Steamhouse India Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Metals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -1505,7 +1511,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
@@ -1516,7 +1522,44 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-addendum-ii-to-drhp_104480.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>Steamhouse India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI12" t="n">
+        <v>2825</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>22.36</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>77.95999999999999</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>28.61</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>12</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/steamhouse-india-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-21)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR12"/>
+  <dimension ref="A1:AR14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -885,17 +885,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rayzon Solar Limited</t>
+          <t>Anchor Offshore Services Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -905,45 +905,91 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Renewables</t>
-        </is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>6400000</v>
+      </c>
+      <c r="L4" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M4" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>105.83</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="S4" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="T4" t="n">
+        <v>-37.65</v>
+      </c>
+      <c r="U4" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="V4" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="W4" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anchor-offshore-services-limited-drhp_104580.html</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anchor%20Offshore%20Services%20Limited-DA_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Manika Plastech Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -958,7 +1004,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -968,7 +1019,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -979,41 +1030,41 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Manika Plastech Ltd</t>
+          <t>Hero Motors Ltd</t>
         </is>
       </c>
       <c r="AM5" t="n">
-        <v>27.91</v>
+        <v>6.64</v>
       </c>
       <c r="AN5" t="n">
-        <v>10.94</v>
+        <v>1.49</v>
       </c>
       <c r="AO5" t="n">
-        <v>62.99</v>
+        <v>9.85</v>
       </c>
       <c r="AP5" t="n">
-        <v>22.31</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/manika-plastech-ipo</t>
+          <t>https://groww.in/ipo/hero-motors-ipo</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LCC Projects Limited</t>
+          <t>SS Retail Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1028,7 +1079,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Retail</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1049,56 +1105,41 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>LCC Projects Ltd.</t>
-        </is>
-      </c>
-      <c r="AI6" t="n">
-        <v>5004</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>89.90000000000001</v>
+          <t>SS Retail Ltd</t>
+        </is>
       </c>
       <c r="AM6" t="n">
-        <v>20.58</v>
+        <v>103.01</v>
       </c>
       <c r="AN6" t="n">
-        <v>7.37</v>
+        <v>203.61</v>
       </c>
       <c r="AO6" t="n">
-        <v>42.56</v>
+        <v>143.23</v>
       </c>
       <c r="AP6" t="n">
-        <v>18.48</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>29.45</v>
+        <v>35.81</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/lcc-projects-ltd</t>
+          <t>https://groww.in/ipo/ss-retail-ipo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sterlite Electric Limited – Second</t>
+          <t>Rayzon Solar Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1113,7 +1154,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1134,19 +1180,19 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>Manika Plastech Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1182,82 +1228,69 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Veegaland Developers Ltd.</t>
+          <t>Manika Plastech Ltd.</t>
         </is>
       </c>
       <c r="AJ8" t="n">
-        <v>9.970000000000001</v>
+        <v>15.18</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.32</v>
+        <v>0.66</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>74.95</v>
       </c>
       <c r="AM8" t="n">
-        <v>13.37</v>
+        <v>27.91</v>
       </c>
       <c r="AN8" t="n">
-        <v>17.76</v>
+        <v>10.94</v>
       </c>
       <c r="AO8" t="n">
-        <v>17.98</v>
+        <v>62.99</v>
       </c>
       <c r="AP8" t="n">
-        <v>8.880000000000001</v>
+        <v>22.31</v>
       </c>
       <c r="AQ8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
+          <t>https://groww.in/stocks/manika-plastech-ltd</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Maharashtra Oil Extractions Limited</t>
+          <t>LCC Projects Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>34.92</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1271,62 +1304,72 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>DRHP_PDF</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
-        </is>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Maharashtra Corporation Ltd.</t>
+          <t>LCC Projects Ltd.</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>20</v>
+        <v>4507</v>
       </c>
       <c r="AJ9" t="n">
-        <v>-0.6</v>
+        <v>31.9</v>
       </c>
       <c r="AK9" t="n">
-        <v>0</v>
+        <v>0.97</v>
       </c>
       <c r="AL9" t="n">
-        <v>16.62</v>
+        <v>89.90000000000001</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>42.56</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>18.48</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>29.45</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
+          <t>https://groww.in/stocks/lcc-projects-ltd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Limited</t>
+          <t>Sterlite Electric Limited – Second</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1341,7 +1384,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -1352,56 +1395,19 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>Kanohar Electricals Ltd.</t>
-        </is>
-      </c>
-      <c r="AI10" t="n">
-        <v>6483</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>74.65000000000001</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>61.38</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>122.61</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>81.56999999999999</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>17.74</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>8.470000000000001</v>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rentomojo Limited</t>
+          <t>Veegaland Developers Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1437,72 +1443,88 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Rentomojo Ltd.</t>
+          <t>Veegaland Developers Ltd.</t>
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>5549</v>
+        <v>707</v>
       </c>
       <c r="AJ11" t="n">
-        <v>35.26</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.79</v>
+        <v>0.32</v>
       </c>
       <c r="AL11" t="n">
-        <v>19.74</v>
+        <v>63.69</v>
       </c>
       <c r="AM11" t="n">
-        <v>30.79</v>
+        <v>13.37</v>
       </c>
       <c r="AN11" t="n">
-        <v>46.72</v>
+        <v>17.76</v>
       </c>
       <c r="AO11" t="n">
-        <v>53.78</v>
+        <v>17.98</v>
       </c>
       <c r="AP11" t="n">
-        <v>11.91</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="AQ11" t="n">
-        <v>19.42</v>
+        <v>10</v>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/rentomojo-ltd</t>
+          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Steamhouse India Limited</t>
+          <t>Maharashtra Oil Extractions Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>34.92</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -1516,50 +1538,210 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/steamhouse-india-limited-prospectus_104485.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>Steamhouse India Ltd.</t>
+          <t>Maharashtra Corporation Ltd.</t>
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>2825</v>
+        <v>20</v>
       </c>
       <c r="AJ12" t="n">
-        <v>22.36</v>
+        <v>-0.6</v>
       </c>
       <c r="AK12" t="n">
-        <v>1.94</v>
+        <v>0</v>
       </c>
       <c r="AL12" t="n">
-        <v>77.95999999999999</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>13.63</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>28.61</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>12</v>
-      </c>
-      <c r="AQ12" t="n">
-        <v>16.67</v>
+        <v>16.62</v>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/steamhouse-india-ltd</t>
+          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Kanohar Electricals Limited</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Kanohar Electricals Ltd.</t>
+        </is>
+      </c>
+      <c r="AI13" t="n">
+        <v>6240</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>74.65000000000001</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>61.38</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>122.61</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>81.56999999999999</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rentomojo Limited</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Rentomojo Ltd.</t>
+        </is>
+      </c>
+      <c r="AI14" t="n">
+        <v>5342</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>35.26</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>19.74</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>30.79</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>46.72</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>53.78</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>19.42</v>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/rentomojo-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-22)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR14"/>
+  <dimension ref="A1:AR15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -795,12 +795,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Iberia Pharmaceuticals India Limited</t>
+          <t>Hi-Tech Flow Solutions Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -815,45 +815,40 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Pharmaceuticals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>96.54000000000001</v>
+        <v>417.17</v>
       </c>
       <c r="R3" t="n">
-        <v>11.32</v>
+        <v>39.86</v>
       </c>
       <c r="S3" t="n">
-        <v>11.13</v>
+        <v>36.42</v>
       </c>
       <c r="T3" t="n">
-        <v>-21.54</v>
+        <v>50.16</v>
       </c>
       <c r="U3" t="n">
-        <v>11.53</v>
+        <v>8.73</v>
       </c>
       <c r="V3" t="n">
-        <v>17.56</v>
+        <v>12.7</v>
       </c>
       <c r="W3" t="n">
-        <v>24.31</v>
+        <v>32.24</v>
       </c>
       <c r="AA3" t="n">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -873,24 +868,24 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iberia-pharmaceuticals-india-limited-drhp_104542.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hi-tech-flow-solutions-limited-drhp_104635.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/IBERIA%20PHARMACEUTICALS%20INDIA%20LIMITED_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/HitechFlowSolutionsDAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anchor Offshore Services Limited</t>
+          <t>Iberia Pharmaceuticals India Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -905,58 +900,49 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Pharmaceuticals</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>6400000</v>
-      </c>
-      <c r="L4" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M4" t="n">
-        <v>7000000</v>
+          <t>Fresh</t>
+        </is>
       </c>
       <c r="N4" t="n">
         <v>10</v>
       </c>
       <c r="Q4" t="n">
-        <v>105.83</v>
+        <v>96.54000000000001</v>
       </c>
       <c r="R4" t="n">
-        <v>-24.4</v>
+        <v>11.32</v>
       </c>
       <c r="S4" t="n">
-        <v>8.039999999999999</v>
+        <v>11.13</v>
       </c>
       <c r="T4" t="n">
-        <v>-37.65</v>
+        <v>-21.54</v>
       </c>
       <c r="U4" t="n">
-        <v>3.97</v>
+        <v>11.53</v>
       </c>
       <c r="V4" t="n">
-        <v>11.37</v>
+        <v>17.56</v>
       </c>
       <c r="W4" t="n">
-        <v>7.47</v>
+        <v>24.31</v>
       </c>
       <c r="AA4" t="n">
-        <v>8.800000000000001</v>
+        <v>34</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -972,99 +958,123 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anchor-offshore-services-limited-drhp_104580.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iberia-pharmaceuticals-india-limited-drhp_104542.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anchor%20Offshore%20Services%20Limited-DA_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/IBERIA%20PHARMACEUTICALS%20INDIA%20LIMITED_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Anchor Offshore Services Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Automobiles</t>
-        </is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>6400000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M5" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>105.83</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="S5" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-37.65</v>
+      </c>
+      <c r="U5" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="V5" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="W5" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>Hero Motors Ltd</t>
-        </is>
-      </c>
-      <c r="AM5" t="n">
-        <v>6.64</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/hero-motors-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anchor-offshore-services-limited-drhp_104580.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anchor%20Offshore%20Services%20Limited-DA_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SS Retail Limited</t>
+          <t>National Stock Exchange of India Ltd</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1079,12 +1089,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Market Infrastructure</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1105,61 +1115,39 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>SS Retail Ltd</t>
-        </is>
-      </c>
-      <c r="AM6" t="n">
-        <v>103.01</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>203.61</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>143.23</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>35.81</v>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/ss-retail-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rayzon Solar Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1169,7 +1157,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1180,19 +1168,41 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Hero Motors Ltd</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/hero-motors-ipo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Manika Plastech Limited</t>
+          <t>Jindal Supreme (India) Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1228,53 +1238,19 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>Manika Plastech Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ8" t="n">
-        <v>15.18</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>74.95</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>27.91</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>10.94</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>62.99</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>22.31</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/manika-plastech-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jindal-supreme-india-limited-prospectus_104621.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LCC Projects Limited</t>
+          <t>Manipal Payment &amp; Identity Solutions Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1310,71 +1286,76 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manipal-payment-and-identity-solutions-limited-prospectus_104619.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>LCC Projects Ltd.</t>
+          <t>Manipal Payment And Identity Solutions Ltd.</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>4507</v>
+        <v>7820</v>
       </c>
       <c r="AJ9" t="n">
-        <v>31.9</v>
+        <v>32.01</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.97</v>
+        <v>0.19</v>
       </c>
       <c r="AL9" t="n">
-        <v>89.90000000000001</v>
+        <v>53.92</v>
       </c>
       <c r="AM9" t="n">
-        <v>20.58</v>
+        <v>1.17</v>
       </c>
       <c r="AN9" t="n">
-        <v>7.37</v>
+        <v>1.12</v>
       </c>
       <c r="AO9" t="n">
-        <v>42.56</v>
+        <v>0.8</v>
       </c>
       <c r="AP9" t="n">
-        <v>18.48</v>
+        <v>1.86</v>
       </c>
       <c r="AQ9" t="n">
-        <v>29.45</v>
+        <v>-2.65</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/lcc-projects-ltd</t>
+          <t>https://groww.in/stocks/manipal-payment-and-identity-solutions-ltd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sterlite Electric Limited – Second</t>
+          <t>SS Retail Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Retail</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1384,7 +1365,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -1395,34 +1376,61 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>SS Retail Ltd</t>
+        </is>
+      </c>
+      <c r="AM10" t="n">
+        <v>103.01</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>203.61</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>143.23</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>35.81</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/ss-retail-ipo</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>Rayzon Solar Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -1432,7 +1440,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -1443,88 +1451,35 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>Veegaland Developers Ltd.</t>
-        </is>
-      </c>
-      <c r="AI11" t="n">
-        <v>707</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>9.970000000000001</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>63.69</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>13.37</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>17.76</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>17.98</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>8.880000000000001</v>
-      </c>
-      <c r="AQ11" t="n">
-        <v>10</v>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Maharashtra Oil Extractions Limited</t>
+          <t>Manika Plastech Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>34.92</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -1538,52 +1493,62 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>DRHP_PDF</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/maharashtra-oil-extractions-limited-drhp_104503.html</t>
-        </is>
-      </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Maharashtra%20Oil%20Extractions%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>Maharashtra Corporation Ltd.</t>
+          <t>Manika Plastech Ltd.</t>
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>20</v>
+        <v>501</v>
       </c>
       <c r="AJ12" t="n">
-        <v>-0.6</v>
+        <v>15.18</v>
       </c>
       <c r="AK12" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>74.95</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>27.91</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>62.99</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>22.31</v>
+      </c>
+      <c r="AQ12" t="n">
         <v>0</v>
       </c>
-      <c r="AL12" t="n">
-        <v>16.62</v>
-      </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/maharashtra-corporation-ltd</t>
+          <t>https://groww.in/stocks/manika-plastech-ltd</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Limited</t>
+          <t>LCC Projects Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1619,66 +1584,66 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kanohar-electricals-limited-prospectus_104483.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>Kanohar Electricals Ltd.</t>
+          <t>LCC Projects Ltd.</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>6240</v>
+        <v>4121</v>
       </c>
       <c r="AJ13" t="n">
-        <v>34.8</v>
+        <v>31.9</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.1</v>
+        <v>0.97</v>
       </c>
       <c r="AL13" t="n">
-        <v>74.65000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="AM13" t="n">
-        <v>61.38</v>
+        <v>20.58</v>
       </c>
       <c r="AN13" t="n">
-        <v>122.61</v>
+        <v>7.37</v>
       </c>
       <c r="AO13" t="n">
-        <v>81.56999999999999</v>
+        <v>42.56</v>
       </c>
       <c r="AP13" t="n">
-        <v>17.74</v>
+        <v>18.48</v>
       </c>
       <c r="AQ13" t="n">
-        <v>8.470000000000001</v>
+        <v>29.45</v>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/kanohar-electricals-ltd</t>
+          <t>https://groww.in/stocks/lcc-projects-ltd</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Rentomojo Limited</t>
+          <t>Sterlite Electric Limited – Second</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1693,7 +1658,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
@@ -1704,44 +1669,92 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rentomojo-limited-prospectus_104482.html</t>
-        </is>
-      </c>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>Rentomojo Ltd.</t>
-        </is>
-      </c>
-      <c r="AI14" t="n">
-        <v>5342</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>35.26</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>19.74</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>30.79</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>46.72</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>53.78</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>11.91</v>
-      </c>
-      <c r="AQ14" t="n">
-        <v>19.42</v>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/rentomojo-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Veegaland Developers Limited</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>Veegaland Developers Ltd.</t>
+        </is>
+      </c>
+      <c r="AI15" t="n">
+        <v>688</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>63.69</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>17.76</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>10</v>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-23)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -1069,7 +1069,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>National Stock Exchange of India Ltd</t>
+          <t>Vardaan Biotech Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1079,22 +1079,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Market Infrastructure</t>
+          <t>Biotechnology</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1115,19 +1115,19 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardaan-biotech-limited_104652.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Amtech Esters Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1142,12 +1142,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1157,7 +1152,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1168,41 +1163,56 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/amtech-esters-limited-prospectus_104640.html</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>Hero Motors Ltd</t>
-        </is>
+          <t>Amtech Esters Ltd.</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>96</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>45.52</v>
       </c>
       <c r="AM7" t="n">
-        <v>6.64</v>
+        <v>13.67</v>
       </c>
       <c r="AN7" t="n">
-        <v>1.49</v>
+        <v>9.77</v>
       </c>
       <c r="AO7" t="n">
-        <v>9.85</v>
+        <v>12.82</v>
       </c>
       <c r="AP7" t="n">
-        <v>8.199999999999999</v>
+        <v>16.4</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>33.33</v>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/hero-motors-ipo</t>
+          <t>https://groww.in/stocks/amtech-esters-ltd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jindal Supreme (India) Limited</t>
+          <t>National Stock Exchange of India Ltd</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1217,7 +1227,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Market Infrastructure</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1238,14 +1253,14 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jindal-supreme-india-limited-prospectus_104621.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Manipal Payment &amp; Identity Solutions Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1265,7 +1280,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1275,7 +1295,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
@@ -1286,51 +1306,45 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manipal-payment-and-identity-solutions-limited-prospectus_104619.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Manipal Payment And Identity Solutions Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>7820</v>
+          <t>Hero Motors Ltd.</t>
+        </is>
       </c>
       <c r="AJ9" t="n">
-        <v>32.01</v>
+        <v>9.18</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>53.92</v>
+        <v>0.99</v>
       </c>
       <c r="AM9" t="n">
-        <v>1.17</v>
+        <v>6.64</v>
       </c>
       <c r="AN9" t="n">
-        <v>1.12</v>
+        <v>1.49</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.8</v>
+        <v>9.85</v>
       </c>
       <c r="AP9" t="n">
-        <v>1.86</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AQ9" t="n">
-        <v>-2.65</v>
+        <v>-2.38</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/manipal-payment-and-identity-solutions-ltd</t>
+          <t>https://groww.in/stocks/hero-motors-ltd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SS Retail Limited</t>
+          <t>Jindal Supreme (India) Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1350,12 +1364,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Retail</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1376,61 +1385,50 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jindal-supreme-india-limited-prospectus_104621.html</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>SS Retail Ltd</t>
-        </is>
-      </c>
-      <c r="AM10" t="n">
-        <v>103.01</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>203.61</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>143.23</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>35.81</v>
+          <t>Jindal Supreme (India) Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.91</v>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/ss-retail-ipo</t>
+          <t>https://groww.in/stocks/jindal-supreme-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rayzon Solar Limited</t>
+          <t>Manipal Payment &amp; Identity Solutions Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Renewables</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -1440,7 +1438,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -1451,19 +1449,56 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manipal-payment-and-identity-solutions-limited-prospectus_104619.html</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>Manipal Payment And Identity Solutions Ltd.</t>
+        </is>
+      </c>
+      <c r="AI11" t="n">
+        <v>7834</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>-2.65</v>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/manipal-payment-and-identity-solutions-ltd</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Manika Plastech Limited</t>
+          <t>SS Retail Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1478,7 +1513,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Retail</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -1499,51 +1539,48 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>Manika Plastech Ltd.</t>
-        </is>
-      </c>
-      <c r="AI12" t="n">
-        <v>501</v>
+          <t>SS Retail Ltd.</t>
+        </is>
       </c>
       <c r="AJ12" t="n">
-        <v>15.18</v>
+        <v>0</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.66</v>
+        <v>0.85</v>
       </c>
       <c r="AL12" t="n">
-        <v>74.95</v>
+        <v>75.73999999999999</v>
       </c>
       <c r="AM12" t="n">
-        <v>27.91</v>
+        <v>103.01</v>
       </c>
       <c r="AN12" t="n">
-        <v>10.94</v>
+        <v>203.61</v>
       </c>
       <c r="AO12" t="n">
-        <v>62.99</v>
+        <v>143.23</v>
       </c>
       <c r="AP12" t="n">
-        <v>22.31</v>
+        <v>35.81</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0</v>
+        <v>47.17</v>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/manika-plastech-ltd</t>
+          <t>https://groww.in/stocks/ss-retail-ltd</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LCC Projects Limited</t>
+          <t>Rayzon Solar Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1553,17 +1590,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -1573,7 +1615,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
@@ -1584,66 +1626,29 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
-        </is>
-      </c>
-      <c r="AH13" t="inlineStr">
-        <is>
-          <t>LCC Projects Ltd.</t>
-        </is>
-      </c>
-      <c r="AI13" t="n">
-        <v>4121</v>
-      </c>
-      <c r="AJ13" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>89.90000000000001</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>20.58</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>7.37</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>42.56</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>18.48</v>
-      </c>
-      <c r="AQ13" t="n">
-        <v>29.45</v>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/lcc-projects-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sterlite Electric Limited – Second</t>
+          <t>Manika Plastech Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1658,7 +1663,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
@@ -1669,19 +1674,56 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sterlite-electric-limited-second-addendum-to-drhp_104506.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Manika Plastech Ltd.</t>
+        </is>
+      </c>
+      <c r="AI14" t="n">
+        <v>484</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>74.95</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>27.91</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>62.99</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>22.31</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/manika-plastech-ltd</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Veegaland Developers Limited</t>
+          <t>LCC Projects Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1717,44 +1759,44 @@
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/veegaland-developers-limited-prospectus_104504.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
         </is>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Veegaland Developers Ltd.</t>
+          <t>LCC Projects Ltd.</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>688</v>
+        <v>4276</v>
       </c>
       <c r="AJ15" t="n">
-        <v>9.970000000000001</v>
+        <v>31.9</v>
       </c>
       <c r="AK15" t="n">
-        <v>0.32</v>
+        <v>0.97</v>
       </c>
       <c r="AL15" t="n">
-        <v>63.69</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="AM15" t="n">
-        <v>13.37</v>
+        <v>20.58</v>
       </c>
       <c r="AN15" t="n">
-        <v>17.76</v>
+        <v>7.37</v>
       </c>
       <c r="AO15" t="n">
-        <v>17.98</v>
+        <v>42.56</v>
       </c>
       <c r="AP15" t="n">
-        <v>8.880000000000001</v>
+        <v>18.48</v>
       </c>
       <c r="AQ15" t="n">
-        <v>10</v>
+        <v>29.45</v>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/veegaland-developers-ltd</t>
+          <t>https://groww.in/stocks/lcc-projects-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-24)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR15"/>
+  <dimension ref="A1:AR12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -880,12 +880,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Iberia Pharmaceuticals India Limited</t>
+          <t>Anchor Offshore Services Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -900,49 +900,58 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Fresh</t>
-        </is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>6400000</v>
+      </c>
+      <c r="L4" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M4" t="n">
+        <v>7000000</v>
       </c>
       <c r="N4" t="n">
         <v>10</v>
       </c>
       <c r="Q4" t="n">
-        <v>96.54000000000001</v>
+        <v>105.83</v>
       </c>
       <c r="R4" t="n">
-        <v>11.32</v>
+        <v>-24.4</v>
       </c>
       <c r="S4" t="n">
-        <v>11.13</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="T4" t="n">
-        <v>-21.54</v>
+        <v>-37.65</v>
       </c>
       <c r="U4" t="n">
-        <v>11.53</v>
+        <v>3.97</v>
       </c>
       <c r="V4" t="n">
-        <v>17.56</v>
+        <v>11.37</v>
       </c>
       <c r="W4" t="n">
-        <v>24.31</v>
+        <v>7.47</v>
       </c>
       <c r="AA4" t="n">
-        <v>34</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -958,34 +967,34 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iberia-pharmaceuticals-india-limited-drhp_104542.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anchor-offshore-services-limited-drhp_104580.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/IBERIA%20PHARMACEUTICALS%20INDIA%20LIMITED_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anchor%20Offshore%20Services%20Limited-DA_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anchor Offshore Services Limited</t>
+          <t>Karamtara Engineering Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -998,50 +1007,9 @@
           <t>Engineering</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>6400000</v>
-      </c>
-      <c r="L5" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M5" t="n">
-        <v>7000000</v>
-      </c>
-      <c r="N5" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>105.83</v>
-      </c>
-      <c r="R5" t="n">
-        <v>-24.4</v>
-      </c>
-      <c r="S5" t="n">
-        <v>8.039999999999999</v>
-      </c>
-      <c r="T5" t="n">
-        <v>-37.65</v>
-      </c>
-      <c r="U5" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="V5" t="n">
-        <v>11.37</v>
-      </c>
-      <c r="W5" t="n">
-        <v>7.47</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>8.800000000000001</v>
-      </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1051,18 +1019,50 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anchor-offshore-services-limited-drhp_104580.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anchor%20Offshore%20Services%20Limited-DA_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/karamtara-engineering-limited-prospectus_104682.html</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Karamtara Engineering Ltd.</t>
+        </is>
+      </c>
+      <c r="AI5" t="n">
+        <v>11652</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>82.01000000000001</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>34.27</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>31.04</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>25.98</v>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/karamtara-engineering-ltd</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AJ7" t="n">
         <v>21.57</v>
@@ -1256,6 +1256,25 @@
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
         </is>
       </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>National Stock Exchange Of India Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ8" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/national-stock-exchange-of-india-ltd</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1314,11 +1333,17 @@
           <t>Hero Motors Ltd.</t>
         </is>
       </c>
+      <c r="AI9" t="n">
+        <v>4474</v>
+      </c>
       <c r="AJ9" t="n">
         <v>9.18</v>
       </c>
       <c r="AK9" t="n">
         <v>0.99</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>61.63</v>
       </c>
       <c r="AM9" t="n">
         <v>6.64</v>
@@ -1393,11 +1418,17 @@
           <t>Jindal Supreme (India) Ltd.</t>
         </is>
       </c>
+      <c r="AI10" t="n">
+        <v>653</v>
+      </c>
       <c r="AJ10" t="n">
         <v>0</v>
       </c>
       <c r="AK10" t="n">
         <v>0.91</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>73.68000000000001</v>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
@@ -1458,7 +1489,7 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>7834</v>
+        <v>8653</v>
       </c>
       <c r="AJ11" t="n">
         <v>32.01</v>
@@ -1547,14 +1578,17 @@
           <t>SS Retail Ltd.</t>
         </is>
       </c>
+      <c r="AI12" t="n">
+        <v>5690</v>
+      </c>
       <c r="AJ12" t="n">
-        <v>0</v>
+        <v>26.54</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.85</v>
+        <v>1.06</v>
       </c>
       <c r="AL12" t="n">
-        <v>75.73999999999999</v>
+        <v>64.86</v>
       </c>
       <c r="AM12" t="n">
         <v>103.01</v>
@@ -1574,229 +1608,6 @@
       <c r="AR12" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/ss-retail-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Rayzon Solar Limited</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Renewables</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rayzon-solar-limited-addendum-to-the-drhp_104532.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Manika Plastech Limited</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manika-plastech-limited-prospectus_104534.html</t>
-        </is>
-      </c>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>Manika Plastech Ltd.</t>
-        </is>
-      </c>
-      <c r="AI14" t="n">
-        <v>484</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>15.18</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>74.95</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>27.91</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>10.94</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>62.99</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>22.31</v>
-      </c>
-      <c r="AQ14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/manika-plastech-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>LCC Projects Limited</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lcc-projects-limited-prospectus_104530.html</t>
-        </is>
-      </c>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>LCC Projects Ltd.</t>
-        </is>
-      </c>
-      <c r="AI15" t="n">
-        <v>4276</v>
-      </c>
-      <c r="AJ15" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="AK15" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>89.90000000000001</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>20.58</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>7.37</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>42.56</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>18.48</v>
-      </c>
-      <c r="AQ15" t="n">
-        <v>29.45</v>
-      </c>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/lcc-projects-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-25)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR12"/>
+  <dimension ref="A1:AR11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,32 +699,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Madhur Iron &amp; Steel India Limited</t>
+          <t>Anjali Labtech Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>UDRHP</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Metals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -733,37 +728,34 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q2" t="n">
-        <v>444.02</v>
+        <v>615.51</v>
       </c>
       <c r="R2" t="n">
-        <v>30.76</v>
+        <v>30.27</v>
       </c>
       <c r="S2" t="n">
-        <v>23.88</v>
+        <v>200.92</v>
       </c>
       <c r="T2" t="n">
-        <v>31.75</v>
+        <v>36.88</v>
       </c>
       <c r="U2" t="n">
-        <v>5.38</v>
+        <v>32.64</v>
       </c>
       <c r="V2" t="n">
-        <v>11.74</v>
+        <v>42.93</v>
       </c>
       <c r="W2" t="n">
-        <v>22.54</v>
+        <v>47.99</v>
       </c>
       <c r="X2" t="n">
-        <v>16.22</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>1.66</v>
+        <v>46.23</v>
       </c>
       <c r="AA2" t="n">
-        <v>61.9</v>
+        <v>85.7</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -772,7 +764,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -783,12 +775,12 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/madhur-iron-and-steel-india-limited-drhp_104575.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anjali-labtech-limited-udrhp-i_104737.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Madhur%20Iron%20And%20Steel%20India%20Limited%20-%20Draft%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anjali%20Labtech%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
@@ -880,12 +872,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anchor Offshore Services Limited</t>
+          <t>Vardaan Biotech Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -900,12 +892,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Biotechnology</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -913,45 +905,39 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="K4" t="n">
-        <v>6400000</v>
-      </c>
-      <c r="L4" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M4" t="n">
-        <v>7000000</v>
-      </c>
       <c r="N4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q4" t="n">
-        <v>105.83</v>
+        <v>167.09</v>
       </c>
       <c r="R4" t="n">
-        <v>-24.4</v>
+        <v>10.56</v>
       </c>
       <c r="S4" t="n">
-        <v>8.039999999999999</v>
+        <v>18.35</v>
       </c>
       <c r="T4" t="n">
-        <v>-37.65</v>
+        <v>4.19</v>
       </c>
       <c r="U4" t="n">
-        <v>3.97</v>
+        <v>10.98</v>
       </c>
       <c r="V4" t="n">
-        <v>11.37</v>
+        <v>17.03</v>
       </c>
       <c r="W4" t="n">
-        <v>7.47</v>
+        <v>18.43</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.19</v>
       </c>
       <c r="AA4" t="n">
-        <v>8.800000000000001</v>
+        <v>31.1</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -967,12 +953,12 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anchor-offshore-services-limited-drhp_104580.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardaan-biotech-limited-drhp_104652.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anchor%20Offshore%20Services%20Limited-DA_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/VARDAAN%20BIOTECH%20LIMITED_p.pdf</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1000,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -1034,7 +1020,7 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>11652</v>
+        <v>11930</v>
       </c>
       <c r="AJ5" t="n">
         <v>18.75</v>
@@ -1069,7 +1055,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vardaan Biotech Limited</t>
+          <t>Amtech Esters Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1079,22 +1065,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Biotechnology</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1115,14 +1096,51 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardaan-biotech-limited_104652.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/amtech-esters-limited-prospectus_104640.html</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Amtech Esters Ltd.</t>
+        </is>
+      </c>
+      <c r="AI6" t="n">
+        <v>96</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>45.52</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>12.82</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/amtech-esters-ltd</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Amtech Esters Limited</t>
+          <t>National Stock Exchange of India Ltd</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1142,7 +1160,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Market Infrastructure</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1163,56 +1186,41 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/amtech-esters-limited-prospectus_104640.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>Amtech Esters Ltd.</t>
+          <t>National Stock Exchange Of India Ltd.</t>
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>98</v>
+        <v>449955</v>
       </c>
       <c r="AJ7" t="n">
-        <v>21.57</v>
+        <v>22.8</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.17</v>
+        <v>0.01</v>
       </c>
       <c r="AL7" t="n">
-        <v>45.52</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>13.67</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>9.77</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>12.82</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>33.33</v>
+        <v>0</v>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/amtech-esters-ltd</t>
+          <t>https://groww.in/stocks/national-stock-exchange-of-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>National Stock Exchange of India Ltd</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1227,12 +1235,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Market Infrastructure</t>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1242,7 +1250,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -1253,33 +1261,51 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>National Stock Exchange Of India Ltd.</t>
-        </is>
+          <t>Hero Motors Ltd.</t>
+        </is>
+      </c>
+      <c r="AI8" t="n">
+        <v>5369</v>
       </c>
       <c r="AJ8" t="n">
-        <v>22.8</v>
+        <v>9.18</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.01</v>
+        <v>0.99</v>
       </c>
       <c r="AL8" t="n">
-        <v>0</v>
+        <v>61.63</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>-2.38</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/national-stock-exchange-of-india-ltd</t>
+          <t>https://groww.in/stocks/hero-motors-ltd</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Jindal Supreme (India) Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1299,12 +1325,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1314,7 +1335,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
@@ -1325,51 +1346,36 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jindal-supreme-india-limited-prospectus_104621.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Hero Motors Ltd.</t>
+          <t>Jindal Supreme (India) Ltd.</t>
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>4474</v>
+        <v>686</v>
       </c>
       <c r="AJ9" t="n">
-        <v>9.18</v>
+        <v>0</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.99</v>
+        <v>0.91</v>
       </c>
       <c r="AL9" t="n">
-        <v>61.63</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>6.64</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>-2.38</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/hero-motors-ltd</t>
+          <t>https://groww.in/stocks/jindal-supreme-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jindal Supreme (India) Limited</t>
+          <t>Manipal Payment &amp; Identity Solutions Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1410,36 +1416,51 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jindal-supreme-india-limited-prospectus_104621.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manipal-payment-and-identity-solutions-limited-prospectus_104619.html</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>Jindal Supreme (India) Ltd.</t>
+          <t>Manipal Payment And Identity Solutions Ltd.</t>
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>653</v>
+        <v>8338</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0</v>
+        <v>32.01</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.91</v>
+        <v>0.19</v>
       </c>
       <c r="AL10" t="n">
-        <v>73.68000000000001</v>
+        <v>53.92</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>-2.65</v>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/jindal-supreme-india-ltd</t>
+          <t>https://groww.in/stocks/manipal-payment-and-identity-solutions-ltd</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Manipal Payment &amp; Identity Solutions Limited</t>
+          <t>SS Retail Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1459,7 +1480,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Retail</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -1480,132 +1506,42 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manipal-payment-and-identity-solutions-limited-prospectus_104619.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Manipal Payment And Identity Solutions Ltd.</t>
+          <t>SS Retail Ltd.</t>
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>8653</v>
+        <v>6041</v>
       </c>
       <c r="AJ11" t="n">
-        <v>32.01</v>
+        <v>26.54</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.19</v>
+        <v>1.06</v>
       </c>
       <c r="AL11" t="n">
-        <v>53.92</v>
+        <v>64.86</v>
       </c>
       <c r="AM11" t="n">
-        <v>1.17</v>
+        <v>103.01</v>
       </c>
       <c r="AN11" t="n">
-        <v>1.12</v>
+        <v>203.61</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.8</v>
+        <v>143.23</v>
       </c>
       <c r="AP11" t="n">
-        <v>1.86</v>
+        <v>35.81</v>
       </c>
       <c r="AQ11" t="n">
-        <v>-2.65</v>
+        <v>47.17</v>
       </c>
       <c r="AR11" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/manipal-payment-and-identity-solutions-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SS Retail Limited</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
-      </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
-        </is>
-      </c>
-      <c r="AH12" t="inlineStr">
-        <is>
-          <t>SS Retail Ltd.</t>
-        </is>
-      </c>
-      <c r="AI12" t="n">
-        <v>5690</v>
-      </c>
-      <c r="AJ12" t="n">
-        <v>26.54</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>64.86</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>103.01</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>203.61</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>143.23</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>35.81</v>
-      </c>
-      <c r="AQ12" t="n">
-        <v>47.17</v>
-      </c>
-      <c r="AR12" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/ss-retail-ltd</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-28)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR11"/>
+  <dimension ref="A1:AR8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -872,12 +872,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vardaan Biotech Limited</t>
+          <t>JSW One Platforms Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -892,12 +892,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Biotechnology</t>
+          <t>Internet Platforms</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -906,34 +906,28 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q4" t="n">
-        <v>167.09</v>
+        <v>5743.39</v>
       </c>
       <c r="R4" t="n">
-        <v>10.56</v>
+        <v>44.93</v>
       </c>
       <c r="S4" t="n">
-        <v>18.35</v>
-      </c>
-      <c r="T4" t="n">
-        <v>4.19</v>
+        <v>-106.49</v>
       </c>
       <c r="U4" t="n">
-        <v>10.98</v>
+        <v>-1.85</v>
       </c>
       <c r="V4" t="n">
-        <v>17.03</v>
+        <v>-1.17</v>
       </c>
       <c r="W4" t="n">
-        <v>18.43</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0.19</v>
+        <v>-19.14</v>
       </c>
       <c r="AA4" t="n">
-        <v>31.1</v>
+        <v>35</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -953,114 +947,117 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardaan-biotech-limited-drhp_104652.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/VARDAAN%20BIOTECH%20LIMITED_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Karamtara Engineering Limited</t>
+          <t>Vardaan Biotech Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Engineering</t>
-        </is>
+          <t>Biotechnology</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>167.09</v>
+      </c>
+      <c r="R5" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="S5" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="T5" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="U5" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="V5" t="n">
+        <v>17.03</v>
+      </c>
+      <c r="W5" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>31.1</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/karamtara-engineering-limited-prospectus_104682.html</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>Karamtara Engineering Ltd.</t>
-        </is>
-      </c>
-      <c r="AI5" t="n">
-        <v>11930</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>18.75</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>82.01000000000001</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>21.26</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>34.27</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>31.04</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>9.640000000000001</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>25.98</v>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/karamtara-engineering-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardaan-biotech-limited-drhp_104652.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/VARDAAN%20BIOTECH%20LIMITED_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Amtech Esters Limited</t>
+          <t>Karamtara Engineering Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1075,7 +1072,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1096,51 +1098,51 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/amtech-esters-limited-prospectus_104640.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/karamtara-engineering-limited-prospectus_104682.html</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>Amtech Esters Ltd.</t>
+          <t>Karamtara Engineering Ltd.</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>96</v>
+        <v>11544</v>
       </c>
       <c r="AJ6" t="n">
-        <v>21.57</v>
+        <v>18.75</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.17</v>
+        <v>0.91</v>
       </c>
       <c r="AL6" t="n">
-        <v>45.52</v>
+        <v>82.01000000000001</v>
       </c>
       <c r="AM6" t="n">
-        <v>13.67</v>
+        <v>21.26</v>
       </c>
       <c r="AN6" t="n">
-        <v>9.77</v>
+        <v>34.27</v>
       </c>
       <c r="AO6" t="n">
-        <v>12.82</v>
+        <v>31.04</v>
       </c>
       <c r="AP6" t="n">
-        <v>16.4</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="AQ6" t="n">
-        <v>33.33</v>
+        <v>25.98</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/amtech-esters-ltd</t>
+          <t>https://groww.in/stocks/karamtara-engineering-ltd</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>National Stock Exchange of India Ltd</t>
+          <t>Amtech Esters Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1160,12 +1162,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Market Infrastructure</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1186,41 +1183,56 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/amtech-esters-limited-prospectus_104640.html</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>National Stock Exchange Of India Ltd.</t>
+          <t>Amtech Esters Ltd.</t>
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>449955</v>
+        <v>99</v>
       </c>
       <c r="AJ7" t="n">
-        <v>22.8</v>
+        <v>21.57</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.01</v>
+        <v>0.17</v>
       </c>
       <c r="AL7" t="n">
-        <v>0</v>
+        <v>45.52</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>12.82</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>33.33</v>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/national-stock-exchange-of-india-ltd</t>
+          <t>https://groww.in/stocks/amtech-esters-ltd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>National Stock Exchange of India Ltd</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1235,12 +1247,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Automobiles</t>
+          <t>Market Infrastructure</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1250,7 +1262,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -1261,289 +1273,29 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-prospectus_104589.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Hero Motors Ltd.</t>
+          <t>National Stock Exchange Of India Ltd.</t>
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>5369</v>
+        <v>443681</v>
       </c>
       <c r="AJ8" t="n">
-        <v>9.18</v>
+        <v>22.8</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.99</v>
+        <v>0.01</v>
       </c>
       <c r="AL8" t="n">
-        <v>61.63</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>6.64</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>-2.38</v>
+        <v>0</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/hero-motors-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Jindal Supreme (India) Limited</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jindal-supreme-india-limited-prospectus_104621.html</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>Jindal Supreme (India) Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>686</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>73.68000000000001</v>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/jindal-supreme-india-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Manipal Payment &amp; Identity Solutions Limited</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/manipal-payment-and-identity-solutions-limited-prospectus_104619.html</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>Manipal Payment And Identity Solutions Ltd.</t>
-        </is>
-      </c>
-      <c r="AI10" t="n">
-        <v>8338</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>32.01</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>53.92</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>-2.65</v>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/manipal-payment-and-identity-solutions-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SS Retail Limited</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ss-retail-limited-prospectus_104599.html</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>SS Retail Ltd.</t>
-        </is>
-      </c>
-      <c r="AI11" t="n">
-        <v>6041</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>26.54</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>64.86</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>103.01</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>203.61</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>143.23</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>35.81</v>
-      </c>
-      <c r="AQ11" t="n">
-        <v>47.17</v>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/ss-retail-ltd</t>
+          <t>https://groww.in/stocks/national-stock-exchange-of-india-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-29)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR8"/>
+  <dimension ref="A1:AR5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -787,12 +787,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hi-Tech Flow Solutions Limited</t>
+          <t>JSW One Platforms Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -807,7 +807,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Internet Platforms</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -816,31 +821,28 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q3" t="n">
-        <v>417.17</v>
+        <v>5743.39</v>
       </c>
       <c r="R3" t="n">
-        <v>39.86</v>
+        <v>44.93</v>
       </c>
       <c r="S3" t="n">
-        <v>36.42</v>
-      </c>
-      <c r="T3" t="n">
-        <v>50.16</v>
+        <v>-106.49</v>
       </c>
       <c r="U3" t="n">
-        <v>8.73</v>
+        <v>-1.85</v>
       </c>
       <c r="V3" t="n">
-        <v>12.7</v>
+        <v>-1.17</v>
       </c>
       <c r="W3" t="n">
-        <v>32.24</v>
+        <v>-19.14</v>
       </c>
       <c r="AA3" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -860,78 +862,44 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hi-tech-flow-solutions-limited-drhp_104635.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/HitechFlowSolutionsDAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JSW One Platforms Limited</t>
+          <t>Swastika Infra Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Internet Platforms</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>5743.39</v>
-      </c>
-      <c r="R4" t="n">
-        <v>44.93</v>
-      </c>
-      <c r="S4" t="n">
-        <v>-106.49</v>
-      </c>
-      <c r="U4" t="n">
-        <v>-1.85</v>
-      </c>
-      <c r="V4" t="n">
-        <v>-1.17</v>
-      </c>
-      <c r="W4" t="n">
-        <v>-19.14</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>35</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -941,90 +909,72 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/swastika-infra-limited-prospectus_104762.html</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Swastika Infra Ltd</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/swastika-infra-ipo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vardaan Biotech Limited</t>
+          <t>Karamtara Engineering Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Biotechnology</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>167.09</v>
-      </c>
-      <c r="R5" t="n">
-        <v>10.56</v>
-      </c>
-      <c r="S5" t="n">
-        <v>18.35</v>
-      </c>
-      <c r="T5" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="U5" t="n">
-        <v>10.98</v>
-      </c>
-      <c r="V5" t="n">
-        <v>17.03</v>
-      </c>
-      <c r="W5" t="n">
-        <v>18.43</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>31.1</v>
+          <t>Engineering</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1034,268 +984,50 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardaan-biotech-limited-drhp_104652.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/VARDAAN%20BIOTECH%20LIMITED_p.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Karamtara Engineering Limited</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr">
-        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/karamtara-engineering-limited-prospectus_104682.html</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>Karamtara Engineering Ltd.</t>
         </is>
       </c>
-      <c r="AI6" t="n">
-        <v>11544</v>
-      </c>
-      <c r="AJ6" t="n">
+      <c r="AI5" t="n">
+        <v>11578</v>
+      </c>
+      <c r="AJ5" t="n">
         <v>18.75</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AK5" t="n">
         <v>0.91</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AL5" t="n">
         <v>82.01000000000001</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="AM5" t="n">
         <v>21.26</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="AN5" t="n">
         <v>34.27</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AO5" t="n">
         <v>31.04</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="AP5" t="n">
         <v>9.640000000000001</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="AQ5" t="n">
         <v>25.98</v>
       </c>
-      <c r="AR6" t="inlineStr">
+      <c r="AR5" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/karamtara-engineering-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Amtech Esters Limited</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/amtech-esters-limited-prospectus_104640.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Amtech Esters Ltd.</t>
-        </is>
-      </c>
-      <c r="AI7" t="n">
-        <v>99</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>21.57</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>45.52</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>13.67</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>9.77</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>12.82</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/amtech-esters-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>National Stock Exchange of India Ltd</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Market Infrastructure</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/national-stock-exchange-of-india-ltd-prospectus_104637.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>National Stock Exchange Of India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI8" t="n">
-        <v>443681</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/national-stock-exchange-of-india-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-30)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR5"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -787,12 +787,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JSW One Platforms Limited</t>
+          <t>Iris Global Services Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Internet Platforms</t>
+          <t>IT Services</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -821,28 +821,37 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>5743.39</v>
+        <v>4156.44</v>
       </c>
       <c r="R3" t="n">
-        <v>44.93</v>
+        <v>28.72</v>
       </c>
       <c r="S3" t="n">
-        <v>-106.49</v>
+        <v>79.5</v>
+      </c>
+      <c r="T3" t="n">
+        <v>27.62</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.85</v>
+        <v>1.91</v>
       </c>
       <c r="V3" t="n">
-        <v>-1.17</v>
+        <v>3.15</v>
       </c>
       <c r="W3" t="n">
-        <v>-19.14</v>
+        <v>26.62</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>98.23999999999999</v>
       </c>
       <c r="AA3" t="n">
-        <v>35</v>
+        <v>58.9</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -862,44 +871,78 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iris-global-services-limited-drhp_104746.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Iris%20Global%20Services%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Swastika Infra Limited</t>
+          <t>JSW One Platforms Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Internet Platforms</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>5743.39</v>
+      </c>
+      <c r="R4" t="n">
+        <v>44.93</v>
+      </c>
+      <c r="S4" t="n">
+        <v>-106.49</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-1.85</v>
+      </c>
+      <c r="V4" t="n">
+        <v>-1.17</v>
+      </c>
+      <c r="W4" t="n">
+        <v>-19.14</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>35</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -909,47 +952,30 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/swastika-infra-limited-prospectus_104762.html</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>Swastika Infra Ltd</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>7.43</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>3.22</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>18.43</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/swastika-infra-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Karamtara Engineering Limited</t>
+          <t>Rays of Belief Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -964,12 +990,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -990,42 +1011,337 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Rays Of Belief Ltd.</t>
+        </is>
+      </c>
+      <c r="AI5" t="n">
+        <v>536</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>68.77</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>106.83</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>278.82</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>190.99</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ultravibrant Integrated Energy Limited</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ultravibrant-integrated-energy-limited_104809.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Moneyview Limited</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/moneyview-limited-prospectus_104787.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Moneyview Ltd</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
+        <v>97.68000000000001</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>227.45</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>114.9</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/moneyview-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Swastika Infra Limited</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/swastika-infra-limited-prospectus_104762.html</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>Swastika Infra Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ8" t="n">
+        <v>26.42</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>84</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>8.109999999999999</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/swastika-infra-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Karamtara Engineering Limited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/karamtara-engineering-limited-prospectus_104682.html</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AH9" t="inlineStr">
         <is>
           <t>Karamtara Engineering Ltd.</t>
         </is>
       </c>
-      <c r="AI5" t="n">
-        <v>11578</v>
-      </c>
-      <c r="AJ5" t="n">
+      <c r="AI9" t="n">
+        <v>11590</v>
+      </c>
+      <c r="AJ9" t="n">
         <v>18.75</v>
       </c>
-      <c r="AK5" t="n">
+      <c r="AK9" t="n">
         <v>0.91</v>
       </c>
-      <c r="AL5" t="n">
+      <c r="AL9" t="n">
         <v>82.01000000000001</v>
       </c>
-      <c r="AM5" t="n">
+      <c r="AM9" t="n">
         <v>21.26</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="AN9" t="n">
         <v>34.27</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="AO9" t="n">
         <v>31.04</v>
       </c>
-      <c r="AP5" t="n">
+      <c r="AP9" t="n">
         <v>9.640000000000001</v>
       </c>
-      <c r="AQ5" t="n">
+      <c r="AQ9" t="n">
         <v>25.98</v>
       </c>
-      <c r="AR5" t="inlineStr">
+      <c r="AR9" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/karamtara-engineering-ltd</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-01)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AR17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -787,12 +787,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Iris Global Services Limited</t>
+          <t>S. D. International Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -807,12 +807,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>IT Services</t>
+          <t>Food Products</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -821,37 +821,31 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q3" t="n">
-        <v>4156.44</v>
+        <v>302.28</v>
       </c>
       <c r="R3" t="n">
-        <v>28.72</v>
+        <v>34.12</v>
       </c>
       <c r="S3" t="n">
-        <v>79.5</v>
+        <v>32.45</v>
       </c>
       <c r="T3" t="n">
-        <v>27.62</v>
+        <v>59.35</v>
       </c>
       <c r="U3" t="n">
-        <v>1.91</v>
+        <v>10.74</v>
       </c>
       <c r="V3" t="n">
-        <v>3.15</v>
+        <v>19.13</v>
       </c>
       <c r="W3" t="n">
-        <v>26.62</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>98.23999999999999</v>
+        <v>29.51</v>
       </c>
       <c r="AA3" t="n">
-        <v>58.9</v>
+        <v>61.6</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -871,24 +865,24 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iris-global-services-limited-drhp_104746.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-d-international-limited_104826.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Iris%20Global%20Services%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S.%20D.%20INTERNATIONAL%20LIMITED_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JSW One Platforms Limited</t>
+          <t>Iris Global Services Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -908,7 +902,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Internet Platforms</t>
+          <t>IT Services</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -917,28 +911,37 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q4" t="n">
-        <v>5743.39</v>
+        <v>4156.44</v>
       </c>
       <c r="R4" t="n">
-        <v>44.93</v>
+        <v>28.72</v>
       </c>
       <c r="S4" t="n">
-        <v>-106.49</v>
+        <v>79.5</v>
+      </c>
+      <c r="T4" t="n">
+        <v>27.62</v>
       </c>
       <c r="U4" t="n">
-        <v>-1.85</v>
+        <v>1.91</v>
       </c>
       <c r="V4" t="n">
-        <v>-1.17</v>
+        <v>3.15</v>
       </c>
       <c r="W4" t="n">
-        <v>-19.14</v>
+        <v>26.62</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>98.23999999999999</v>
       </c>
       <c r="AA4" t="n">
-        <v>35</v>
+        <v>58.9</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -958,19 +961,19 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iris-global-services-limited-drhp_104746.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Iris%20Global%20Services%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rays of Belief Limited</t>
+          <t>S G Encon Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -980,22 +983,68 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Telecom</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Telecom Services</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>21029642</v>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>286.97</v>
+      </c>
+      <c r="R5" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="S5" t="n">
+        <v>22.89</v>
+      </c>
+      <c r="T5" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="U5" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="V5" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="W5" t="n">
+        <v>24.03</v>
+      </c>
+      <c r="X5" t="n">
+        <v>29.49</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>55.9</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1005,62 +1054,30 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>Rays Of Belief Ltd.</t>
-        </is>
-      </c>
-      <c r="AI5" t="n">
-        <v>536</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>16.24</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>68.77</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>106.83</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>9.06</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>278.82</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>190.99</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-g-encon-limited_104828.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S%20G%20Encon%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ultravibrant Integrated Energy Limited</t>
+          <t>Royal Chain Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1075,17 +1092,49 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Power</t>
-        </is>
+          <t>Jewellery</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>202.6</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="S6" t="n">
+        <v>173.34</v>
+      </c>
+      <c r="T6" t="n">
+        <v>173.71</v>
+      </c>
+      <c r="U6" t="n">
+        <v>85.56</v>
+      </c>
+      <c r="V6" t="n">
+        <v>142.27</v>
+      </c>
+      <c r="W6" t="n">
+        <v>53.34</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>50.6</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1095,45 +1144,84 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ultravibrant-integrated-energy-limited_104809.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/royal-chain-limited-drhp_104015.html</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Royal%20Chain%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Moneyview Limited</t>
+          <t>JSW One Platforms Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Internet Platforms</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>5743.39</v>
+      </c>
+      <c r="R7" t="n">
+        <v>44.93</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-106.49</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-1.85</v>
+      </c>
+      <c r="V7" t="n">
+        <v>-1.17</v>
+      </c>
+      <c r="W7" t="n">
+        <v>-19.14</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>35</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1143,47 +1231,30 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/moneyview-limited-prospectus_104787.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Moneyview Ltd</t>
-        </is>
-      </c>
-      <c r="AM7" t="n">
-        <v>97.68000000000001</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>227.45</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>114.9</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/moneyview-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Swastika Infra Limited</t>
+          <t>SRIT India Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1219,53 +1290,41 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/swastika-infra-limited-prospectus_104762.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Swastika Infra Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ8" t="n">
-        <v>26.42</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>84</v>
+          <t>SRIT India Ltd</t>
+        </is>
       </c>
       <c r="AM8" t="n">
-        <v>7.43</v>
+        <v>121.24</v>
       </c>
       <c r="AN8" t="n">
-        <v>3.22</v>
+        <v>91.84</v>
       </c>
       <c r="AO8" t="n">
-        <v>18.43</v>
+        <v>310.94</v>
       </c>
       <c r="AP8" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>8.109999999999999</v>
+        <v>56.75</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/swastika-infra-ltd</t>
+          <t>https://groww.in/ipo/srit-india-ipo</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Karamtara Engineering Limited</t>
+          <t>A ONE Steels Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1280,12 +1339,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1306,44 +1365,589 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/karamtara-engineering-limited-prospectus_104682.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Karamtara Engineering Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>11590</v>
+          <t>A-One Steels India Ltd.</t>
+        </is>
       </c>
       <c r="AJ9" t="n">
-        <v>18.75</v>
+        <v>15.07</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.91</v>
+        <v>1.25</v>
       </c>
       <c r="AL9" t="n">
-        <v>82.01000000000001</v>
+        <v>85.86</v>
       </c>
       <c r="AM9" t="n">
-        <v>21.26</v>
+        <v>11.35</v>
       </c>
       <c r="AN9" t="n">
-        <v>34.27</v>
+        <v>7.3</v>
       </c>
       <c r="AO9" t="n">
-        <v>31.04</v>
+        <v>24.38</v>
       </c>
       <c r="AP9" t="n">
-        <v>9.640000000000001</v>
+        <v>8.18</v>
       </c>
       <c r="AQ9" t="n">
-        <v>25.98</v>
+        <v>12.35</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/karamtara-engineering-ltd</t>
+          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>J B Ecotex Limited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/j-b-ecotex-limited_104830.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>German Green Steel and Power Limited</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Metals</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-prospectus_104824.html</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>German Green Steel &amp; Power Ltd</t>
+        </is>
+      </c>
+      <c r="AM11" t="n">
+        <v>28.46</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>21.85</v>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/german-green-steel-and-power-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Adroit Industries (India) Limited</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/adroit-industries-india-limited-prospectus_104835.html</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>Adroit Industries (India) Ltd</t>
+        </is>
+      </c>
+      <c r="AI12" t="n">
+        <v>1113</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>20.31</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>71.86</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/adroit-industries-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rays of Belief Limited</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Rays Of Belief Ltd.</t>
+        </is>
+      </c>
+      <c r="AI13" t="n">
+        <v>490</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>68.77</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>106.83</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>278.82</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>190.99</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ultravibrant Integrated Energy Limited</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ultravibrant-integrated-energy-limited_104809.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Acevector Limited</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/acevector-limited-prospectus_104868.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Moneyview Limited</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/moneyview-limited-prospectus_104787.html</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>Moneyview Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ16" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>97.68000000000001</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>227.45</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>114.9</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>61.76</v>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/moneyview-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Swastika Infra Limited</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/swastika-infra-limited-prospectus_104762.html</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>Swastika Infra Ltd.</t>
+        </is>
+      </c>
+      <c r="AI17" t="n">
+        <v>716</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>26.42</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>57.41</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>8.109999999999999</v>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/swastika-infra-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-02)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR17"/>
+  <dimension ref="A1:AR23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,17 +699,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Anjali Labtech Limited</t>
+          <t>S. D. International Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -719,7 +719,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Food Products</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -728,34 +733,31 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>615.51</v>
+        <v>302.28</v>
       </c>
       <c r="R2" t="n">
-        <v>30.27</v>
+        <v>34.12</v>
       </c>
       <c r="S2" t="n">
-        <v>200.92</v>
+        <v>32.45</v>
       </c>
       <c r="T2" t="n">
-        <v>36.88</v>
+        <v>59.35</v>
       </c>
       <c r="U2" t="n">
-        <v>32.64</v>
+        <v>10.74</v>
       </c>
       <c r="V2" t="n">
-        <v>42.93</v>
+        <v>19.13</v>
       </c>
       <c r="W2" t="n">
-        <v>47.99</v>
-      </c>
-      <c r="X2" t="n">
-        <v>46.23</v>
+        <v>29.51</v>
       </c>
       <c r="AA2" t="n">
-        <v>85.7</v>
+        <v>61.6</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -764,7 +766,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -775,24 +777,24 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/anjali-labtech-limited-udrhp-i_104737.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-d-international-limited_104826.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Anjali%20Labtech%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S.%20D.%20INTERNATIONAL%20LIMITED_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S. D. International Limited</t>
+          <t>Ultravibrant Integrated Energy Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -807,12 +809,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Food Products</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -824,28 +826,25 @@
         <v>10</v>
       </c>
       <c r="Q3" t="n">
-        <v>302.28</v>
+        <v>383.99</v>
       </c>
       <c r="R3" t="n">
-        <v>34.12</v>
+        <v>57.32</v>
       </c>
       <c r="S3" t="n">
-        <v>32.45</v>
+        <v>33.39</v>
       </c>
       <c r="T3" t="n">
-        <v>59.35</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="U3" t="n">
-        <v>10.74</v>
-      </c>
-      <c r="V3" t="n">
-        <v>19.13</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="W3" t="n">
-        <v>29.51</v>
+        <v>82.12</v>
       </c>
       <c r="AA3" t="n">
-        <v>61.6</v>
+        <v>59.9</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -865,24 +864,24 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-d-international-limited_104826.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ultravibrant-integrated-energy-limited-drhp_104809.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S.%20D.%20INTERNATIONAL%20LIMITED_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/ULTRAVIBRANT%20INTEGRATED%20ENERGY%20LIMITED_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Iris Global Services Limited</t>
+          <t>Ekkaa Electronics (India) Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -897,12 +896,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>IT Services</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -911,37 +910,31 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q4" t="n">
-        <v>4156.44</v>
+        <v>1221.76</v>
       </c>
       <c r="R4" t="n">
-        <v>28.72</v>
+        <v>146.07</v>
       </c>
       <c r="S4" t="n">
-        <v>79.5</v>
+        <v>65.38</v>
       </c>
       <c r="T4" t="n">
-        <v>27.62</v>
+        <v>177.59</v>
       </c>
       <c r="U4" t="n">
-        <v>1.91</v>
+        <v>5.35</v>
       </c>
       <c r="V4" t="n">
-        <v>3.15</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="W4" t="n">
-        <v>26.62</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>98.23999999999999</v>
+        <v>25.99</v>
       </c>
       <c r="AA4" t="n">
-        <v>58.9</v>
+        <v>59</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -961,24 +954,24 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iris-global-services-limited-drhp_104746.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/ekkaa-electronics-india-limited-drhp_104862.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Iris%20Global%20Services%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EKKAA%20ELECTRONICS%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S G Encon Limited</t>
+          <t>Iris Global Services Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -993,12 +986,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Telecom Services</t>
+          <t>IT Services</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1006,41 +999,38 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="K5" t="n">
-        <v>21029642</v>
-      </c>
       <c r="N5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>286.97</v>
+        <v>4156.44</v>
       </c>
       <c r="R5" t="n">
-        <v>3.94</v>
+        <v>28.72</v>
       </c>
       <c r="S5" t="n">
-        <v>22.89</v>
+        <v>79.5</v>
       </c>
       <c r="T5" t="n">
-        <v>64.2</v>
+        <v>27.62</v>
       </c>
       <c r="U5" t="n">
-        <v>7.96</v>
+        <v>1.91</v>
       </c>
       <c r="V5" t="n">
-        <v>10.77</v>
+        <v>3.15</v>
       </c>
       <c r="W5" t="n">
-        <v>24.03</v>
-      </c>
-      <c r="X5" t="n">
-        <v>29.49</v>
+        <v>26.62</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.09</v>
+        <v>0.79</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>98.23999999999999</v>
       </c>
       <c r="AA5" t="n">
-        <v>55.9</v>
+        <v>58.9</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -1060,24 +1050,24 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-g-encon-limited_104828.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iris-global-services-limited-drhp_104746.html</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S%20G%20Encon%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Iris%20Global%20Services%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Royal Chain Limited</t>
+          <t>S G Encon Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1092,45 +1082,54 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Telecom</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Telecom Services</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
+      </c>
+      <c r="K6" t="n">
+        <v>21029642</v>
       </c>
       <c r="N6" t="n">
         <v>10</v>
       </c>
       <c r="Q6" t="n">
-        <v>202.6</v>
+        <v>286.97</v>
       </c>
       <c r="R6" t="n">
-        <v>0.05</v>
+        <v>3.94</v>
       </c>
       <c r="S6" t="n">
-        <v>173.34</v>
+        <v>22.89</v>
       </c>
       <c r="T6" t="n">
-        <v>173.71</v>
+        <v>64.2</v>
       </c>
       <c r="U6" t="n">
-        <v>85.56</v>
+        <v>7.96</v>
       </c>
       <c r="V6" t="n">
-        <v>142.27</v>
+        <v>10.77</v>
       </c>
       <c r="W6" t="n">
-        <v>53.34</v>
+        <v>24.03</v>
+      </c>
+      <c r="X6" t="n">
+        <v>29.49</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.09</v>
       </c>
       <c r="AA6" t="n">
-        <v>50.6</v>
+        <v>55.9</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
@@ -1150,24 +1149,24 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/royal-chain-limited-drhp_104015.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-g-encon-limited_104828.html</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Royal%20Chain%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S%20G%20Encon%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JSW One Platforms Limited</t>
+          <t>Royal Chain Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1182,12 +1181,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Internet Platforms</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1199,25 +1198,28 @@
         <v>10</v>
       </c>
       <c r="Q7" t="n">
-        <v>5743.39</v>
+        <v>202.6</v>
       </c>
       <c r="R7" t="n">
-        <v>44.93</v>
+        <v>0.05</v>
       </c>
       <c r="S7" t="n">
-        <v>-106.49</v>
+        <v>173.34</v>
+      </c>
+      <c r="T7" t="n">
+        <v>173.71</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.85</v>
+        <v>85.56</v>
       </c>
       <c r="V7" t="n">
-        <v>-1.17</v>
+        <v>142.27</v>
       </c>
       <c r="W7" t="n">
-        <v>-19.14</v>
+        <v>53.34</v>
       </c>
       <c r="AA7" t="n">
-        <v>35</v>
+        <v>50.6</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
@@ -1237,34 +1239,34 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/jsw-one-platforms-limited-drhp_104742.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/royal-chain-limited-drhp_104015.html</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/JSW One Platforms Limited - Draft Abridged Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Royal%20Chain%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SRIT India Limited</t>
+          <t>AITMC Ventures Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>UDRHP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1272,54 +1274,69 @@
           <t>Unclassified</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>106.76</v>
+      </c>
+      <c r="R8" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="S8" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-17.09</v>
+      </c>
+      <c r="U8" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="V8" t="n">
+        <v>26.74</v>
+      </c>
+      <c r="W8" t="n">
+        <v>19.04</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>39</v>
+      </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>SRIT India Ltd</t>
-        </is>
-      </c>
-      <c r="AM8" t="n">
-        <v>121.24</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>91.84</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>310.94</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>56.75</v>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/srit-india-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/aitmc-ventures-limited-udrhp-i_104864.html</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/AITMC%20Ventures%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A ONE Steels Limited</t>
+          <t>Jagatjit Agri Engineering Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1329,27 +1346,53 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Metals</t>
-        </is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="N9" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>413.97</v>
+      </c>
+      <c r="R9" t="n">
+        <v>331.55</v>
+      </c>
+      <c r="V9" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="W9" t="n">
+        <v>53.89</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>36.2</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -1359,74 +1402,50 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>A-One Steels India Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ9" t="n">
-        <v>15.07</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>85.86</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>11.35</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>24.38</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>8.18</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>12.35</v>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>J B Ecotex Limited</t>
+          <t>Arohan Financial Services Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NBFC</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1436,7 +1455,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -1447,39 +1466,39 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/j-b-ecotex-limited_104830.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>German Green Steel and Power Limited</t>
+          <t>Koolking Industries India Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -1489,7 +1508,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -1500,61 +1519,34 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-prospectus_104824.html</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>German Green Steel &amp; Power Ltd</t>
-        </is>
-      </c>
-      <c r="AM11" t="n">
-        <v>28.46</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>20.93</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>53.91</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>21.85</v>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/german-green-steel-and-power-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/koolking-industries-india-limited_104848.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Adroit Industries (India) Limited</t>
+          <t>Sai Infinium Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Diversified Industrials</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -1575,51 +1567,29 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/adroit-industries-india-limited-prospectus_104835.html</t>
-        </is>
-      </c>
-      <c r="AH12" t="inlineStr">
-        <is>
-          <t>Adroit Industries (India) Ltd</t>
-        </is>
-      </c>
-      <c r="AI12" t="n">
-        <v>1113</v>
-      </c>
-      <c r="AJ12" t="n">
-        <v>20.31</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>71.86</v>
-      </c>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/adroit-industries-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sai-infinium-limited_104850.html</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rays of Belief Limited</t>
+          <t>J Infratech Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1645,76 +1615,34 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
-        </is>
-      </c>
-      <c r="AH13" t="inlineStr">
-        <is>
-          <t>Rays Of Belief Ltd.</t>
-        </is>
-      </c>
-      <c r="AI13" t="n">
-        <v>490</v>
-      </c>
-      <c r="AJ13" t="n">
-        <v>16.24</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>68.77</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>106.83</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>9.06</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>278.82</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>190.99</v>
-      </c>
-      <c r="AQ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/j-infratech-limited_104846.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ultravibrant Integrated Energy Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Power</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -1735,19 +1663,41 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ultravibrant-integrated-energy-limited_104809.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Runwal Enterprises Ltd</t>
+        </is>
+      </c>
+      <c r="AM14" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/runwal-enterprises-ipo</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Acevector Limited</t>
+          <t>SRIT India Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1783,19 +1733,41 @@
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/acevector-limited-prospectus_104868.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>SRIT India Ltd</t>
+        </is>
+      </c>
+      <c r="AM15" t="n">
+        <v>121.24</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>91.84</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>310.94</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>56.75</v>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/srit-india-ipo</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Moneyview Limited</t>
+          <t>A ONE Steels Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1810,7 +1782,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Metals</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -1831,60 +1808,66 @@
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/moneyview-limited-prospectus_104787.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
         </is>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Moneyview Ltd.</t>
-        </is>
+          <t>A-One Steels India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI16" t="n">
+        <v>3221</v>
       </c>
       <c r="AJ16" t="n">
-        <v>17.63</v>
+        <v>15.07</v>
       </c>
       <c r="AK16" t="n">
-        <v>2.33</v>
+        <v>1.25</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>74.51000000000001</v>
       </c>
       <c r="AM16" t="n">
-        <v>97.68000000000001</v>
+        <v>11.35</v>
       </c>
       <c r="AN16" t="n">
-        <v>227.45</v>
+        <v>7.3</v>
       </c>
       <c r="AO16" t="n">
-        <v>114.9</v>
+        <v>24.38</v>
       </c>
       <c r="AP16" t="n">
-        <v>18.24</v>
+        <v>8.18</v>
       </c>
       <c r="AQ16" t="n">
-        <v>61.76</v>
+        <v>12.35</v>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/moneyview-ltd</t>
+          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Swastika Infra Limited</t>
+          <t>J B Ecotex Limited</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1910,42 +1893,458 @@
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/j-b-ecotex-limited_104830.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>German Green Steel and Power Limited</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Metals</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-prospectus_104824.html</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>German Green Steel &amp; Power Ltd</t>
+        </is>
+      </c>
+      <c r="AM18" t="n">
+        <v>28.46</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>21.85</v>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/german-green-steel-and-power-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Adroit Industries (India) Limited</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/adroit-industries-india-limited-prospectus_104835.html</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>Adroit Industries (India) Ltd</t>
+        </is>
+      </c>
+      <c r="AI19" t="n">
+        <v>1057</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>20.31</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>71.86</v>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/adroit-industries-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rays of Belief Limited</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>Rays Of Belief Ltd.</t>
+        </is>
+      </c>
+      <c r="AI20" t="n">
+        <v>474</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>68.77</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>106.83</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>278.82</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>190.99</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Acevector Limited</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/acevector-limited-prospectus_104868.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Moneyview Limited</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/moneyview-limited-prospectus_104787.html</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>Moneyview Ltd.</t>
+        </is>
+      </c>
+      <c r="AI22" t="n">
+        <v>9511</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>19.31</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>97.68000000000001</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>227.45</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>114.9</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>61.76</v>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/moneyview-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Swastika Infra Limited</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr">
+        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/swastika-infra-limited-prospectus_104762.html</t>
         </is>
       </c>
-      <c r="AH17" t="inlineStr">
+      <c r="AH23" t="inlineStr">
         <is>
           <t>Swastika Infra Ltd.</t>
         </is>
       </c>
-      <c r="AI17" t="n">
-        <v>716</v>
-      </c>
-      <c r="AJ17" t="n">
+      <c r="AI23" t="n">
+        <v>737</v>
+      </c>
+      <c r="AJ23" t="n">
         <v>26.42</v>
       </c>
-      <c r="AK17" t="n">
+      <c r="AK23" t="n">
         <v>0.73</v>
       </c>
-      <c r="AL17" t="n">
+      <c r="AL23" t="n">
         <v>57.41</v>
       </c>
-      <c r="AM17" t="n">
+      <c r="AM23" t="n">
         <v>7.43</v>
       </c>
-      <c r="AN17" t="n">
+      <c r="AN23" t="n">
         <v>3.22</v>
       </c>
-      <c r="AO17" t="n">
+      <c r="AO23" t="n">
         <v>18.43</v>
       </c>
-      <c r="AP17" t="n">
+      <c r="AP23" t="n">
         <v>5.08</v>
       </c>
-      <c r="AQ17" t="n">
+      <c r="AQ23" t="n">
         <v>8.109999999999999</v>
       </c>
-      <c r="AR17" t="inlineStr">
+      <c r="AR23" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/swastika-infra-ltd</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-03)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR23"/>
+  <dimension ref="A1:AR22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1668,8 +1668,17 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Ltd</t>
-        </is>
+          <t>Runwal Enterprises Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ14" t="n">
+        <v>17.21</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>99.98999999999999</v>
       </c>
       <c r="AM14" t="n">
         <v>2.45</v>
@@ -1685,7 +1694,7 @@
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/runwal-enterprises-ipo</t>
+          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
         </is>
       </c>
     </row>
@@ -1951,8 +1960,14 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>German Green Steel &amp; Power Ltd</t>
-        </is>
+          <t>German Green Steel and Power Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ18" t="n">
+        <v>18.95</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0.8100000000000001</v>
       </c>
       <c r="AM18" t="n">
         <v>28.46</v>
@@ -1968,7 +1983,7 @@
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/german-green-steel-and-power-ipo</t>
+          <t>https://groww.in/stocks/german-green-steel-and-power-ltd</t>
         </is>
       </c>
     </row>
@@ -2262,91 +2277,6 @@
       <c r="AR22" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/moneyview-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Swastika Infra Limited</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE23" t="inlineStr"/>
-      <c r="AF23" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/swastika-infra-limited-prospectus_104762.html</t>
-        </is>
-      </c>
-      <c r="AH23" t="inlineStr">
-        <is>
-          <t>Swastika Infra Ltd.</t>
-        </is>
-      </c>
-      <c r="AI23" t="n">
-        <v>737</v>
-      </c>
-      <c r="AJ23" t="n">
-        <v>26.42</v>
-      </c>
-      <c r="AK23" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="AL23" t="n">
-        <v>57.41</v>
-      </c>
-      <c r="AM23" t="n">
-        <v>7.43</v>
-      </c>
-      <c r="AN23" t="n">
-        <v>3.22</v>
-      </c>
-      <c r="AO23" t="n">
-        <v>18.43</v>
-      </c>
-      <c r="AP23" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="AQ23" t="n">
-        <v>8.109999999999999</v>
-      </c>
-      <c r="AR23" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/swastika-infra-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-05)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR22"/>
+  <dimension ref="A1:AR34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S. D. International Limited</t>
+          <t>Kataline Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -719,12 +719,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Food Products</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -736,28 +731,31 @@
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>302.28</v>
+        <v>220.58</v>
       </c>
       <c r="R2" t="n">
-        <v>34.12</v>
+        <v>38.79</v>
       </c>
       <c r="S2" t="n">
-        <v>32.45</v>
+        <v>26.83</v>
       </c>
       <c r="T2" t="n">
-        <v>59.35</v>
+        <v>61.15</v>
       </c>
       <c r="U2" t="n">
-        <v>10.74</v>
+        <v>12.16</v>
       </c>
       <c r="V2" t="n">
-        <v>19.13</v>
+        <v>16.44</v>
       </c>
       <c r="W2" t="n">
-        <v>29.51</v>
+        <v>26.27</v>
+      </c>
+      <c r="X2" t="n">
+        <v>34.86</v>
       </c>
       <c r="AA2" t="n">
-        <v>61.6</v>
+        <v>77.8</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -777,24 +775,24 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-d-international-limited_104826.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kataline-limited-drhp_104993.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S.%20D.%20INTERNATIONAL%20LIMITED_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/KATALINE%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ultravibrant Integrated Energy Limited</t>
+          <t>J Infratech Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -809,42 +807,54 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
+      </c>
+      <c r="L3" t="n">
+        <v>10000000</v>
       </c>
       <c r="N3" t="n">
         <v>10</v>
       </c>
       <c r="Q3" t="n">
-        <v>383.99</v>
+        <v>1721.76</v>
       </c>
       <c r="R3" t="n">
-        <v>57.32</v>
+        <v>22.01</v>
       </c>
       <c r="S3" t="n">
-        <v>33.39</v>
+        <v>246.59</v>
       </c>
       <c r="T3" t="n">
-        <v>67.34999999999999</v>
+        <v>26.24</v>
       </c>
       <c r="U3" t="n">
-        <v>8.699999999999999</v>
+        <v>14.32</v>
+      </c>
+      <c r="V3" t="n">
+        <v>25.14</v>
       </c>
       <c r="W3" t="n">
-        <v>82.12</v>
+        <v>41.75</v>
+      </c>
+      <c r="X3" t="n">
+        <v>39.72</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1.04</v>
       </c>
       <c r="AA3" t="n">
-        <v>59.9</v>
+        <v>74</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -864,24 +874,24 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/ultravibrant-integrated-energy-limited-drhp_104809.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/j-infratech-limited-drhp_104846.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/ULTRAVIBRANT%20INTEGRATED%20ENERGY%20LIMITED_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/J%20Infratech%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ekkaa Electronics (India) Limited</t>
+          <t>Shreejikrupa Project Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -901,7 +911,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -913,28 +923,34 @@
         <v>5</v>
       </c>
       <c r="Q4" t="n">
-        <v>1221.76</v>
+        <v>1385.68</v>
       </c>
       <c r="R4" t="n">
-        <v>146.07</v>
+        <v>62.52</v>
       </c>
       <c r="S4" t="n">
-        <v>65.38</v>
+        <v>79.34</v>
       </c>
       <c r="T4" t="n">
-        <v>177.59</v>
+        <v>19.36</v>
       </c>
       <c r="U4" t="n">
-        <v>5.35</v>
+        <v>5.66</v>
       </c>
       <c r="V4" t="n">
-        <v>9.369999999999999</v>
+        <v>8.91</v>
       </c>
       <c r="W4" t="n">
-        <v>25.99</v>
+        <v>26.53</v>
+      </c>
+      <c r="X4" t="n">
+        <v>21.66</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>85.56</v>
       </c>
       <c r="AA4" t="n">
-        <v>59</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -954,24 +970,24 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/ekkaa-electronics-india-limited-drhp_104862.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/shreejikrupa-project-limited-drhp_104991.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EKKAA%20ELECTRONICS%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/SHREEJIKRUPA%20PROJECT%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Iris Global Services Limited</t>
+          <t>Ekkaa Electronics (India) Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -986,12 +1002,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>IT Services</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1000,37 +1016,31 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q5" t="n">
-        <v>4156.44</v>
+        <v>1221.76</v>
       </c>
       <c r="R5" t="n">
-        <v>28.72</v>
+        <v>146.07</v>
       </c>
       <c r="S5" t="n">
-        <v>79.5</v>
+        <v>65.38</v>
       </c>
       <c r="T5" t="n">
-        <v>27.62</v>
+        <v>177.59</v>
       </c>
       <c r="U5" t="n">
-        <v>1.91</v>
+        <v>5.35</v>
       </c>
       <c r="V5" t="n">
-        <v>3.15</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="W5" t="n">
-        <v>26.62</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>98.23999999999999</v>
+        <v>25.99</v>
       </c>
       <c r="AA5" t="n">
-        <v>58.9</v>
+        <v>59</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -1050,19 +1060,19 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/iris-global-services-limited-drhp_104746.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/ekkaa-electronics-india-limited-drhp_104862.html</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Iris%20Global%20Services%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EKKAA%20ELECTRONICS%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S G Encon Limited</t>
+          <t>Biocon Electric Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1082,54 +1092,46 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Telecom</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Telecom Services</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
-      </c>
-      <c r="K6" t="n">
-        <v>21029642</v>
       </c>
       <c r="N6" t="n">
         <v>10</v>
       </c>
       <c r="Q6" t="n">
-        <v>286.97</v>
+        <v>196.73</v>
       </c>
       <c r="R6" t="n">
-        <v>3.94</v>
+        <v>37.94</v>
       </c>
       <c r="S6" t="n">
-        <v>22.89</v>
+        <v>14.14</v>
       </c>
       <c r="T6" t="n">
-        <v>64.2</v>
+        <v>22.96</v>
       </c>
       <c r="U6" t="n">
-        <v>7.96</v>
+        <v>7.14</v>
       </c>
       <c r="V6" t="n">
-        <v>10.77</v>
+        <v>12.94</v>
       </c>
       <c r="W6" t="n">
-        <v>24.03</v>
+        <v>24.05</v>
       </c>
       <c r="X6" t="n">
-        <v>29.49</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0.09</v>
+        <v>12.19</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>90</v>
       </c>
       <c r="AA6" t="n">
-        <v>55.9</v>
+        <v>58.1</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
@@ -1149,24 +1151,24 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/s-g-encon-limited_104828.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/biocon-electric-limited-drhp_104995.html</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/S%20G%20Encon%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Biocon%20Electric%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Royal Chain Limited</t>
+          <t>Anarock Property Consultants Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1181,12 +1183,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1195,31 +1197,34 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>202.6</v>
+        <v>881.9</v>
       </c>
       <c r="R7" t="n">
-        <v>0.05</v>
+        <v>33.83</v>
       </c>
       <c r="S7" t="n">
-        <v>173.34</v>
+        <v>93.22</v>
       </c>
       <c r="T7" t="n">
-        <v>173.71</v>
+        <v>53.38</v>
       </c>
       <c r="U7" t="n">
-        <v>85.56</v>
+        <v>10.57</v>
       </c>
       <c r="V7" t="n">
-        <v>142.27</v>
+        <v>17.1</v>
       </c>
       <c r="W7" t="n">
-        <v>53.34</v>
+        <v>15.64</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>66.41</v>
       </c>
       <c r="AA7" t="n">
-        <v>50.6</v>
+        <v>57.6</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
@@ -1239,29 +1244,29 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/royal-chain-limited-drhp_104015.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/anarock-property-consultants-limited_105006.html</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Royal%20Chain%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Anarock%20Property%20Consultants%20Limited%20-%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AITMC Ventures Limited</t>
+          <t>Royal Chain Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1271,7 +1276,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1280,31 +1290,31 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q8" t="n">
-        <v>106.76</v>
+        <v>202.6</v>
       </c>
       <c r="R8" t="n">
-        <v>22.05</v>
+        <v>0.05</v>
       </c>
       <c r="S8" t="n">
-        <v>13.38</v>
+        <v>173.34</v>
       </c>
       <c r="T8" t="n">
-        <v>-17.09</v>
+        <v>173.71</v>
       </c>
       <c r="U8" t="n">
-        <v>12.54</v>
+        <v>85.56</v>
       </c>
       <c r="V8" t="n">
-        <v>26.74</v>
+        <v>142.27</v>
       </c>
       <c r="W8" t="n">
-        <v>19.04</v>
+        <v>53.34</v>
       </c>
       <c r="AA8" t="n">
-        <v>39</v>
+        <v>50.6</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
@@ -1313,7 +1323,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -1324,24 +1334,24 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/aitmc-ventures-limited-udrhp-i_104864.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/royal-chain-limited-drhp_104015.html</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/AITMC%20Ventures%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Royal%20Chain%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jagatjit Agri Engineering Limited</t>
+          <t>Vardhman Appliances Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1361,7 +1371,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1369,26 +1379,35 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="L9" t="n">
-        <v>3100000</v>
-      </c>
       <c r="N9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>413.97</v>
+        <v>869.62</v>
       </c>
       <c r="R9" t="n">
-        <v>331.55</v>
+        <v>4.03</v>
+      </c>
+      <c r="S9" t="n">
+        <v>22.48</v>
+      </c>
+      <c r="T9" t="n">
+        <v>21.42</v>
+      </c>
+      <c r="U9" t="n">
+        <v>2.59</v>
       </c>
       <c r="V9" t="n">
-        <v>13.46</v>
+        <v>5.98</v>
       </c>
       <c r="W9" t="n">
-        <v>53.89</v>
+        <v>25.27</v>
+      </c>
+      <c r="X9" t="n">
+        <v>24.01</v>
       </c>
       <c r="AA9" t="n">
-        <v>36.2</v>
+        <v>45.3</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1408,29 +1427,29 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardhman-appliances-limited-drhp_104999.html</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Vardhman%20Appliances%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Arohan Financial Services Limited</t>
+          <t>Pci Infraprojects Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1440,50 +1459,90 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>NBFC</t>
-        </is>
+          <t>Renewables</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>304.09</v>
+      </c>
+      <c r="R10" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="S10" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="T10" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="U10" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="V10" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="W10" t="n">
+        <v>36.29</v>
+      </c>
+      <c r="X10" t="n">
+        <v>39.97</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>43.9</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Koolking Industries India Limited</t>
+          <t>AITMC Ventures Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>UDRHP</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1493,40 +1552,72 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Diversified Industrials</t>
-        </is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>106.76</v>
+      </c>
+      <c r="R11" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="S11" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="T11" t="n">
+        <v>-17.09</v>
+      </c>
+      <c r="U11" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="V11" t="n">
+        <v>26.74</v>
+      </c>
+      <c r="W11" t="n">
+        <v>19.04</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>39</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/koolking-industries-india-limited_104848.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/aitmc-ventures-limited-udrhp-i_104864.html</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/AITMC%20Ventures%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sai Infinium Limited</t>
+          <t>Jagatjit Agri Engineering Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1546,12 +1637,43 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="N12" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>413.97</v>
+      </c>
+      <c r="R12" t="n">
+        <v>331.55</v>
+      </c>
+      <c r="V12" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="W12" t="n">
+        <v>53.89</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>36.2</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
@@ -1561,20 +1683,25 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sai-infinium-limited_104850.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>J Infratech Limited</t>
+          <t>Koolking Industries India Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1594,12 +1721,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>526.75</v>
+      </c>
+      <c r="R13" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="W13" t="n">
+        <v>35.28</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>22.6</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>MONITOR</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -1609,35 +1761,40 @@
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/j-infratech-limited_104846.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/koolking-industries-india-limited-drhp_104848.html</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Koolking%20Industries%20India%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>Arete 22 Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1663,65 +1820,39 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
-        </is>
-      </c>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>Runwal Enterprises Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ14" t="n">
-        <v>17.21</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>99.98999999999999</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited_105016.html</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SRIT India Limited</t>
+          <t>Deon Energy Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Power</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -1742,61 +1873,39 @@
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
-        </is>
-      </c>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>SRIT India Ltd</t>
-        </is>
-      </c>
-      <c r="AM15" t="n">
-        <v>121.24</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>91.84</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>310.94</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>56.75</v>
-      </c>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/srit-india-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/deon-energy-limited_105012.html</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>A ONE Steels Limited</t>
+          <t>Rathod Jewellery Manufacturing Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -1817,56 +1926,19 @@
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
-        </is>
-      </c>
-      <c r="AH16" t="inlineStr">
-        <is>
-          <t>A-One Steels India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI16" t="n">
-        <v>3221</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>15.07</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>74.51000000000001</v>
-      </c>
-      <c r="AM16" t="n">
-        <v>11.35</v>
-      </c>
-      <c r="AN16" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="AO16" t="n">
-        <v>24.38</v>
-      </c>
-      <c r="AP16" t="n">
-        <v>8.18</v>
-      </c>
-      <c r="AQ16" t="n">
-        <v>12.35</v>
-      </c>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rathod-jewellery-manufacturing-limited_105014.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>J B Ecotex Limited</t>
+          <t>Inox Clean Energy Limited</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1881,7 +1953,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Power</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
@@ -1902,39 +1979,34 @@
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/j-b-ecotex-limited_104830.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited_105010.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>German Green Steel and Power Limited</t>
+          <t>Rudra Green Ship Recycling Limited</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Metals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
@@ -1944,7 +2016,7 @@
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
@@ -1955,57 +2027,29 @@
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-prospectus_104824.html</t>
-        </is>
-      </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>German Green Steel and Power Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ18" t="n">
-        <v>18.95</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AM18" t="n">
-        <v>28.46</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>20.93</v>
-      </c>
-      <c r="AO18" t="n">
-        <v>53.91</v>
-      </c>
-      <c r="AP18" t="n">
-        <v>21.85</v>
-      </c>
-      <c r="AR18" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/german-green-steel-and-power-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited_105008.html</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Adroit Industries (India) Limited</t>
+          <t>Sanghvi Housing and Infrastructure Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2015,7 +2059,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Diversified Industrials</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
@@ -2036,56 +2080,44 @@
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/adroit-industries-india-limited-prospectus_104835.html</t>
-        </is>
-      </c>
-      <c r="AH19" t="inlineStr">
-        <is>
-          <t>Adroit Industries (India) Ltd</t>
-        </is>
-      </c>
-      <c r="AI19" t="n">
-        <v>1057</v>
-      </c>
-      <c r="AJ19" t="n">
-        <v>20.31</v>
-      </c>
-      <c r="AK19" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="AL19" t="n">
-        <v>71.86</v>
-      </c>
-      <c r="AR19" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/adroit-industries-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sanghvi-housing-and-infrastructure-limited-drhp_105004.html</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Sanghvi%20Housing_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Rays of Belief Limited</t>
+          <t>Tanvi Exports India Limited</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Agri Exports</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -2106,66 +2138,29 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
-        </is>
-      </c>
-      <c r="AH20" t="inlineStr">
-        <is>
-          <t>Rays Of Belief Ltd.</t>
-        </is>
-      </c>
-      <c r="AI20" t="n">
-        <v>474</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>16.24</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>68.77</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>106.83</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>9.06</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>278.82</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>190.99</v>
-      </c>
-      <c r="AQ20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR20" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tanvi-exports-india-limited_105002.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Acevector Limited</t>
+          <t>Nnt Developers Limited</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2191,34 +2186,39 @@
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/acevector-limited-prospectus_104868.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited_105000.html</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Moneyview Limited</t>
+          <t>Kian-M Export Limited</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Agri Exports</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -2239,42 +2239,865 @@
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kian-m-export-limited_104874.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Arohan Financial Services Limited</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>NBFC</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sai Infinium Limited</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sai-infinium-limited_104850.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sonaselection India Limited</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sonaselection-india-limited-prospectus_104876.html</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>Sonaselection India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>525</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>32.66</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>64.52</v>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/sonaselection-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Runwal Enterprises Limited</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>Runwal Enterprises Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ26" t="n">
+        <v>17.21</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>84.61</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SRIT India Limited</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>SRIT India Ltd</t>
+        </is>
+      </c>
+      <c r="AM27" t="n">
+        <v>121.24</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>91.84</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>310.94</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>56.75</v>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/srit-india-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>A ONE Steels Limited</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Metals</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>A-One Steels India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>3221</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>15.07</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>74.51000000000001</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>11.35</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>24.38</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>J B Ecotex Limited</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/j-b-ecotex-limited_104830.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Adroit Industries (India) Limited</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/adroit-industries-india-limited-prospectus_104835.html</t>
+        </is>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>Adroit Industries (India) Ltd</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>1057</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>20.31</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>71.86</v>
+      </c>
+      <c r="AR30" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/adroit-industries-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>German Green Steel and Power Limited</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Metals</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-prospectus_104824.html</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>German Green Steel and Power Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ31" t="n">
+        <v>18.95</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>68.54000000000001</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>28.46</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>21.85</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="AR31" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/german-green-steel-and-power-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Rays of Belief Limited</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>Rays Of Belief Ltd.</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>474</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>68.77</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>106.83</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>278.82</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>190.99</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR32" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Acevector Limited</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/acevector-limited-prospectus_104868.html</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>AceVector Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ33" t="n">
+        <v>-59.54</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>49.96</v>
+      </c>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/acevector-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Moneyview Limited</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr"/>
+      <c r="AF34" t="inlineStr">
+        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/moneyview-limited-prospectus_104787.html</t>
         </is>
       </c>
-      <c r="AH22" t="inlineStr">
+      <c r="AH34" t="inlineStr">
         <is>
           <t>Moneyview Ltd.</t>
         </is>
       </c>
-      <c r="AI22" t="n">
+      <c r="AI34" t="n">
         <v>9511</v>
       </c>
-      <c r="AJ22" t="n">
+      <c r="AJ34" t="n">
         <v>17.63</v>
       </c>
-      <c r="AK22" t="n">
+      <c r="AK34" t="n">
         <v>2.33</v>
       </c>
-      <c r="AL22" t="n">
+      <c r="AL34" t="n">
         <v>19.31</v>
       </c>
-      <c r="AM22" t="n">
+      <c r="AM34" t="n">
         <v>97.68000000000001</v>
       </c>
-      <c r="AN22" t="n">
+      <c r="AN34" t="n">
         <v>227.45</v>
       </c>
-      <c r="AO22" t="n">
+      <c r="AO34" t="n">
         <v>114.9</v>
       </c>
-      <c r="AP22" t="n">
+      <c r="AP34" t="n">
         <v>18.24</v>
       </c>
-      <c r="AQ22" t="n">
+      <c r="AQ34" t="n">
         <v>61.76</v>
       </c>
-      <c r="AR22" t="inlineStr">
+      <c r="AR34" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/moneyview-ltd</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-06)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR34"/>
+  <dimension ref="A1:AR32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kataline Limited</t>
+          <t>Pentacle Consultants I Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -719,43 +719,57 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NBFC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
+      </c>
+      <c r="J2" t="n">
+        <v>22.17</v>
       </c>
       <c r="N2" t="n">
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>220.58</v>
+        <v>91.73</v>
       </c>
       <c r="R2" t="n">
-        <v>38.79</v>
+        <v>52.3</v>
       </c>
       <c r="S2" t="n">
-        <v>26.83</v>
+        <v>28.86</v>
       </c>
       <c r="T2" t="n">
-        <v>61.15</v>
+        <v>174.54</v>
       </c>
       <c r="U2" t="n">
-        <v>12.16</v>
+        <v>31.46</v>
       </c>
       <c r="V2" t="n">
-        <v>16.44</v>
+        <v>36.04</v>
       </c>
       <c r="W2" t="n">
-        <v>26.27</v>
+        <v>49.11</v>
       </c>
       <c r="X2" t="n">
-        <v>34.86</v>
+        <v>33.57</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>70.79000000000001</v>
       </c>
       <c r="AA2" t="n">
-        <v>77.8</v>
+        <v>85.3</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -775,24 +789,24 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kataline-limited-drhp_104993.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pentacle-consultants-i-limited_105039.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/KATALINE%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Pentacle%20Consultants%20(I)%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J Infratech Limited</t>
+          <t>Kataline Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -807,54 +821,43 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
-      </c>
-      <c r="L3" t="n">
-        <v>10000000</v>
       </c>
       <c r="N3" t="n">
         <v>10</v>
       </c>
       <c r="Q3" t="n">
-        <v>1721.76</v>
+        <v>220.58</v>
       </c>
       <c r="R3" t="n">
-        <v>22.01</v>
+        <v>38.79</v>
       </c>
       <c r="S3" t="n">
-        <v>246.59</v>
+        <v>26.83</v>
       </c>
       <c r="T3" t="n">
-        <v>26.24</v>
+        <v>61.15</v>
       </c>
       <c r="U3" t="n">
-        <v>14.32</v>
+        <v>12.16</v>
       </c>
       <c r="V3" t="n">
-        <v>25.14</v>
+        <v>16.44</v>
       </c>
       <c r="W3" t="n">
-        <v>41.75</v>
+        <v>26.27</v>
       </c>
       <c r="X3" t="n">
-        <v>39.72</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>1.04</v>
+        <v>34.86</v>
       </c>
       <c r="AA3" t="n">
-        <v>74</v>
+        <v>77.8</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -874,19 +877,19 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/j-infratech-limited-drhp_104846.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kataline-limited-drhp_104993.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/J%20Infratech%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/KATALINE%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shreejikrupa Project Limited</t>
+          <t>Sanghvi Housing and Infrastructure Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -920,37 +923,34 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q4" t="n">
-        <v>1385.68</v>
+        <v>101.84</v>
       </c>
       <c r="R4" t="n">
-        <v>62.52</v>
+        <v>34.73</v>
       </c>
       <c r="S4" t="n">
-        <v>79.34</v>
+        <v>26.26</v>
       </c>
       <c r="T4" t="n">
-        <v>19.36</v>
+        <v>26.21</v>
       </c>
       <c r="U4" t="n">
-        <v>5.66</v>
+        <v>25.14</v>
       </c>
       <c r="V4" t="n">
-        <v>8.91</v>
+        <v>35.22</v>
       </c>
       <c r="W4" t="n">
-        <v>26.53</v>
+        <v>36.72</v>
       </c>
       <c r="X4" t="n">
-        <v>21.66</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>85.56</v>
+        <v>20.26</v>
       </c>
       <c r="AA4" t="n">
-        <v>65.09999999999999</v>
+        <v>77.3</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -970,24 +970,24 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/shreejikrupa-project-limited-drhp_104991.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sanghvi-housing-and-infrastructure-limited-drhp_105004.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/SHREEJIKRUPA%20PROJECT%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Sanghvi%20Housing_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ekkaa Electronics (India) Limited</t>
+          <t>PES Installations Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1002,12 +1002,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Hospitals</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1015,32 +1015,41 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>5794480</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2483360</v>
+      </c>
+      <c r="M5" t="n">
+        <v>8277840</v>
+      </c>
       <c r="N5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q5" t="n">
-        <v>1221.76</v>
+        <v>110.56</v>
       </c>
       <c r="R5" t="n">
-        <v>146.07</v>
+        <v>37.65</v>
       </c>
       <c r="S5" t="n">
-        <v>65.38</v>
+        <v>23.12</v>
       </c>
       <c r="T5" t="n">
-        <v>177.59</v>
+        <v>76.45999999999999</v>
       </c>
       <c r="U5" t="n">
-        <v>5.35</v>
+        <v>20.91</v>
       </c>
       <c r="V5" t="n">
-        <v>9.369999999999999</v>
+        <v>29.91</v>
       </c>
       <c r="W5" t="n">
-        <v>25.99</v>
+        <v>36.5</v>
       </c>
       <c r="AA5" t="n">
-        <v>59</v>
+        <v>70.3</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -1060,24 +1069,24 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/ekkaa-electronics-india-limited-drhp_104862.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pes-installations-limited-drhp_105018.html</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EKKAA%20ELECTRONICS%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PES%20Installations%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Biocon Electric Limited</t>
+          <t>Shreejikrupa Project Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1092,7 +1101,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1101,37 +1115,37 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q6" t="n">
-        <v>196.73</v>
+        <v>1385.68</v>
       </c>
       <c r="R6" t="n">
-        <v>37.94</v>
+        <v>62.52</v>
       </c>
       <c r="S6" t="n">
-        <v>14.14</v>
+        <v>79.34</v>
       </c>
       <c r="T6" t="n">
-        <v>22.96</v>
+        <v>19.36</v>
       </c>
       <c r="U6" t="n">
-        <v>7.14</v>
+        <v>5.66</v>
       </c>
       <c r="V6" t="n">
-        <v>12.94</v>
+        <v>8.91</v>
       </c>
       <c r="W6" t="n">
-        <v>24.05</v>
+        <v>26.53</v>
       </c>
       <c r="X6" t="n">
-        <v>12.19</v>
+        <v>21.66</v>
       </c>
       <c r="Z6" t="n">
-        <v>90</v>
+        <v>85.56</v>
       </c>
       <c r="AA6" t="n">
-        <v>58.1</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
@@ -1151,19 +1165,19 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/biocon-electric-limited-drhp_104995.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/shreejikrupa-project-limited-drhp_104991.html</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Biocon%20Electric%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/SHREEJIKRUPA%20PROJECT%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Anarock Property Consultants Limited</t>
+          <t>Baanganga Gold &amp; Diamond (I) Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1183,12 +1197,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1197,34 +1211,31 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q7" t="n">
-        <v>881.9</v>
+        <v>3626.29</v>
       </c>
       <c r="R7" t="n">
-        <v>33.83</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="S7" t="n">
-        <v>93.22</v>
+        <v>111.78</v>
       </c>
       <c r="T7" t="n">
-        <v>53.38</v>
+        <v>214.43</v>
       </c>
       <c r="U7" t="n">
-        <v>10.57</v>
+        <v>3.07</v>
       </c>
       <c r="V7" t="n">
-        <v>17.1</v>
+        <v>4.57</v>
       </c>
       <c r="W7" t="n">
-        <v>15.64</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>66.41</v>
+        <v>59.49</v>
       </c>
       <c r="AA7" t="n">
-        <v>57.6</v>
+        <v>64</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
@@ -1244,24 +1255,24 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/anarock-property-consultants-limited_105006.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/baanganga-gold-and-diamond-i-limited-drhp_105025.html</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Anarock%20Property%20Consultants%20Limited%20-%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Baanganga%20Gold%20&amp;%20Diamond%20(I)%20Limited-Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Royal Chain Limited</t>
+          <t>Tanvi Exports India Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1276,12 +1287,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Agri Exports</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1293,28 +1304,31 @@
         <v>10</v>
       </c>
       <c r="Q8" t="n">
-        <v>202.6</v>
+        <v>1139.94</v>
       </c>
       <c r="R8" t="n">
-        <v>0.05</v>
+        <v>13.04</v>
       </c>
       <c r="S8" t="n">
-        <v>173.34</v>
+        <v>65.8</v>
       </c>
       <c r="T8" t="n">
-        <v>173.71</v>
+        <v>255.97</v>
       </c>
       <c r="U8" t="n">
-        <v>85.56</v>
+        <v>5.76</v>
       </c>
       <c r="V8" t="n">
-        <v>142.27</v>
+        <v>8.08</v>
       </c>
       <c r="W8" t="n">
-        <v>53.34</v>
+        <v>60.71</v>
+      </c>
+      <c r="X8" t="n">
+        <v>38.61</v>
       </c>
       <c r="AA8" t="n">
-        <v>50.6</v>
+        <v>62.9</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
@@ -1334,24 +1348,24 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/royal-chain-limited-drhp_104015.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tanvi-exports-india-limited-drhp_105002.html</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Royal%20Chain%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tanvi%20Exports%20India%20Limited-%20%20draft%20abridged%20prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vardhman Appliances Limited</t>
+          <t>B S Sponge Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1366,12 +1380,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1379,35 +1393,41 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="J9" t="n">
+        <v>1000</v>
+      </c>
       <c r="N9" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q9" t="n">
-        <v>869.62</v>
+        <v>2592.52</v>
       </c>
       <c r="R9" t="n">
-        <v>4.03</v>
+        <v>18.5</v>
       </c>
       <c r="S9" t="n">
-        <v>22.48</v>
+        <v>171.11</v>
       </c>
       <c r="T9" t="n">
-        <v>21.42</v>
+        <v>8</v>
       </c>
       <c r="U9" t="n">
-        <v>2.59</v>
+        <v>6.57</v>
       </c>
       <c r="V9" t="n">
-        <v>5.98</v>
+        <v>14.83</v>
       </c>
       <c r="W9" t="n">
-        <v>25.27</v>
+        <v>24.18</v>
       </c>
       <c r="X9" t="n">
-        <v>24.01</v>
+        <v>22.9</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.97</v>
       </c>
       <c r="AA9" t="n">
-        <v>45.3</v>
+        <v>57.9</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1427,19 +1447,19 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vardhman-appliances-limited-drhp_104999.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/b-s-sponge-limited-drhp_105023.html</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Vardhman%20Appliances%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/B%20S%20Sponge%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Pci Infraprojects Limited</t>
+          <t>Anarock Property Consultants Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1459,12 +1479,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1473,34 +1493,34 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>304.09</v>
+        <v>881.9</v>
       </c>
       <c r="R10" t="n">
-        <v>7.68</v>
+        <v>33.83</v>
       </c>
       <c r="S10" t="n">
-        <v>23.85</v>
+        <v>93.22</v>
       </c>
       <c r="T10" t="n">
-        <v>-3.8</v>
+        <v>53.38</v>
       </c>
       <c r="U10" t="n">
-        <v>7.84</v>
+        <v>10.57</v>
       </c>
       <c r="V10" t="n">
-        <v>17.59</v>
+        <v>17.1</v>
       </c>
       <c r="W10" t="n">
-        <v>36.29</v>
-      </c>
-      <c r="X10" t="n">
-        <v>39.97</v>
+        <v>15.64</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>66.41</v>
       </c>
       <c r="AA10" t="n">
-        <v>43.9</v>
+        <v>57.6</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
@@ -1520,29 +1540,29 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/anarock-property-consultants-limited-drhp_104988.html</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Anarock%20Property%20Consultants%20Limited%20-%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AITMC Ventures Limited</t>
+          <t>Nnt Developers Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1557,35 +1577,41 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q11" t="n">
-        <v>106.76</v>
+        <v>223.66</v>
       </c>
       <c r="R11" t="n">
-        <v>22.05</v>
+        <v>7.97</v>
       </c>
       <c r="S11" t="n">
-        <v>13.38</v>
+        <v>21.57</v>
       </c>
       <c r="T11" t="n">
-        <v>-17.09</v>
+        <v>5.7</v>
       </c>
       <c r="U11" t="n">
-        <v>12.54</v>
+        <v>9.56</v>
       </c>
       <c r="V11" t="n">
-        <v>26.74</v>
+        <v>14.72</v>
       </c>
       <c r="W11" t="n">
-        <v>19.04</v>
+        <v>24.43</v>
+      </c>
+      <c r="X11" t="n">
+        <v>33.73</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.39</v>
       </c>
       <c r="AA11" t="n">
-        <v>39</v>
+        <v>47.3</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
@@ -1594,7 +1620,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -1605,24 +1631,24 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/aitmc-ventures-limited-udrhp-i_104864.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/AITMC%20Ventures%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jagatjit Agri Engineering Limited</t>
+          <t>Tenty Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1642,7 +1668,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1650,26 +1676,32 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="L12" t="n">
-        <v>3100000</v>
-      </c>
       <c r="N12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q12" t="n">
-        <v>413.97</v>
+        <v>822.25</v>
       </c>
       <c r="R12" t="n">
-        <v>331.55</v>
+        <v>97.91</v>
+      </c>
+      <c r="S12" t="n">
+        <v>22.65</v>
+      </c>
+      <c r="T12" t="n">
+        <v>232.88</v>
+      </c>
+      <c r="U12" t="n">
+        <v>2.67</v>
       </c>
       <c r="V12" t="n">
-        <v>13.46</v>
+        <v>9.66</v>
       </c>
       <c r="W12" t="n">
-        <v>53.89</v>
+        <v>6.76</v>
       </c>
       <c r="AA12" t="n">
-        <v>36.2</v>
+        <v>44.2</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -1689,24 +1721,24 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Koolking Industries India Limited</t>
+          <t>Pci Infraprojects Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1721,12 +1753,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Diversified Industrials</t>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1735,23 +1767,38 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q13" t="n">
-        <v>526.75</v>
+        <v>304.09</v>
       </c>
       <c r="R13" t="n">
-        <v>9.02</v>
+        <v>7.68</v>
+      </c>
+      <c r="S13" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="U13" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="V13" t="n">
+        <v>17.59</v>
       </c>
       <c r="W13" t="n">
-        <v>35.28</v>
+        <v>36.29</v>
+      </c>
+      <c r="X13" t="n">
+        <v>39.97</v>
       </c>
       <c r="AA13" t="n">
-        <v>22.6</v>
+        <v>43.9</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>MONITOR</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -1767,24 +1814,24 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/koolking-industries-india-limited-drhp_104848.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Koolking%20Industries%20India%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Arete 22 Limited</t>
+          <t>Jagatjit Agri Engineering Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1799,12 +1846,43 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>413.97</v>
+      </c>
+      <c r="R14" t="n">
+        <v>331.55</v>
+      </c>
+      <c r="V14" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="W14" t="n">
+        <v>53.89</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>36.2</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -1814,20 +1892,25 @@
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited_105016.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Deon Energy Limited</t>
+          <t>Electromech Infraprojects Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1847,17 +1930,47 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>270.65</v>
+      </c>
+      <c r="N15" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>427.05</v>
+      </c>
+      <c r="R15" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="S15" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="T15" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="U15" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="V15" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="W15" t="n">
+        <v>24.34</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>35.9</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -1867,20 +1980,25 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/deon-energy-limited_105012.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Rathod Jewellery Manufacturing Limited</t>
+          <t>Everbrands India Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1900,17 +2018,40 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Jewellery</t>
-        </is>
+          <t>Internet Platforms</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>693.09</v>
+      </c>
+      <c r="R16" t="n">
+        <v>9561.1</v>
+      </c>
+      <c r="V16" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="W16" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>28.2</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -1920,25 +2061,30 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rathod-jewellery-manufacturing-limited_105014.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Inox Clean Energy Limited</t>
+          <t>Pm Cona Industries Limited</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1953,12 +2099,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
@@ -1979,14 +2125,14 @@
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited_105010.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rudra Green Ship Recycling Limited</t>
+          <t>Inox Air Products Limited</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2006,8 +2152,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Medical Devices</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>77156663</v>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -2027,14 +2189,19 @@
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited_105008.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sanghvi Housing and Infrastructure Limited</t>
+          <t>Arete 22 Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2054,12 +2221,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
@@ -2080,19 +2242,14 @@
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sanghvi-housing-and-infrastructure-limited-drhp_105004.html</t>
-        </is>
-      </c>
-      <c r="AG19" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Sanghvi%20Housing_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited_105016.html</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tanvi Exports India Limited</t>
+          <t>Deon Energy Limited</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2112,12 +2269,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Agri Exports</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -2138,14 +2295,14 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tanvi-exports-india-limited_105002.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/deon-energy-limited_105012.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nnt Developers Limited</t>
+          <t>Rathod Jewellery Manufacturing Limited</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2165,7 +2322,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
@@ -2186,19 +2348,19 @@
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited_105000.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rathod-jewellery-manufacturing-limited_105014.html</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kian-M Export Limited</t>
+          <t>Inox Clean Energy Limited</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2213,12 +2375,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Agri Exports</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -2239,24 +2401,24 @@
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kian-m-export-limited_104874.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited_105010.html</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Arohan Financial Services Limited</t>
+          <t>Rudra Green Ship Recycling Limited</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2266,12 +2428,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>NBFC</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -2281,7 +2438,7 @@
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD23" t="inlineStr">
@@ -2292,14 +2449,14 @@
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited_105008.html</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sai Infinium Limited</t>
+          <t>Kian-M Export Limited</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2319,7 +2476,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Agri Exports</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -2340,14 +2502,14 @@
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sai-infinium-limited_104850.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kian-m-export-limited_104874.html</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sonaselection India Limited</t>
+          <t>Arohan Financial Services Limited</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2357,17 +2519,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>NBFC</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -2377,7 +2544,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
@@ -2388,36 +2555,14 @@
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sonaselection-india-limited-prospectus_104876.html</t>
-        </is>
-      </c>
-      <c r="AH25" t="inlineStr">
-        <is>
-          <t>Sonaselection India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI25" t="n">
-        <v>525</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>32.66</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>64.52</v>
-      </c>
-      <c r="AR25" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/sonaselection-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>Sonaselection India Limited</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2458,48 +2603,36 @@
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sonaselection-india-limited-prospectus_104876.html</t>
         </is>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Ltd.</t>
-        </is>
+          <t>Sonaselection India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI26" t="n">
+        <v>527</v>
       </c>
       <c r="AJ26" t="n">
-        <v>17.21</v>
+        <v>32.66</v>
       </c>
       <c r="AK26" t="n">
-        <v>1.91</v>
+        <v>2.48</v>
       </c>
       <c r="AL26" t="n">
-        <v>84.61</v>
-      </c>
-      <c r="AM26" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="AN26" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="AO26" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="AP26" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AQ26" t="n">
-        <v>0</v>
+        <v>64.52</v>
       </c>
       <c r="AR26" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
+          <t>https://groww.in/stocks/sonaselection-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SRIT India Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2540,36 +2673,51 @@
       <c r="AE27" t="inlineStr"/>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
         </is>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>SRIT India Ltd</t>
-        </is>
+          <t>Runwal Enterprises Ltd.</t>
+        </is>
+      </c>
+      <c r="AI27" t="n">
+        <v>4418</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>17.21</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>84.61</v>
       </c>
       <c r="AM27" t="n">
-        <v>121.24</v>
+        <v>2.45</v>
       </c>
       <c r="AN27" t="n">
-        <v>91.84</v>
+        <v>3.89</v>
       </c>
       <c r="AO27" t="n">
-        <v>310.94</v>
+        <v>3.91</v>
       </c>
       <c r="AP27" t="n">
-        <v>56.75</v>
+        <v>1.03</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>0</v>
       </c>
       <c r="AR27" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/srit-india-ipo</t>
+          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>A ONE Steels Limited</t>
+          <t>SRIT India Limited</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2589,12 +2737,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Metals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -2615,71 +2758,70 @@
       <c r="AE28" t="inlineStr"/>
       <c r="AF28" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
         </is>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>A-One Steels India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI28" t="n">
-        <v>3221</v>
+          <t>Srit India Ltd.</t>
+        </is>
       </c>
       <c r="AJ28" t="n">
-        <v>15.07</v>
+        <v>22.4</v>
       </c>
       <c r="AK28" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="AL28" t="n">
-        <v>74.51000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="AM28" t="n">
-        <v>11.35</v>
+        <v>121.24</v>
       </c>
       <c r="AN28" t="n">
-        <v>7.3</v>
+        <v>91.84</v>
       </c>
       <c r="AO28" t="n">
-        <v>24.38</v>
+        <v>310.94</v>
       </c>
       <c r="AP28" t="n">
-        <v>8.18</v>
+        <v>56.75</v>
       </c>
       <c r="AQ28" t="n">
-        <v>12.35</v>
+        <v>13.85</v>
       </c>
       <c r="AR28" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
+          <t>https://groww.in/stocks/srit-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>J B Ecotex Limited</t>
+          <t>A ONE Steels Limited</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Metals</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -2700,7 +2842,44 @@
       <c r="AE29" t="inlineStr"/>
       <c r="AF29" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/j-b-ecotex-limited_104830.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>A-One Steels India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>3003</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>15.07</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>74.51000000000001</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>11.35</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="AO29" t="n">
+        <v>24.38</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2941,7 @@
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>1057</v>
+        <v>1005</v>
       </c>
       <c r="AJ30" t="n">
         <v>20.31</v>
@@ -2836,6 +3015,9 @@
           <t>German Green Steel and Power Ltd.</t>
         </is>
       </c>
+      <c r="AI31" t="n">
+        <v>966</v>
+      </c>
       <c r="AJ31" t="n">
         <v>18.95</v>
       </c>
@@ -2948,158 +3130,6 @@
       <c r="AR32" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/rays-of-belief-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Acevector Limited</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB33" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC33" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE33" t="inlineStr"/>
-      <c r="AF33" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/acevector-limited-prospectus_104868.html</t>
-        </is>
-      </c>
-      <c r="AH33" t="inlineStr">
-        <is>
-          <t>AceVector Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ33" t="n">
-        <v>-59.54</v>
-      </c>
-      <c r="AK33" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AL33" t="n">
-        <v>49.96</v>
-      </c>
-      <c r="AR33" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/acevector-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Moneyview Limited</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB34" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC34" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE34" t="inlineStr"/>
-      <c r="AF34" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/moneyview-limited-prospectus_104787.html</t>
-        </is>
-      </c>
-      <c r="AH34" t="inlineStr">
-        <is>
-          <t>Moneyview Ltd.</t>
-        </is>
-      </c>
-      <c r="AI34" t="n">
-        <v>9511</v>
-      </c>
-      <c r="AJ34" t="n">
-        <v>17.63</v>
-      </c>
-      <c r="AK34" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="AL34" t="n">
-        <v>19.31</v>
-      </c>
-      <c r="AM34" t="n">
-        <v>97.68000000000001</v>
-      </c>
-      <c r="AN34" t="n">
-        <v>227.45</v>
-      </c>
-      <c r="AO34" t="n">
-        <v>114.9</v>
-      </c>
-      <c r="AP34" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="AQ34" t="n">
-        <v>61.76</v>
-      </c>
-      <c r="AR34" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/moneyview-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-07)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR32"/>
+  <dimension ref="A1:AR31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1552,7 +1552,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nnt Developers Limited</t>
+          <t>Inox Clean Energy Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1572,46 +1572,45 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Power</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>223.66</v>
+        <v>178.13</v>
       </c>
       <c r="R11" t="n">
-        <v>7.97</v>
+        <v>20.8</v>
       </c>
       <c r="S11" t="n">
-        <v>21.57</v>
+        <v>30.98</v>
       </c>
       <c r="T11" t="n">
-        <v>5.7</v>
+        <v>1891.07</v>
       </c>
       <c r="U11" t="n">
-        <v>9.56</v>
+        <v>17.39</v>
       </c>
       <c r="V11" t="n">
-        <v>14.72</v>
+        <v>18.11</v>
       </c>
       <c r="W11" t="n">
-        <v>24.43</v>
-      </c>
-      <c r="X11" t="n">
-        <v>33.73</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>0.39</v>
+        <v>1.33</v>
       </c>
       <c r="AA11" t="n">
-        <v>47.3</v>
+        <v>47.6</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
@@ -1631,19 +1630,19 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited-drhp_105010.html</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Clean%20Energy%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tenty Limited</t>
+          <t>Nnt Developers Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1663,45 +1662,46 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Manufacturing</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="N12" t="n">
         <v>10</v>
       </c>
       <c r="Q12" t="n">
-        <v>822.25</v>
+        <v>223.66</v>
       </c>
       <c r="R12" t="n">
-        <v>97.91</v>
+        <v>7.97</v>
       </c>
       <c r="S12" t="n">
-        <v>22.65</v>
+        <v>21.57</v>
       </c>
       <c r="T12" t="n">
-        <v>232.88</v>
+        <v>5.7</v>
       </c>
       <c r="U12" t="n">
-        <v>2.67</v>
+        <v>9.56</v>
       </c>
       <c r="V12" t="n">
-        <v>9.66</v>
+        <v>14.72</v>
       </c>
       <c r="W12" t="n">
-        <v>6.76</v>
+        <v>24.43</v>
+      </c>
+      <c r="X12" t="n">
+        <v>33.73</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.39</v>
       </c>
       <c r="AA12" t="n">
-        <v>44.2</v>
+        <v>47.3</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -1721,19 +1721,19 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pci Infraprojects Limited</t>
+          <t>Tenty Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1753,12 +1753,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1770,31 +1770,28 @@
         <v>10</v>
       </c>
       <c r="Q13" t="n">
-        <v>304.09</v>
+        <v>822.25</v>
       </c>
       <c r="R13" t="n">
-        <v>7.68</v>
+        <v>97.91</v>
       </c>
       <c r="S13" t="n">
-        <v>23.85</v>
+        <v>22.65</v>
       </c>
       <c r="T13" t="n">
-        <v>-3.8</v>
+        <v>232.88</v>
       </c>
       <c r="U13" t="n">
-        <v>7.84</v>
+        <v>2.67</v>
       </c>
       <c r="V13" t="n">
-        <v>17.59</v>
+        <v>9.66</v>
       </c>
       <c r="W13" t="n">
-        <v>36.29</v>
-      </c>
-      <c r="X13" t="n">
-        <v>39.97</v>
+        <v>6.76</v>
       </c>
       <c r="AA13" t="n">
-        <v>43.9</v>
+        <v>44.2</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
@@ -1814,24 +1811,24 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jagatjit Agri Engineering Limited</t>
+          <t>Pci Infraprojects Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1846,12 +1843,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1859,26 +1856,35 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="L14" t="n">
-        <v>3100000</v>
-      </c>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q14" t="n">
-        <v>413.97</v>
+        <v>304.09</v>
       </c>
       <c r="R14" t="n">
-        <v>331.55</v>
+        <v>7.68</v>
+      </c>
+      <c r="S14" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="U14" t="n">
+        <v>7.84</v>
       </c>
       <c r="V14" t="n">
-        <v>13.46</v>
+        <v>17.59</v>
       </c>
       <c r="W14" t="n">
-        <v>53.89</v>
+        <v>36.29</v>
+      </c>
+      <c r="X14" t="n">
+        <v>39.97</v>
       </c>
       <c r="AA14" t="n">
-        <v>36.2</v>
+        <v>43.9</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
@@ -1898,24 +1904,24 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Electromech Infraprojects Limited</t>
+          <t>Jagatjit Agri Engineering Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1930,7 +1936,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1938,35 +1949,26 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>270.65</v>
+      <c r="L15" t="n">
+        <v>3100000</v>
       </c>
       <c r="N15" t="n">
         <v>5</v>
       </c>
       <c r="Q15" t="n">
-        <v>427.05</v>
+        <v>413.97</v>
       </c>
       <c r="R15" t="n">
-        <v>4.54</v>
-      </c>
-      <c r="S15" t="n">
-        <v>36.19</v>
-      </c>
-      <c r="T15" t="n">
-        <v>22.75</v>
-      </c>
-      <c r="U15" t="n">
-        <v>8.41</v>
+        <v>331.55</v>
       </c>
       <c r="V15" t="n">
-        <v>10.8</v>
+        <v>13.46</v>
       </c>
       <c r="W15" t="n">
-        <v>24.34</v>
+        <v>53.89</v>
       </c>
       <c r="AA15" t="n">
-        <v>35.9</v>
+        <v>36.2</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
@@ -1986,19 +1988,19 @@
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Everbrands India Limited</t>
+          <t>Electromech Infraprojects Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2018,36 +2020,43 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Internet Platforms</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Fresh</t>
-        </is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>270.65</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q16" t="n">
-        <v>693.09</v>
+        <v>427.05</v>
       </c>
       <c r="R16" t="n">
-        <v>9561.1</v>
+        <v>4.54</v>
+      </c>
+      <c r="S16" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="T16" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="U16" t="n">
+        <v>8.41</v>
       </c>
       <c r="V16" t="n">
-        <v>10.16</v>
+        <v>10.8</v>
       </c>
       <c r="W16" t="n">
-        <v>10.16</v>
+        <v>24.34</v>
       </c>
       <c r="AA16" t="n">
-        <v>28.2</v>
+        <v>35.9</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
@@ -2067,24 +2076,24 @@
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pm Cona Industries Limited</t>
+          <t>Everbrands India Limited</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2099,17 +2108,40 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Diversified Industrials</t>
-        </is>
+          <t>Internet Platforms</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>693.09</v>
+      </c>
+      <c r="R17" t="n">
+        <v>9561.1</v>
+      </c>
+      <c r="V17" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="W17" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>28.2</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2119,57 +2151,51 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Inox Air Products Limited</t>
+          <t>Nityas Gems and Jewellery Limited</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Medical Devices</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L18" t="n">
-        <v>77156663</v>
-      </c>
-      <c r="N18" t="n">
-        <v>1</v>
+          <t>Jewellery</t>
+        </is>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -2189,24 +2215,41 @@
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
-        </is>
-      </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>Nityas Gems &amp; Jewellery Ltd</t>
+        </is>
+      </c>
+      <c r="AM18" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/nityas-gems-jewellery-ipo</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Arete 22 Limited</t>
+          <t>Pm Cona Industries Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2221,7 +2264,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
@@ -2242,39 +2290,34 @@
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited_105016.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deon Energy Limited</t>
+          <t>Vishal Nirmiti Limited</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Power</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -2295,14 +2338,36 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/deon-energy-limited_105012.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>Vishal Nirmiti Ltd</t>
+        </is>
+      </c>
+      <c r="AM20" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/vishal-nirmiti-ipo</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rathod Jewellery Manufacturing Limited</t>
+          <t>Inox Air Products Limited</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2322,13 +2387,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Jewellery</t>
-        </is>
+          <t>Medical Devices</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>77156663</v>
+      </c>
+      <c r="N21" t="n">
+        <v>1</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
@@ -2348,14 +2424,19 @@
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rathod-jewellery-manufacturing-limited_105014.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Inox Clean Energy Limited</t>
+          <t>Arete 22 Limited</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2375,12 +2456,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Power</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -2401,14 +2477,14 @@
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited_105010.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited_105016.html</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rudra Green Ship Recycling Limited</t>
+          <t>Deon Energy Limited</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2428,7 +2504,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Power</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -2449,19 +2530,19 @@
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited_105008.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/deon-energy-limited_105012.html</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Kian-M Export Limited</t>
+          <t>Rathod Jewellery Manufacturing Limited</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2476,12 +2557,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Agri Exports</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -2502,24 +2583,24 @@
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kian-m-export-limited_104874.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rathod-jewellery-manufacturing-limited_105014.html</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Arohan Financial Services Limited</t>
+          <t>Rudra Green Ship Recycling Limited</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2529,12 +2610,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>NBFC</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -2544,7 +2620,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
@@ -2555,14 +2631,14 @@
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited_105008.html</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sonaselection India Limited</t>
+          <t>Kian-M Export Limited</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2572,17 +2648,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Agri Exports</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -2603,36 +2684,14 @@
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sonaselection-india-limited-prospectus_104876.html</t>
-        </is>
-      </c>
-      <c r="AH26" t="inlineStr">
-        <is>
-          <t>Sonaselection India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI26" t="n">
-        <v>527</v>
-      </c>
-      <c r="AJ26" t="n">
-        <v>32.66</v>
-      </c>
-      <c r="AK26" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="AL26" t="n">
-        <v>64.52</v>
-      </c>
-      <c r="AR26" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/sonaselection-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kian-m-export-limited_104874.html</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>Arohan Financial Services Limited</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2642,17 +2701,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>NBFC</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -2662,7 +2726,7 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
@@ -2673,51 +2737,14 @@
       <c r="AE27" t="inlineStr"/>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
-        </is>
-      </c>
-      <c r="AH27" t="inlineStr">
-        <is>
-          <t>Runwal Enterprises Ltd.</t>
-        </is>
-      </c>
-      <c r="AI27" t="n">
-        <v>4418</v>
-      </c>
-      <c r="AJ27" t="n">
-        <v>17.21</v>
-      </c>
-      <c r="AK27" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="AL27" t="n">
-        <v>84.61</v>
-      </c>
-      <c r="AM27" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="AN27" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="AO27" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="AP27" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AQ27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR27" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SRIT India Limited</t>
+          <t>Sonaselection India Limited</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2758,45 +2785,36 @@
       <c r="AE28" t="inlineStr"/>
       <c r="AF28" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sonaselection-india-limited-prospectus_104876.html</t>
         </is>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>Srit India Ltd.</t>
-        </is>
+          <t>Sonaselection India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>540</v>
       </c>
       <c r="AJ28" t="n">
-        <v>22.4</v>
+        <v>32.66</v>
       </c>
       <c r="AK28" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="AM28" t="n">
-        <v>121.24</v>
-      </c>
-      <c r="AN28" t="n">
-        <v>91.84</v>
-      </c>
-      <c r="AO28" t="n">
-        <v>310.94</v>
-      </c>
-      <c r="AP28" t="n">
-        <v>56.75</v>
-      </c>
-      <c r="AQ28" t="n">
-        <v>13.85</v>
+        <v>2.48</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>64.52</v>
       </c>
       <c r="AR28" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/srit-india-ltd</t>
+          <t>https://groww.in/stocks/sonaselection-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>A ONE Steels Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2816,12 +2834,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Metals</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -2842,56 +2855,56 @@
       <c r="AE29" t="inlineStr"/>
       <c r="AF29" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
         </is>
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>A-One Steels India Ltd.</t>
+          <t>Runwal Enterprises Ltd.</t>
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>3003</v>
+        <v>4292</v>
       </c>
       <c r="AJ29" t="n">
-        <v>15.07</v>
+        <v>22.29</v>
       </c>
       <c r="AK29" t="n">
-        <v>1.25</v>
+        <v>3.52</v>
       </c>
       <c r="AL29" t="n">
-        <v>74.51000000000001</v>
+        <v>84.61</v>
       </c>
       <c r="AM29" t="n">
-        <v>11.35</v>
+        <v>2.45</v>
       </c>
       <c r="AN29" t="n">
-        <v>7.3</v>
+        <v>3.89</v>
       </c>
       <c r="AO29" t="n">
-        <v>24.38</v>
+        <v>3.91</v>
       </c>
       <c r="AP29" t="n">
-        <v>8.18</v>
+        <v>1.03</v>
       </c>
       <c r="AQ29" t="n">
-        <v>12.35</v>
+        <v>0</v>
       </c>
       <c r="AR29" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
+          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Adroit Industries (India) Limited</t>
+          <t>SRIT India Limited</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2906,12 +2919,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Diversified Industrials</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -2932,41 +2940,56 @@
       <c r="AE30" t="inlineStr"/>
       <c r="AF30" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/adroit-industries-india-limited-prospectus_104835.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
         </is>
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>Adroit Industries (India) Ltd</t>
+          <t>Srit India Ltd.</t>
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>1005</v>
+        <v>997</v>
       </c>
       <c r="AJ30" t="n">
-        <v>20.31</v>
+        <v>22.4</v>
       </c>
       <c r="AK30" t="n">
-        <v>0.41</v>
+        <v>0.23</v>
       </c>
       <c r="AL30" t="n">
-        <v>71.86</v>
+        <v>62.71</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>121.24</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>91.84</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>310.94</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>56.75</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>13.85</v>
       </c>
       <c r="AR30" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/adroit-industries-india-ltd</t>
+          <t>https://groww.in/stocks/srit-india-ltd</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>German Green Steel and Power Limited</t>
+          <t>A ONE Steels Limited</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3007,129 +3030,44 @@
       <c r="AE31" t="inlineStr"/>
       <c r="AF31" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/german-green-steel-and-power-limited-prospectus_104824.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
         </is>
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>German Green Steel and Power Ltd.</t>
+          <t>A-One Steels India Ltd.</t>
         </is>
       </c>
       <c r="AI31" t="n">
-        <v>966</v>
+        <v>2975</v>
       </c>
       <c r="AJ31" t="n">
-        <v>18.95</v>
+        <v>15.07</v>
       </c>
       <c r="AK31" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="AL31" t="n">
-        <v>68.54000000000001</v>
+        <v>74.51000000000001</v>
       </c>
       <c r="AM31" t="n">
-        <v>28.46</v>
+        <v>11.35</v>
       </c>
       <c r="AN31" t="n">
-        <v>20.93</v>
+        <v>7.3</v>
       </c>
       <c r="AO31" t="n">
-        <v>53.91</v>
+        <v>24.38</v>
       </c>
       <c r="AP31" t="n">
-        <v>21.85</v>
+        <v>8.18</v>
       </c>
       <c r="AQ31" t="n">
-        <v>2.16</v>
+        <v>12.35</v>
       </c>
       <c r="AR31" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/german-green-steel-and-power-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Rays of Belief Limited</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB32" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC32" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE32" t="inlineStr"/>
-      <c r="AF32" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/rays-of-belief-limited-prospectus_104816.html</t>
-        </is>
-      </c>
-      <c r="AH32" t="inlineStr">
-        <is>
-          <t>Rays Of Belief Ltd.</t>
-        </is>
-      </c>
-      <c r="AI32" t="n">
-        <v>474</v>
-      </c>
-      <c r="AJ32" t="n">
-        <v>16.24</v>
-      </c>
-      <c r="AK32" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AL32" t="n">
-        <v>68.77</v>
-      </c>
-      <c r="AM32" t="n">
-        <v>106.83</v>
-      </c>
-      <c r="AN32" t="n">
-        <v>9.06</v>
-      </c>
-      <c r="AO32" t="n">
-        <v>278.82</v>
-      </c>
-      <c r="AP32" t="n">
-        <v>190.99</v>
-      </c>
-      <c r="AQ32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR32" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/rays-of-belief-ltd</t>
+          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-08)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR31"/>
+  <dimension ref="A1:AR26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -982,12 +982,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PES Installations Limited</t>
+          <t>Grace Renewable Energy Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1002,54 +1002,48 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Hospitals</t>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
-      </c>
-      <c r="K5" t="n">
-        <v>5794480</v>
-      </c>
-      <c r="L5" t="n">
-        <v>2483360</v>
-      </c>
-      <c r="M5" t="n">
-        <v>8277840</v>
       </c>
       <c r="N5" t="n">
         <v>10</v>
       </c>
       <c r="Q5" t="n">
-        <v>110.56</v>
+        <v>205.84</v>
       </c>
       <c r="R5" t="n">
-        <v>37.65</v>
+        <v>70.83</v>
       </c>
       <c r="S5" t="n">
-        <v>23.12</v>
+        <v>18.67</v>
       </c>
       <c r="T5" t="n">
-        <v>76.45999999999999</v>
+        <v>91.06</v>
       </c>
       <c r="U5" t="n">
-        <v>20.91</v>
+        <v>9.07</v>
       </c>
       <c r="V5" t="n">
-        <v>29.91</v>
+        <v>12.53</v>
       </c>
       <c r="W5" t="n">
-        <v>36.5</v>
+        <v>65.73</v>
+      </c>
+      <c r="X5" t="n">
+        <v>80.45</v>
       </c>
       <c r="AA5" t="n">
-        <v>70.3</v>
+        <v>74.7</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -1069,19 +1063,19 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pes-installations-limited-drhp_105018.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/grace-renewable-energy-limited-drhp_105099.html</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PES%20Installations%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Grace%20Renewable%20Energy%20Limited%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shreejikrupa Project Limited</t>
+          <t>Rathod Jewellery Manufacturing Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1101,51 +1095,54 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>10360000</v>
+      </c>
+      <c r="M6" t="n">
+        <v>10360000</v>
       </c>
       <c r="N6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q6" t="n">
-        <v>1385.68</v>
+        <v>667.33</v>
       </c>
       <c r="R6" t="n">
-        <v>62.52</v>
+        <v>31.39</v>
       </c>
       <c r="S6" t="n">
-        <v>79.34</v>
+        <v>50.47</v>
       </c>
       <c r="T6" t="n">
-        <v>19.36</v>
+        <v>48.55</v>
       </c>
       <c r="U6" t="n">
-        <v>5.66</v>
+        <v>7.56</v>
       </c>
       <c r="V6" t="n">
-        <v>8.91</v>
+        <v>10.76</v>
       </c>
       <c r="W6" t="n">
-        <v>26.53</v>
+        <v>38.07</v>
       </c>
       <c r="X6" t="n">
-        <v>21.66</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>85.56</v>
+        <v>29.32</v>
       </c>
       <c r="AA6" t="n">
-        <v>65.09999999999999</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
@@ -1165,19 +1162,19 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/shreejikrupa-project-limited-drhp_104991.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rathod-jewellery-manufacturing-limited-drhp_105014.html</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/SHREEJIKRUPA%20PROJECT%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Rathod%20Jewellery%20Manufacturing%20Limited%20dap_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baanganga Gold &amp; Diamond (I) Limited</t>
+          <t>PES Installations Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1197,12 +1194,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Hospitals</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1210,32 +1207,41 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="K7" t="n">
+        <v>5794480</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2483360</v>
+      </c>
+      <c r="M7" t="n">
+        <v>8277840</v>
+      </c>
       <c r="N7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q7" t="n">
-        <v>3626.29</v>
+        <v>110.56</v>
       </c>
       <c r="R7" t="n">
-        <v>78.90000000000001</v>
+        <v>37.65</v>
       </c>
       <c r="S7" t="n">
-        <v>111.78</v>
+        <v>23.12</v>
       </c>
       <c r="T7" t="n">
-        <v>214.43</v>
+        <v>76.45999999999999</v>
       </c>
       <c r="U7" t="n">
-        <v>3.07</v>
+        <v>20.91</v>
       </c>
       <c r="V7" t="n">
-        <v>4.57</v>
+        <v>29.91</v>
       </c>
       <c r="W7" t="n">
-        <v>59.49</v>
+        <v>36.5</v>
       </c>
       <c r="AA7" t="n">
-        <v>64</v>
+        <v>70.3</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
@@ -1255,19 +1261,19 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/baanganga-gold-and-diamond-i-limited-drhp_105025.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pes-installations-limited-drhp_105018.html</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Baanganga%20Gold%20&amp;%20Diamond%20(I)%20Limited-Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PES%20Installations%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tanvi Exports India Limited</t>
+          <t>Shreejikrupa Project Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1287,12 +1293,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Agri Exports</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1301,34 +1307,37 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q8" t="n">
-        <v>1139.94</v>
+        <v>1385.68</v>
       </c>
       <c r="R8" t="n">
-        <v>13.04</v>
+        <v>62.52</v>
       </c>
       <c r="S8" t="n">
-        <v>65.8</v>
+        <v>79.34</v>
       </c>
       <c r="T8" t="n">
-        <v>255.97</v>
+        <v>19.36</v>
       </c>
       <c r="U8" t="n">
-        <v>5.76</v>
+        <v>5.66</v>
       </c>
       <c r="V8" t="n">
-        <v>8.08</v>
+        <v>8.91</v>
       </c>
       <c r="W8" t="n">
-        <v>60.71</v>
+        <v>26.53</v>
       </c>
       <c r="X8" t="n">
-        <v>38.61</v>
+        <v>21.66</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>85.56</v>
       </c>
       <c r="AA8" t="n">
-        <v>62.9</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
@@ -1348,19 +1357,19 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tanvi-exports-india-limited-drhp_105002.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/shreejikrupa-project-limited-drhp_104991.html</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tanvi%20Exports%20India%20Limited-%20%20draft%20abridged%20prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/SHREEJIKRUPA%20PROJECT%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B S Sponge Limited</t>
+          <t>Baanganga Gold &amp; Diamond (I) Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1380,12 +1389,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1393,41 +1402,32 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>1000</v>
-      </c>
       <c r="N9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q9" t="n">
-        <v>2592.52</v>
+        <v>3626.29</v>
       </c>
       <c r="R9" t="n">
-        <v>18.5</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="S9" t="n">
-        <v>171.11</v>
+        <v>111.78</v>
       </c>
       <c r="T9" t="n">
-        <v>8</v>
+        <v>214.43</v>
       </c>
       <c r="U9" t="n">
-        <v>6.57</v>
+        <v>3.07</v>
       </c>
       <c r="V9" t="n">
-        <v>14.83</v>
+        <v>4.57</v>
       </c>
       <c r="W9" t="n">
-        <v>24.18</v>
-      </c>
-      <c r="X9" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>0.97</v>
+        <v>59.49</v>
       </c>
       <c r="AA9" t="n">
-        <v>57.9</v>
+        <v>64</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1447,19 +1447,19 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/b-s-sponge-limited-drhp_105023.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/baanganga-gold-and-diamond-i-limited-drhp_105025.html</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/B%20S%20Sponge%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Baanganga%20Gold%20&amp;%20Diamond%20(I)%20Limited-Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Anarock Property Consultants Limited</t>
+          <t>Tanvi Exports India Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1479,12 +1479,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Agri Exports</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1493,34 +1493,34 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q10" t="n">
-        <v>881.9</v>
+        <v>1139.94</v>
       </c>
       <c r="R10" t="n">
-        <v>33.83</v>
+        <v>13.04</v>
       </c>
       <c r="S10" t="n">
-        <v>93.22</v>
+        <v>65.8</v>
       </c>
       <c r="T10" t="n">
-        <v>53.38</v>
+        <v>255.97</v>
       </c>
       <c r="U10" t="n">
-        <v>10.57</v>
+        <v>5.76</v>
       </c>
       <c r="V10" t="n">
-        <v>17.1</v>
+        <v>8.08</v>
       </c>
       <c r="W10" t="n">
-        <v>15.64</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>66.41</v>
+        <v>60.71</v>
+      </c>
+      <c r="X10" t="n">
+        <v>38.61</v>
       </c>
       <c r="AA10" t="n">
-        <v>57.6</v>
+        <v>62.9</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
@@ -1540,19 +1540,19 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/anarock-property-consultants-limited-drhp_104988.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tanvi-exports-india-limited-drhp_105002.html</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Anarock%20Property%20Consultants%20Limited%20-%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tanvi%20Exports%20India%20Limited-%20%20draft%20abridged%20prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Inox Clean Energy Limited</t>
+          <t>Deon Energy Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1586,31 +1586,34 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q11" t="n">
-        <v>178.13</v>
+        <v>456.28</v>
       </c>
       <c r="R11" t="n">
-        <v>20.8</v>
+        <v>52.84</v>
       </c>
       <c r="S11" t="n">
-        <v>30.98</v>
+        <v>46.06</v>
       </c>
       <c r="T11" t="n">
-        <v>1891.07</v>
+        <v>74.39</v>
       </c>
       <c r="U11" t="n">
-        <v>17.39</v>
+        <v>10.1</v>
       </c>
       <c r="V11" t="n">
-        <v>18.11</v>
+        <v>13.9</v>
       </c>
       <c r="W11" t="n">
-        <v>1.33</v>
+        <v>94.95</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.16</v>
       </c>
       <c r="AA11" t="n">
-        <v>47.6</v>
+        <v>61.5</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
@@ -1630,24 +1633,24 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited-drhp_105010.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/deon-energy-limited-drhp_105012.html</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Clean%20Energy%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Deon%20Energy%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nnt Developers Limited</t>
+          <t>Integrum Energy Infrastructure Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1662,46 +1665,48 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Power</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q12" t="n">
-        <v>223.66</v>
+        <v>693.84</v>
       </c>
       <c r="R12" t="n">
-        <v>7.97</v>
+        <v>489.67</v>
       </c>
       <c r="S12" t="n">
-        <v>21.57</v>
+        <v>63.16</v>
       </c>
       <c r="T12" t="n">
-        <v>5.7</v>
+        <v>400.13</v>
       </c>
       <c r="U12" t="n">
-        <v>9.56</v>
+        <v>9.1</v>
       </c>
       <c r="V12" t="n">
-        <v>14.72</v>
+        <v>12.72</v>
       </c>
       <c r="W12" t="n">
-        <v>24.43</v>
-      </c>
-      <c r="X12" t="n">
-        <v>33.73</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>0.39</v>
+        <v>42.2</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>90.66</v>
       </c>
       <c r="AA12" t="n">
-        <v>47.3</v>
+        <v>61.2</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -1721,19 +1726,19 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integrum-energy-infrastructure-limited-drhp_105075.html</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/INTEGRUM%20ENERGY%20INFRASTRUCTURE%20LIMITED-Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tenty Limited</t>
+          <t>Arete 22 Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1770,28 +1775,25 @@
         <v>10</v>
       </c>
       <c r="Q13" t="n">
-        <v>822.25</v>
+        <v>537.95</v>
       </c>
       <c r="R13" t="n">
-        <v>97.91</v>
+        <v>153.28</v>
       </c>
       <c r="S13" t="n">
-        <v>22.65</v>
+        <v>44.97</v>
       </c>
       <c r="T13" t="n">
-        <v>232.88</v>
+        <v>263.98</v>
       </c>
       <c r="U13" t="n">
-        <v>2.67</v>
-      </c>
-      <c r="V13" t="n">
-        <v>9.66</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="W13" t="n">
-        <v>6.76</v>
+        <v>75.22</v>
       </c>
       <c r="AA13" t="n">
-        <v>44.2</v>
+        <v>60</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
@@ -1811,19 +1813,19 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited-drhp_105016.html</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Arete%2022%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pci Infraprojects Limited</t>
+          <t>B S Sponge Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1843,48 +1845,54 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
+      </c>
+      <c r="J14" t="n">
+        <v>1000</v>
       </c>
       <c r="N14" t="n">
         <v>10</v>
       </c>
       <c r="Q14" t="n">
-        <v>304.09</v>
+        <v>2592.52</v>
       </c>
       <c r="R14" t="n">
-        <v>7.68</v>
+        <v>18.5</v>
       </c>
       <c r="S14" t="n">
-        <v>23.85</v>
+        <v>171.11</v>
       </c>
       <c r="T14" t="n">
-        <v>-3.8</v>
+        <v>8</v>
       </c>
       <c r="U14" t="n">
-        <v>7.84</v>
+        <v>6.57</v>
       </c>
       <c r="V14" t="n">
-        <v>17.59</v>
+        <v>14.83</v>
       </c>
       <c r="W14" t="n">
-        <v>36.29</v>
+        <v>24.18</v>
       </c>
       <c r="X14" t="n">
-        <v>39.97</v>
+        <v>22.9</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0.97</v>
       </c>
       <c r="AA14" t="n">
-        <v>43.9</v>
+        <v>57.9</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
@@ -1904,24 +1912,24 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/b-s-sponge-limited-drhp_105023.html</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/B%20S%20Sponge%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jagatjit Agri Engineering Limited</t>
+          <t>Anarock Property Consultants Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1936,12 +1944,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1949,26 +1957,35 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="L15" t="n">
-        <v>3100000</v>
-      </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>413.97</v>
+        <v>881.9</v>
       </c>
       <c r="R15" t="n">
-        <v>331.55</v>
+        <v>33.83</v>
+      </c>
+      <c r="S15" t="n">
+        <v>93.22</v>
+      </c>
+      <c r="T15" t="n">
+        <v>53.38</v>
+      </c>
+      <c r="U15" t="n">
+        <v>10.57</v>
       </c>
       <c r="V15" t="n">
-        <v>13.46</v>
+        <v>17.1</v>
       </c>
       <c r="W15" t="n">
-        <v>53.89</v>
+        <v>15.64</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>66.41</v>
       </c>
       <c r="AA15" t="n">
-        <v>36.2</v>
+        <v>57.6</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
@@ -1988,19 +2005,19 @@
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jagatjit-agri-engineering-limited-drhp_104866.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/anarock-property-consultants-limited-drhp_104988.html</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/DAP%20Jagatjit%20Agri%20Engineering%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Anarock%20Property%20Consultants%20Limited%20-%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Electromech Infraprojects Limited</t>
+          <t>Rudra Green Ship Recycling Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2027,36 +2044,39 @@
         <is>
           <t>Both</t>
         </is>
-      </c>
-      <c r="J16" t="n">
-        <v>270.65</v>
       </c>
       <c r="N16" t="n">
         <v>5</v>
       </c>
       <c r="Q16" t="n">
-        <v>427.05</v>
+        <v>204.52</v>
       </c>
       <c r="R16" t="n">
-        <v>4.54</v>
+        <v>14.13</v>
       </c>
       <c r="S16" t="n">
-        <v>36.19</v>
+        <v>12.65</v>
       </c>
       <c r="T16" t="n">
-        <v>22.75</v>
+        <v>28.83</v>
       </c>
       <c r="U16" t="n">
-        <v>8.41</v>
+        <v>6.17</v>
       </c>
       <c r="V16" t="n">
-        <v>10.8</v>
+        <v>10.65</v>
       </c>
       <c r="W16" t="n">
-        <v>24.34</v>
+        <v>27.4</v>
+      </c>
+      <c r="X16" t="n">
+        <v>19.03</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>98.86</v>
       </c>
       <c r="AA16" t="n">
-        <v>35.9</v>
+        <v>53.4</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
@@ -2076,19 +2096,19 @@
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited-drhp_105008.html</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Rudra%20Green%20Ship%20Recycling%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Everbrands India Limited</t>
+          <t>Inox Clean Energy Limited</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2108,36 +2128,45 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Internet Platforms</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="N17" t="n">
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>693.09</v>
+        <v>178.13</v>
       </c>
       <c r="R17" t="n">
-        <v>9561.1</v>
+        <v>20.8</v>
+      </c>
+      <c r="S17" t="n">
+        <v>30.98</v>
+      </c>
+      <c r="T17" t="n">
+        <v>1891.07</v>
+      </c>
+      <c r="U17" t="n">
+        <v>17.39</v>
       </c>
       <c r="V17" t="n">
-        <v>10.16</v>
+        <v>18.11</v>
       </c>
       <c r="W17" t="n">
-        <v>10.16</v>
+        <v>1.33</v>
       </c>
       <c r="AA17" t="n">
-        <v>28.2</v>
+        <v>47.6</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
@@ -2157,49 +2186,81 @@
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited-drhp_105010.html</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Clean%20Energy%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nityas Gems and Jewellery Limited</t>
+          <t>Tenty Limited</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Jewellery</t>
-        </is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>822.25</v>
+      </c>
+      <c r="R18" t="n">
+        <v>97.91</v>
+      </c>
+      <c r="S18" t="n">
+        <v>22.65</v>
+      </c>
+      <c r="T18" t="n">
+        <v>232.88</v>
+      </c>
+      <c r="U18" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="V18" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="W18" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>44.2</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2209,47 +2270,30 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
-        </is>
-      </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>Nityas Gems &amp; Jewellery Ltd</t>
-        </is>
-      </c>
-      <c r="AM18" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AO18" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AP18" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="AR18" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/nityas-gems-jewellery-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pm Cona Industries Limited</t>
+          <t>Pci Infraprojects Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2264,17 +2308,52 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Diversified Industrials</t>
-        </is>
+          <t>Renewables</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>304.09</v>
+      </c>
+      <c r="R19" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="S19" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="T19" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="U19" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="V19" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="W19" t="n">
+        <v>36.29</v>
+      </c>
+      <c r="X19" t="n">
+        <v>39.97</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>43.9</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2284,35 +2363,40 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Vishal Nirmiti Limited</t>
+          <t>Electromech Infraprojects Limited</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2320,9 +2404,44 @@
           <t>Unclassified</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>270.65</v>
+      </c>
+      <c r="N20" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>427.05</v>
+      </c>
+      <c r="R20" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="S20" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="T20" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="U20" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="V20" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="W20" t="n">
+        <v>24.34</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>35.9</v>
+      </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2332,42 +2451,25 @@
       </c>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
-        </is>
-      </c>
-      <c r="AH20" t="inlineStr">
-        <is>
-          <t>Vishal Nirmiti Ltd</t>
-        </is>
-      </c>
-      <c r="AM20" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="AR20" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/vishal-nirmiti-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Inox Air Products Limited</t>
+          <t>Everbrands India Limited</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2387,28 +2489,40 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Medical Devices</t>
+          <t>Internet Platforms</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L21" t="n">
-        <v>77156663</v>
+          <t>Fresh</t>
+        </is>
       </c>
       <c r="N21" t="n">
         <v>1</v>
       </c>
+      <c r="Q21" t="n">
+        <v>693.09</v>
+      </c>
+      <c r="R21" t="n">
+        <v>9561.1</v>
+      </c>
+      <c r="V21" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="W21" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>28.2</v>
+      </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -2418,45 +2532,50 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Arete 22 Limited</t>
+          <t>Nityas Gems and Jewellery Limited</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -2477,19 +2596,50 @@
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited_105016.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>Nityas Gems And Jewellery Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ22" t="n">
+        <v>36.47</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/nityas-gems-and-jewellery-ltd</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Deon Energy Limited</t>
+          <t>Pm Cona Industries Limited</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2504,12 +2654,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -2530,39 +2680,34 @@
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/deon-energy-limited_105012.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rathod Jewellery Manufacturing Limited</t>
+          <t>Vishal Nirmiti Limited</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -2583,14 +2728,48 @@
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rathod-jewellery-manufacturing-limited_105014.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>Vishal Nirmiti Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ24" t="n">
+        <v>28.78</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>73.42</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>-2.27</v>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/vishal-nirmiti-ltd</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rudra Green Ship Recycling Limited</t>
+          <t>Inox Air Products Limited</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2610,8 +2789,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Medical Devices</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>77156663</v>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
@@ -2631,19 +2826,24 @@
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited_105008.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kian-M Export Limited</t>
+          <t>Nnt Developers Limited</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2658,12 +2858,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Agri Exports</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -2684,390 +2879,12 @@
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/kian-m-export-limited_104874.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Arohan Financial Services Limited</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>NBFC</t>
-        </is>
-      </c>
-      <c r="AB27" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC27" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE27" t="inlineStr"/>
-      <c r="AF27" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arohan-financial-services-limited-addendum-to-drhp_104860.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Sonaselection India Limited</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB28" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC28" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE28" t="inlineStr"/>
-      <c r="AF28" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/sonaselection-india-limited-prospectus_104876.html</t>
-        </is>
-      </c>
-      <c r="AH28" t="inlineStr">
-        <is>
-          <t>Sonaselection India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI28" t="n">
-        <v>540</v>
-      </c>
-      <c r="AJ28" t="n">
-        <v>32.66</v>
-      </c>
-      <c r="AK28" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="AL28" t="n">
-        <v>64.52</v>
-      </c>
-      <c r="AR28" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/sonaselection-india-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Runwal Enterprises Limited</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB29" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC29" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE29" t="inlineStr"/>
-      <c r="AF29" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/runwal-enterprises-limited-prospectus_104856.html</t>
-        </is>
-      </c>
-      <c r="AH29" t="inlineStr">
-        <is>
-          <t>Runwal Enterprises Ltd.</t>
-        </is>
-      </c>
-      <c r="AI29" t="n">
-        <v>4292</v>
-      </c>
-      <c r="AJ29" t="n">
-        <v>22.29</v>
-      </c>
-      <c r="AK29" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="AL29" t="n">
-        <v>84.61</v>
-      </c>
-      <c r="AM29" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="AN29" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="AO29" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="AP29" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AQ29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR29" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/runwal-enterprises-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SRIT India Limited</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB30" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC30" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE30" t="inlineStr"/>
-      <c r="AF30" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/srit-india-limited-prospectus_104852.html</t>
-        </is>
-      </c>
-      <c r="AH30" t="inlineStr">
-        <is>
-          <t>Srit India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI30" t="n">
-        <v>997</v>
-      </c>
-      <c r="AJ30" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="AK30" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="AL30" t="n">
-        <v>62.71</v>
-      </c>
-      <c r="AM30" t="n">
-        <v>121.24</v>
-      </c>
-      <c r="AN30" t="n">
-        <v>91.84</v>
-      </c>
-      <c r="AO30" t="n">
-        <v>310.94</v>
-      </c>
-      <c r="AP30" t="n">
-        <v>56.75</v>
-      </c>
-      <c r="AQ30" t="n">
-        <v>13.85</v>
-      </c>
-      <c r="AR30" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/srit-india-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>A ONE Steels Limited</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Metals</t>
-        </is>
-      </c>
-      <c r="AB31" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC31" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE31" t="inlineStr"/>
-      <c r="AF31" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/a-one-steels-limited-prospectus_104844.html</t>
-        </is>
-      </c>
-      <c r="AH31" t="inlineStr">
-        <is>
-          <t>A-One Steels India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI31" t="n">
-        <v>2975</v>
-      </c>
-      <c r="AJ31" t="n">
-        <v>15.07</v>
-      </c>
-      <c r="AK31" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="AL31" t="n">
-        <v>74.51000000000001</v>
-      </c>
-      <c r="AM31" t="n">
-        <v>11.35</v>
-      </c>
-      <c r="AN31" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="AO31" t="n">
-        <v>24.38</v>
-      </c>
-      <c r="AP31" t="n">
-        <v>8.18</v>
-      </c>
-      <c r="AQ31" t="n">
-        <v>12.35</v>
-      </c>
-      <c r="AR31" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/aone-steels-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-09)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -2198,7 +2198,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tenty Limited</t>
+          <t>Nnt Developers Limited</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2218,45 +2218,46 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Manufacturing</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="N18" t="n">
         <v>10</v>
       </c>
       <c r="Q18" t="n">
-        <v>822.25</v>
+        <v>223.66</v>
       </c>
       <c r="R18" t="n">
-        <v>97.91</v>
+        <v>7.97</v>
       </c>
       <c r="S18" t="n">
-        <v>22.65</v>
+        <v>21.57</v>
       </c>
       <c r="T18" t="n">
-        <v>232.88</v>
+        <v>5.7</v>
       </c>
       <c r="U18" t="n">
-        <v>2.67</v>
+        <v>9.56</v>
       </c>
       <c r="V18" t="n">
-        <v>9.66</v>
+        <v>14.72</v>
       </c>
       <c r="W18" t="n">
-        <v>6.76</v>
+        <v>24.43</v>
+      </c>
+      <c r="X18" t="n">
+        <v>33.73</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0.39</v>
       </c>
       <c r="AA18" t="n">
-        <v>44.2</v>
+        <v>47.3</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -2276,19 +2277,19 @@
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pci Infraprojects Limited</t>
+          <t>Tenty Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2308,12 +2309,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2325,31 +2326,28 @@
         <v>10</v>
       </c>
       <c r="Q19" t="n">
-        <v>304.09</v>
+        <v>822.25</v>
       </c>
       <c r="R19" t="n">
-        <v>7.68</v>
+        <v>97.91</v>
       </c>
       <c r="S19" t="n">
-        <v>23.85</v>
+        <v>22.65</v>
       </c>
       <c r="T19" t="n">
-        <v>-3.8</v>
+        <v>232.88</v>
       </c>
       <c r="U19" t="n">
-        <v>7.84</v>
+        <v>2.67</v>
       </c>
       <c r="V19" t="n">
-        <v>17.59</v>
+        <v>9.66</v>
       </c>
       <c r="W19" t="n">
-        <v>36.29</v>
-      </c>
-      <c r="X19" t="n">
-        <v>39.97</v>
+        <v>6.76</v>
       </c>
       <c r="AA19" t="n">
-        <v>43.9</v>
+        <v>44.2</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
@@ -2369,19 +2367,19 @@
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Electromech Infraprojects Limited</t>
+          <t>Pci Infraprojects Limited</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2401,7 +2399,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2409,35 +2412,35 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>270.65</v>
-      </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q20" t="n">
-        <v>427.05</v>
+        <v>304.09</v>
       </c>
       <c r="R20" t="n">
-        <v>4.54</v>
+        <v>7.68</v>
       </c>
       <c r="S20" t="n">
-        <v>36.19</v>
+        <v>23.85</v>
       </c>
       <c r="T20" t="n">
-        <v>22.75</v>
+        <v>-3.8</v>
       </c>
       <c r="U20" t="n">
-        <v>8.41</v>
+        <v>7.84</v>
       </c>
       <c r="V20" t="n">
-        <v>10.8</v>
+        <v>17.59</v>
       </c>
       <c r="W20" t="n">
-        <v>24.34</v>
+        <v>36.29</v>
+      </c>
+      <c r="X20" t="n">
+        <v>39.97</v>
       </c>
       <c r="AA20" t="n">
-        <v>35.9</v>
+        <v>43.9</v>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
@@ -2457,19 +2460,19 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Everbrands India Limited</t>
+          <t>Electromech Infraprojects Limited</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2489,36 +2492,43 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Internet Platforms</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Fresh</t>
-        </is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>270.65</v>
       </c>
       <c r="N21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q21" t="n">
-        <v>693.09</v>
+        <v>427.05</v>
       </c>
       <c r="R21" t="n">
-        <v>9561.1</v>
+        <v>4.54</v>
+      </c>
+      <c r="S21" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="T21" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="U21" t="n">
+        <v>8.41</v>
       </c>
       <c r="V21" t="n">
-        <v>10.16</v>
+        <v>10.8</v>
       </c>
       <c r="W21" t="n">
-        <v>10.16</v>
+        <v>24.34</v>
       </c>
       <c r="AA21" t="n">
-        <v>28.2</v>
+        <v>35.9</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
@@ -2538,49 +2548,72 @@
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Nityas Gems and Jewellery Limited</t>
+          <t>Everbrands India Limited</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Jewellery</t>
-        </is>
+          <t>Internet Platforms</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>693.09</v>
+      </c>
+      <c r="R22" t="n">
+        <v>9561.1</v>
+      </c>
+      <c r="V22" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="W22" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>28.2</v>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC22" t="inlineStr">
@@ -2590,76 +2623,50 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
-        </is>
-      </c>
-      <c r="AH22" t="inlineStr">
-        <is>
-          <t>Nityas Gems And Jewellery Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ22" t="n">
-        <v>36.47</v>
-      </c>
-      <c r="AK22" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AP22" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="AQ22" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="AR22" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/nityas-gems-and-jewellery-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pm Cona Industries Limited</t>
+          <t>Nityas Gems and Jewellery Limited</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Diversified Industrials</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -2680,14 +2687,51 @@
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>Nityas Gems And Jewellery Ltd.</t>
+        </is>
+      </c>
+      <c r="AI23" t="n">
+        <v>485</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>36.47</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>43.51</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AO23" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AP23" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/nityas-gems-and-jewellery-ltd</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Vishal Nirmiti Limited</t>
+          <t>Pm Cona Industries Limited</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2697,17 +2741,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -2728,85 +2777,35 @@
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
-        </is>
-      </c>
-      <c r="AH24" t="inlineStr">
-        <is>
-          <t>Vishal Nirmiti Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ24" t="n">
-        <v>28.78</v>
-      </c>
-      <c r="AK24" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AL24" t="n">
-        <v>73.42</v>
-      </c>
-      <c r="AM24" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="AN24" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="AO24" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="AP24" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>-2.27</v>
-      </c>
-      <c r="AR24" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/vishal-nirmiti-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Inox Air Products Limited</t>
+          <t>Vishal Nirmiti Limited</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Medical Devices</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L25" t="n">
-        <v>77156663</v>
-      </c>
-      <c r="N25" t="n">
-        <v>1</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
@@ -2826,19 +2825,51 @@
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
-        </is>
-      </c>
-      <c r="AG25" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>Vishal Nirmiti Ltd.</t>
+        </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>539</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>28.78</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>-2.27</v>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/vishal-nirmiti-ltd</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Nnt Developers Limited</t>
+          <t>Inox Air Products Limited</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2858,8 +2889,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Medical Devices</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>77156663</v>
+      </c>
+      <c r="N26" t="n">
+        <v>1</v>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
@@ -2879,12 +2926,12 @@
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
         </is>
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-11)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -1738,7 +1738,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Arete 22 Limited</t>
+          <t>B S Sponge Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1758,42 +1758,54 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
+      </c>
+      <c r="J13" t="n">
+        <v>1000</v>
       </c>
       <c r="N13" t="n">
         <v>10</v>
       </c>
       <c r="Q13" t="n">
-        <v>537.95</v>
+        <v>2592.52</v>
       </c>
       <c r="R13" t="n">
-        <v>153.28</v>
+        <v>18.5</v>
       </c>
       <c r="S13" t="n">
-        <v>44.97</v>
+        <v>171.11</v>
       </c>
       <c r="T13" t="n">
-        <v>263.98</v>
+        <v>8</v>
       </c>
       <c r="U13" t="n">
-        <v>8.359999999999999</v>
+        <v>6.57</v>
+      </c>
+      <c r="V13" t="n">
+        <v>14.83</v>
       </c>
       <c r="W13" t="n">
-        <v>75.22</v>
+        <v>24.18</v>
+      </c>
+      <c r="X13" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0.97</v>
       </c>
       <c r="AA13" t="n">
-        <v>60</v>
+        <v>57.9</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
@@ -1813,19 +1825,19 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited-drhp_105016.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/b-s-sponge-limited-drhp_105023.html</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Arete%2022%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/B%20S%20Sponge%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>B S Sponge Limited</t>
+          <t>Anarock Property Consultants Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1845,12 +1857,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1858,41 +1870,35 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>1000</v>
-      </c>
       <c r="N14" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>2592.52</v>
+        <v>881.9</v>
       </c>
       <c r="R14" t="n">
-        <v>18.5</v>
+        <v>33.83</v>
       </c>
       <c r="S14" t="n">
-        <v>171.11</v>
+        <v>93.22</v>
       </c>
       <c r="T14" t="n">
-        <v>8</v>
+        <v>53.38</v>
       </c>
       <c r="U14" t="n">
-        <v>6.57</v>
+        <v>10.57</v>
       </c>
       <c r="V14" t="n">
-        <v>14.83</v>
+        <v>17.1</v>
       </c>
       <c r="W14" t="n">
-        <v>24.18</v>
-      </c>
-      <c r="X14" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>0.97</v>
+        <v>15.64</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>66.41</v>
       </c>
       <c r="AA14" t="n">
-        <v>57.9</v>
+        <v>57.6</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
@@ -1912,19 +1918,19 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/b-s-sponge-limited-drhp_105023.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/anarock-property-consultants-limited-drhp_104988.html</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/B%20S%20Sponge%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Anarock%20Property%20Consultants%20Limited%20-%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Anarock Property Consultants Limited</t>
+          <t>Rudra Green Ship Recycling Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1944,12 +1950,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1958,34 +1959,37 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q15" t="n">
-        <v>881.9</v>
+        <v>204.52</v>
       </c>
       <c r="R15" t="n">
-        <v>33.83</v>
+        <v>14.13</v>
       </c>
       <c r="S15" t="n">
-        <v>93.22</v>
+        <v>12.65</v>
       </c>
       <c r="T15" t="n">
-        <v>53.38</v>
+        <v>28.83</v>
       </c>
       <c r="U15" t="n">
-        <v>10.57</v>
+        <v>6.17</v>
       </c>
       <c r="V15" t="n">
-        <v>17.1</v>
+        <v>10.65</v>
       </c>
       <c r="W15" t="n">
-        <v>15.64</v>
+        <v>27.4</v>
+      </c>
+      <c r="X15" t="n">
+        <v>19.03</v>
       </c>
       <c r="Z15" t="n">
-        <v>66.41</v>
+        <v>98.86</v>
       </c>
       <c r="AA15" t="n">
-        <v>57.6</v>
+        <v>53.4</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
@@ -2005,19 +2009,19 @@
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/anarock-property-consultants-limited-drhp_104988.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited-drhp_105008.html</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Anarock%20Property%20Consultants%20Limited%20-%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Rudra%20Green%20Ship%20Recycling%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Rudra Green Ship Recycling Limited</t>
+          <t>Inox Clean Energy Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2037,7 +2041,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Power</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2046,37 +2055,31 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>204.52</v>
+        <v>178.13</v>
       </c>
       <c r="R16" t="n">
-        <v>14.13</v>
+        <v>20.8</v>
       </c>
       <c r="S16" t="n">
-        <v>12.65</v>
+        <v>30.98</v>
       </c>
       <c r="T16" t="n">
-        <v>28.83</v>
+        <v>1891.07</v>
       </c>
       <c r="U16" t="n">
-        <v>6.17</v>
+        <v>17.39</v>
       </c>
       <c r="V16" t="n">
-        <v>10.65</v>
+        <v>18.11</v>
       </c>
       <c r="W16" t="n">
-        <v>27.4</v>
-      </c>
-      <c r="X16" t="n">
-        <v>19.03</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>98.86</v>
+        <v>1.33</v>
       </c>
       <c r="AA16" t="n">
-        <v>53.4</v>
+        <v>47.6</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
@@ -2096,19 +2099,19 @@
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/rudra-green-ship-recycling-limited-drhp_105008.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited-drhp_105010.html</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Rudra%20Green%20Ship%20Recycling%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Clean%20Energy%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Inox Clean Energy Limited</t>
+          <t>Nnt Developers Limited</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2128,45 +2131,46 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Power</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q17" t="n">
-        <v>178.13</v>
+        <v>223.66</v>
       </c>
       <c r="R17" t="n">
-        <v>20.8</v>
+        <v>7.97</v>
       </c>
       <c r="S17" t="n">
-        <v>30.98</v>
+        <v>21.57</v>
       </c>
       <c r="T17" t="n">
-        <v>1891.07</v>
+        <v>5.7</v>
       </c>
       <c r="U17" t="n">
-        <v>17.39</v>
+        <v>9.56</v>
       </c>
       <c r="V17" t="n">
-        <v>18.11</v>
+        <v>14.72</v>
       </c>
       <c r="W17" t="n">
-        <v>1.33</v>
+        <v>24.43</v>
+      </c>
+      <c r="X17" t="n">
+        <v>33.73</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0.39</v>
       </c>
       <c r="AA17" t="n">
-        <v>47.6</v>
+        <v>47.3</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
@@ -2186,19 +2190,19 @@
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-clean-energy-limited-drhp_105010.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Clean%20Energy%20Limited_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nnt Developers Limited</t>
+          <t>Tenty Limited</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2218,46 +2222,45 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="N18" t="n">
         <v>10</v>
       </c>
       <c r="Q18" t="n">
-        <v>223.66</v>
+        <v>822.25</v>
       </c>
       <c r="R18" t="n">
-        <v>7.97</v>
+        <v>97.91</v>
       </c>
       <c r="S18" t="n">
-        <v>21.57</v>
+        <v>22.65</v>
       </c>
       <c r="T18" t="n">
-        <v>5.7</v>
+        <v>232.88</v>
       </c>
       <c r="U18" t="n">
-        <v>9.56</v>
+        <v>2.67</v>
       </c>
       <c r="V18" t="n">
-        <v>14.72</v>
+        <v>9.66</v>
       </c>
       <c r="W18" t="n">
-        <v>24.43</v>
-      </c>
-      <c r="X18" t="n">
-        <v>33.73</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>0.39</v>
+        <v>6.76</v>
       </c>
       <c r="AA18" t="n">
-        <v>47.3</v>
+        <v>44.2</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -2277,19 +2280,19 @@
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nnt-developers-limited-drhp_105000.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/NNT%20DEVELOPERS%20LIMITED%20-%20%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Tenty Limited</t>
+          <t>Pci Infraprojects Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2309,12 +2312,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2326,28 +2329,31 @@
         <v>10</v>
       </c>
       <c r="Q19" t="n">
-        <v>822.25</v>
+        <v>304.09</v>
       </c>
       <c r="R19" t="n">
-        <v>97.91</v>
+        <v>7.68</v>
       </c>
       <c r="S19" t="n">
-        <v>22.65</v>
+        <v>23.85</v>
       </c>
       <c r="T19" t="n">
-        <v>232.88</v>
+        <v>-3.8</v>
       </c>
       <c r="U19" t="n">
-        <v>2.67</v>
+        <v>7.84</v>
       </c>
       <c r="V19" t="n">
-        <v>9.66</v>
+        <v>17.59</v>
       </c>
       <c r="W19" t="n">
-        <v>6.76</v>
+        <v>36.29</v>
+      </c>
+      <c r="X19" t="n">
+        <v>39.97</v>
       </c>
       <c r="AA19" t="n">
-        <v>44.2</v>
+        <v>43.9</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
@@ -2367,19 +2373,19 @@
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tenty-limited-drhp_105006.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Tenty%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pci Infraprojects Limited</t>
+          <t>Electromech Infraprojects Limited</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2399,12 +2405,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Renewables</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2412,35 +2413,35 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="J20" t="n">
+        <v>270.65</v>
+      </c>
       <c r="N20" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q20" t="n">
-        <v>304.09</v>
+        <v>427.05</v>
       </c>
       <c r="R20" t="n">
-        <v>7.68</v>
+        <v>4.54</v>
       </c>
       <c r="S20" t="n">
-        <v>23.85</v>
+        <v>36.19</v>
       </c>
       <c r="T20" t="n">
-        <v>-3.8</v>
+        <v>22.75</v>
       </c>
       <c r="U20" t="n">
-        <v>7.84</v>
+        <v>8.41</v>
       </c>
       <c r="V20" t="n">
-        <v>17.59</v>
+        <v>10.8</v>
       </c>
       <c r="W20" t="n">
-        <v>36.29</v>
-      </c>
-      <c r="X20" t="n">
-        <v>39.97</v>
+        <v>24.34</v>
       </c>
       <c r="AA20" t="n">
-        <v>43.9</v>
+        <v>35.9</v>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
@@ -2460,19 +2461,19 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pci-infraprojects-limited-drhp_104989.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/PCI%20INFRAPROJECTS%20LIMITED%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Electromech Infraprojects Limited</t>
+          <t>Everbrands India Limited</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2492,43 +2493,36 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Internet Platforms</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>270.65</v>
+          <t>Fresh</t>
+        </is>
       </c>
       <c r="N21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>427.05</v>
+        <v>693.09</v>
       </c>
       <c r="R21" t="n">
-        <v>4.54</v>
-      </c>
-      <c r="S21" t="n">
-        <v>36.19</v>
-      </c>
-      <c r="T21" t="n">
-        <v>22.75</v>
-      </c>
-      <c r="U21" t="n">
-        <v>8.41</v>
+        <v>9561.1</v>
       </c>
       <c r="V21" t="n">
-        <v>10.8</v>
+        <v>10.16</v>
       </c>
       <c r="W21" t="n">
-        <v>24.34</v>
+        <v>10.16</v>
       </c>
       <c r="AA21" t="n">
-        <v>35.9</v>
+        <v>28.2</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
@@ -2548,72 +2542,49 @@
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/electromech-infraprojects-limited-drhp_105027.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Electromech%20Infraprojects%20Limited%20-%20ADP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Everbrands India Limited</t>
+          <t>Nityas Gems and Jewellery Limited</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Internet Platforms</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>693.09</v>
-      </c>
-      <c r="R22" t="n">
-        <v>9561.1</v>
-      </c>
-      <c r="V22" t="n">
-        <v>10.16</v>
-      </c>
-      <c r="W22" t="n">
-        <v>10.16</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>28.2</v>
+          <t>Jewellery</t>
+        </is>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC22" t="inlineStr">
@@ -2623,50 +2594,82 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/everbrands-india-limited-drhp_105022.html</t>
-        </is>
-      </c>
-      <c r="AG22" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/EverBrandsIndiaLimitedDAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>Nityas Gems And Jewellery Ltd.</t>
+        </is>
+      </c>
+      <c r="AI22" t="n">
+        <v>485</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>36.47</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>43.51</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/nityas-gems-and-jewellery-ltd</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Nityas Gems and Jewellery Limited</t>
+          <t>Pm Cona Industries Limited</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -2687,51 +2690,14 @@
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
-        </is>
-      </c>
-      <c r="AH23" t="inlineStr">
-        <is>
-          <t>Nityas Gems And Jewellery Ltd.</t>
-        </is>
-      </c>
-      <c r="AI23" t="n">
-        <v>485</v>
-      </c>
-      <c r="AJ23" t="n">
-        <v>36.47</v>
-      </c>
-      <c r="AK23" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="AL23" t="n">
-        <v>43.51</v>
-      </c>
-      <c r="AM23" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="AN23" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AO23" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AP23" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="AQ23" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="AR23" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/nityas-gems-and-jewellery-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pm Cona Industries Limited</t>
+          <t>Vishal Nirmiti Limited</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2741,22 +2707,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Diversified Industrials</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -2777,35 +2738,88 @@
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>Vishal Nirmiti Ltd.</t>
+        </is>
+      </c>
+      <c r="AI24" t="n">
+        <v>539</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>28.78</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>-2.27</v>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/vishal-nirmiti-ltd</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Vishal Nirmiti Limited</t>
+          <t>Inox Air Products Limited</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Medical Devices</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>77156663</v>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
@@ -2825,51 +2839,19 @@
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
-        </is>
-      </c>
-      <c r="AH25" t="inlineStr">
-        <is>
-          <t>Vishal Nirmiti Ltd.</t>
-        </is>
-      </c>
-      <c r="AI25" t="n">
-        <v>539</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>28.78</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="AN25" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="AO25" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="AP25" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="AQ25" t="n">
-        <v>-2.27</v>
-      </c>
-      <c r="AR25" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/vishal-nirmiti-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Inox Air Products Limited</t>
+          <t>Arete 22 Limited</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2889,24 +2871,8 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Medical Devices</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L26" t="n">
-        <v>77156663</v>
-      </c>
-      <c r="N26" t="n">
-        <v>1</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
@@ -2926,12 +2892,12 @@
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/inox-air-products-limited-drhp_105024.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/arete-22-limited-drhp_105016.html</t>
         </is>
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Inox%20Air%20Products%20Limited-%20Draft%20Abridged%20prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Arete%2022%20Limited_p.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-13)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR8"/>
+  <dimension ref="A1:AR5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pentacle Consultants I Limited</t>
+          <t>Grace Renewable Energy Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -719,57 +719,48 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NBFC</t>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
-      </c>
-      <c r="J2" t="n">
-        <v>22.17</v>
       </c>
       <c r="N2" t="n">
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>91.73</v>
+        <v>205.84</v>
       </c>
       <c r="R2" t="n">
-        <v>52.3</v>
+        <v>70.83</v>
       </c>
       <c r="S2" t="n">
-        <v>28.86</v>
+        <v>18.67</v>
       </c>
       <c r="T2" t="n">
-        <v>174.54</v>
+        <v>91.06</v>
       </c>
       <c r="U2" t="n">
-        <v>31.46</v>
+        <v>9.07</v>
       </c>
       <c r="V2" t="n">
-        <v>36.04</v>
+        <v>12.53</v>
       </c>
       <c r="W2" t="n">
-        <v>49.11</v>
+        <v>65.73</v>
       </c>
       <c r="X2" t="n">
-        <v>33.57</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>70.79000000000001</v>
+        <v>80.45</v>
       </c>
       <c r="AA2" t="n">
-        <v>85.3</v>
+        <v>74.7</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -789,19 +780,19 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pentacle-consultants-i-limited_105039.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/grace-renewable-energy-limited-drhp_105099.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Pentacle%20Consultants%20(I)%20Limited-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Grace%20Renewable%20Energy%20Limited%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Grace Renewable Energy Limited</t>
+          <t>Integrum Energy Infrastructure Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -826,7 +817,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -835,34 +826,34 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>205.84</v>
+        <v>693.84</v>
       </c>
       <c r="R3" t="n">
-        <v>70.83</v>
+        <v>489.67</v>
       </c>
       <c r="S3" t="n">
-        <v>18.67</v>
+        <v>63.16</v>
       </c>
       <c r="T3" t="n">
-        <v>91.06</v>
+        <v>400.13</v>
       </c>
       <c r="U3" t="n">
-        <v>9.07</v>
+        <v>9.1</v>
       </c>
       <c r="V3" t="n">
-        <v>12.53</v>
+        <v>12.72</v>
       </c>
       <c r="W3" t="n">
-        <v>65.73</v>
-      </c>
-      <c r="X3" t="n">
-        <v>80.45</v>
+        <v>42.2</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>90.66</v>
       </c>
       <c r="AA3" t="n">
-        <v>74.7</v>
+        <v>61.2</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -882,132 +873,92 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/grace-renewable-energy-limited-drhp_105099.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integrum-energy-infrastructure-limited-drhp_105075.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Grace%20Renewable%20Energy%20Limited%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/INTEGRUM%20ENERGY%20INFRASTRUCTURE%20LIMITED-Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Integrum Energy Infrastructure Limited</t>
+          <t>Matangi Rubber Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>693.84</v>
-      </c>
-      <c r="R4" t="n">
-        <v>489.67</v>
-      </c>
-      <c r="S4" t="n">
-        <v>63.16</v>
-      </c>
-      <c r="T4" t="n">
-        <v>400.13</v>
-      </c>
-      <c r="U4" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="V4" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="W4" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>90.66</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>61.2</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integrum-energy-infrastructure-limited-drhp_105075.html</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/INTEGRUM%20ENERGY%20INFRASTRUCTURE%20LIMITED-Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/matangi-rubber-limited-addendum-to-the-drhp_105143.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Matangi Rubber Limited</t>
+          <t>Nityas Gems and Jewellery Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1017,7 +968,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -1028,235 +979,44 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/matangi-rubber-limited-addendum-to-the-drhp_105143.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Nityas Gems and Jewellery Limited</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr">
-        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>Nityas Gems And Jewellery Ltd.</t>
         </is>
       </c>
-      <c r="AI6" t="n">
-        <v>460</v>
-      </c>
-      <c r="AJ6" t="n">
+      <c r="AI5" t="n">
+        <v>437</v>
+      </c>
+      <c r="AJ5" t="n">
         <v>36.47</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AK5" t="n">
         <v>0.38</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AL5" t="n">
         <v>43.51</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="AM5" t="n">
         <v>2.19</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="AN5" t="n">
         <v>1.06</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AO5" t="n">
         <v>2.03</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="AP5" t="n">
         <v>3.88</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="AQ5" t="n">
         <v>6.67</v>
       </c>
-      <c r="AR6" t="inlineStr">
+      <c r="AR5" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/nityas-gems-and-jewellery-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Pm Cona Industries Limited</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Diversified Industrials</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/pm-cona-industries-limited_105041.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Vishal Nirmiti Limited</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/vishal-nirmiti-limited-prospectus_105057.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>Vishal Nirmiti Ltd.</t>
-        </is>
-      </c>
-      <c r="AI8" t="n">
-        <v>512</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>28.78</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>-2.27</v>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/vishal-nirmiti-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-14)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR5"/>
+  <dimension ref="A1:AR4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Grace Renewable Energy Limited</t>
+          <t>Soleos Energy Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -733,34 +733,34 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q2" t="n">
-        <v>205.84</v>
+        <v>281.16</v>
       </c>
       <c r="R2" t="n">
-        <v>70.83</v>
+        <v>26.74</v>
       </c>
       <c r="S2" t="n">
-        <v>18.67</v>
+        <v>21.48</v>
       </c>
       <c r="T2" t="n">
-        <v>91.06</v>
+        <v>-13.51</v>
       </c>
       <c r="U2" t="n">
-        <v>9.07</v>
+        <v>7.64</v>
       </c>
       <c r="V2" t="n">
-        <v>12.53</v>
+        <v>10.65</v>
       </c>
       <c r="W2" t="n">
-        <v>65.73</v>
-      </c>
-      <c r="X2" t="n">
-        <v>80.45</v>
+        <v>10.8</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.51</v>
       </c>
       <c r="AA2" t="n">
-        <v>74.7</v>
+        <v>32.8</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -780,105 +780,60 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/grace-renewable-energy-limited-drhp_105099.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/soleos-energy-limited-drhp_105196.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Grace%20Renewable%20Energy%20Limited%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Soleos%20Energy%20Limited_Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Integrum Energy Infrastructure Limited</t>
+          <t>Oswal Cables Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>693.84</v>
-      </c>
-      <c r="R3" t="n">
-        <v>489.67</v>
-      </c>
-      <c r="S3" t="n">
-        <v>63.16</v>
-      </c>
-      <c r="T3" t="n">
-        <v>400.13</v>
-      </c>
-      <c r="U3" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="V3" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="W3" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>90.66</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>61.2</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integrum-energy-infrastructure-limited-drhp_105075.html</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/INTEGRUM%20ENERGY%20INFRASTRUCTURE%20LIMITED-Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oswal-cables-limited-addendum-to-drhp_105234.html</t>
         </is>
       </c>
     </row>
@@ -927,96 +882,6 @@
       <c r="AF4" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/matangi-rubber-limited-addendum-to-the-drhp_105143.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Nityas Gems and Jewellery Limited</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/nityas-gems-and-jewellery-limited-prospectus_105059.html</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>Nityas Gems And Jewellery Ltd.</t>
-        </is>
-      </c>
-      <c r="AI5" t="n">
-        <v>437</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>36.47</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>43.51</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/nityas-gems-and-jewellery-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-15)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR4"/>
+  <dimension ref="A1:AR5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,32 +699,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Soleos Energy Limited</t>
+          <t>Paramotor Digital Technology Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>UDRHP</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>IT Services</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -733,34 +733,31 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>281.16</v>
+        <v>20.92</v>
       </c>
       <c r="R2" t="n">
-        <v>26.74</v>
+        <v>-96.53</v>
       </c>
       <c r="S2" t="n">
-        <v>21.48</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="T2" t="n">
-        <v>-13.51</v>
+        <v>-84.40000000000001</v>
       </c>
       <c r="U2" t="n">
-        <v>7.64</v>
+        <v>44.1</v>
       </c>
       <c r="V2" t="n">
-        <v>10.65</v>
+        <v>58.97</v>
       </c>
       <c r="W2" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0.51</v>
+        <v>23.56</v>
       </c>
       <c r="AA2" t="n">
-        <v>32.8</v>
+        <v>34.2</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -769,7 +766,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -780,29 +777,29 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/soleos-energy-limited-drhp_105196.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/paramotor-digital-technology-limited-udrhp-i_105258.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Soleos%20Energy%20Limited_Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Paramotor%20Digital%20Technology%20Limited_DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Oswal Cables Limited</t>
+          <t>Soleos Energy Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -812,40 +809,85 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>281.16</v>
+      </c>
+      <c r="R3" t="n">
+        <v>26.74</v>
+      </c>
+      <c r="S3" t="n">
+        <v>21.48</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-13.51</v>
+      </c>
+      <c r="U3" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="V3" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="W3" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>32.8</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oswal-cables-limited-addendum-to-drhp_105234.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/soleos-energy-limited-drhp_105196.html</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Soleos%20Energy%20Limited_Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Matangi Rubber Limited</t>
+          <t>Oswal Cables Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -880,6 +922,54 @@
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oswal-cables-limited-addendum-to-drhp_105234.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Matangi Rubber Limited</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/matangi-rubber-limited-addendum-to-the-drhp_105143.html</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-17)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR5"/>
+  <dimension ref="A1:AR4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -927,54 +927,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Matangi Rubber Limited</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/matangi-rubber-limited-addendum-to-the-drhp_105143.html</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-19)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR4"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -879,54 +879,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Oswal Cables Limited</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oswal-cables-limited-addendum-to-drhp_105234.html</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-20)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -786,99 +786,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Soleos Energy Limited</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>281.16</v>
-      </c>
-      <c r="R3" t="n">
-        <v>26.74</v>
-      </c>
-      <c r="S3" t="n">
-        <v>21.48</v>
-      </c>
-      <c r="T3" t="n">
-        <v>-13.51</v>
-      </c>
-      <c r="U3" t="n">
-        <v>7.64</v>
-      </c>
-      <c r="V3" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="W3" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>32.8</v>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>DIG DEEPER</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>DRHP_PDF, derived</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/soleos-energy-limited-drhp_105196.html</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Soleos%20Energy%20Limited_Prospectus_p.pdf</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-21)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR2"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,17 +699,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Paramotor Digital Technology Limited</t>
+          <t>Tablespace Technologies Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -727,41 +727,9 @@
           <t>IT Services</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>20.92</v>
-      </c>
-      <c r="R2" t="n">
-        <v>-96.53</v>
-      </c>
-      <c r="S2" t="n">
-        <v>9.220000000000001</v>
-      </c>
-      <c r="T2" t="n">
-        <v>-84.40000000000001</v>
-      </c>
-      <c r="U2" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="V2" t="n">
-        <v>58.97</v>
-      </c>
-      <c r="W2" t="n">
-        <v>23.56</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>34.2</v>
-      </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -771,18 +739,92 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/paramotor-digital-technology-limited-udrhp-i_105258.html</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Paramotor%20Digital%20Technology%20Limited_DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tablespace-technologies-limited-addendum-to-drhp_105343.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HD Fire Protect Limited</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/hd-fire-protect-limited-prospectus_105337.html</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>HD Fire Protect Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ3" t="n">
+        <v>30.97</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>130.81</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>256.65</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>202.73</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>28.91</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>23.62</v>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/hd-fire-protect-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-22)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AR5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,7 +699,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tablespace Technologies Limited</t>
+          <t>Hunger Pangs Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -719,45 +719,77 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>IT Services</t>
-        </is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>27929760</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>155.5</v>
+      </c>
+      <c r="R2" t="n">
+        <v>46.56</v>
+      </c>
+      <c r="S2" t="n">
+        <v>-0.98</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-0.63</v>
+      </c>
+      <c r="V2" t="n">
+        <v>16.51</v>
+      </c>
+      <c r="W2" t="n">
+        <v>-24</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>20.5</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>MONITOR</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tablespace-technologies-limited-addendum-to-drhp_105343.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/hunger-pangs-limited-drhp_105347.html</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Draft%20Abridged%20prospectus%20of%20Hunger%20Pangs%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HD Fire Protect Limited</t>
+          <t>Tonbo Imaging India Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -793,36 +825,143 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tablespace Technologies Limited</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>IT Services</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tablespace-technologies-limited-addendum-to-drhp_105343.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HD Fire Protect Limited</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
+        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/hd-fire-protect-limited-prospectus_105337.html</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>HD Fire Protect Ltd.</t>
         </is>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AI5" t="n">
+        <v>5383</v>
+      </c>
+      <c r="AJ5" t="n">
         <v>30.97</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AK5" t="n">
         <v>0</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="AL5" t="n">
+        <v>85</v>
+      </c>
+      <c r="AM5" t="n">
         <v>130.81</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="AN5" t="n">
         <v>256.65</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="AO5" t="n">
         <v>202.73</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="AP5" t="n">
         <v>28.91</v>
       </c>
-      <c r="AQ3" t="n">
+      <c r="AQ5" t="n">
         <v>23.62</v>
       </c>
-      <c r="AR3" t="inlineStr">
+      <c r="AR5" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/hd-fire-protect-ltd</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-23)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR5"/>
+  <dimension ref="A1:AR4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -828,6 +828,22 @@
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
         </is>
       </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Tonbo Imaging India Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/tonbo-imaging-india-ltd</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -879,91 +895,6 @@
       <c r="AF4" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tablespace-technologies-limited-addendum-to-drhp_105343.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>HD Fire Protect Limited</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/hd-fire-protect-limited-prospectus_105337.html</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>HD Fire Protect Ltd.</t>
-        </is>
-      </c>
-      <c r="AI5" t="n">
-        <v>5383</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>30.97</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>85</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>130.81</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>256.65</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>202.73</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>28.91</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>23.62</v>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/hd-fire-protect-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-26)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR4"/>
+  <dimension ref="A1:AR7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,7 +699,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hunger Pangs Limited</t>
+          <t>GAMP Services Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -727,36 +727,42 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>27929760</v>
-      </c>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>155.5</v>
+        <v>45.81</v>
       </c>
       <c r="R2" t="n">
-        <v>46.56</v>
+        <v>28.35</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.98</v>
+        <v>10.97</v>
+      </c>
+      <c r="T2" t="n">
+        <v>37.91</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.63</v>
+        <v>23.82</v>
       </c>
       <c r="V2" t="n">
-        <v>16.51</v>
+        <v>33.14</v>
       </c>
       <c r="W2" t="n">
-        <v>-24</v>
+        <v>53.21</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>99.98999999999999</v>
       </c>
       <c r="AA2" t="n">
-        <v>20.5</v>
+        <v>68.3</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>MONITOR</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -772,34 +778,34 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/hunger-pangs-limited-drhp_105347.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/gamp-services-limited-drhp_105424.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Draft%20Abridged%20prospectus%20of%20Hunger%20Pangs%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/GAMP%20Services%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tonbo Imaging India Limited</t>
+          <t>Hunger Pangs Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -807,9 +813,41 @@
           <t>Unclassified</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>27929760</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>155.5</v>
+      </c>
+      <c r="R3" t="n">
+        <v>46.56</v>
+      </c>
+      <c r="S3" t="n">
+        <v>-0.98</v>
+      </c>
+      <c r="U3" t="n">
+        <v>-0.63</v>
+      </c>
+      <c r="V3" t="n">
+        <v>16.51</v>
+      </c>
+      <c r="W3" t="n">
+        <v>-24</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>20.5</v>
+      </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>MONITOR</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -819,41 +857,30 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>Tonbo Imaging India Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/tonbo-imaging-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/hunger-pangs-limited-drhp_105347.html</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Draft%20Abridged%20prospectus%20of%20Hunger%20Pangs%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tablespace Technologies Limited</t>
+          <t>Oravel Stays Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -868,12 +895,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>IT Services</t>
+          <t>Hospitality</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -893,6 +920,177 @@
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Integris Medtech Limited</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tonbo Imaging India Limited</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Tonbo Imaging India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI6" t="n">
+        <v>6494</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>14.56</v>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/tonbo-imaging-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tablespace Technologies Limited</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>IT Services</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tablespace-technologies-limited-addendum-to-drhp_105343.html</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-27)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR7"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -875,17 +875,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oravel Stays Limited</t>
+          <t>INTELLIUS RECODE LIMITED - Notice to Investors</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -895,12 +895,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Hospitality</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -910,7 +905,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -921,14 +916,14 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/intellius-recode-limited-notice-to-investors_105445.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Integris Medtech Limited</t>
+          <t>Oravel Stays Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -948,7 +943,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Hospitality</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -969,29 +969,29 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tonbo Imaging India Limited</t>
+          <t>Integris Medtech Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -1017,51 +1017,29 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>Tonbo Imaging India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI6" t="n">
-        <v>6494</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>14.56</v>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/tonbo-imaging-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tablespace Technologies Limited</t>
+          <t>Jio Platforms Ltd.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1071,7 +1049,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>IT Services</t>
+          <t>Internet Platforms</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1081,7 +1059,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1091,6 +1069,151 @@
       </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jio-platforms-ltd-prospectus_105427.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Jio Platforms Ltd</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
+        <v>21.46</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>67.68000000000001</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/reliance-jio-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tonbo Imaging India Limited</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>Tonbo Imaging India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI8" t="n">
+        <v>6948</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>14.56</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/tonbo-imaging-india-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tablespace Technologies Limited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>IT Services</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tablespace-technologies-limited-addendum-to-drhp_105343.html</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-28)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AR6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GAMP Services Limited</t>
+          <t>INTELLIUS RECODE LIMITED - Notice to Investors</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -722,47 +722,9 @@
           <t>Unclassified</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>45.81</v>
-      </c>
-      <c r="R2" t="n">
-        <v>28.35</v>
-      </c>
-      <c r="S2" t="n">
-        <v>10.97</v>
-      </c>
-      <c r="T2" t="n">
-        <v>37.91</v>
-      </c>
-      <c r="U2" t="n">
-        <v>23.82</v>
-      </c>
-      <c r="V2" t="n">
-        <v>33.14</v>
-      </c>
-      <c r="W2" t="n">
-        <v>53.21</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>99.98999999999999</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>68.3</v>
-      </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -772,127 +734,90 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/gamp-services-limited-drhp_105424.html</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/GAMP%20Services%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/intellius-recode-limited-notice-to-investors_105445.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hunger Pangs Limited</t>
+          <t>Oravel Stays Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>27929760</v>
-      </c>
-      <c r="N3" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>155.5</v>
-      </c>
-      <c r="R3" t="n">
-        <v>46.56</v>
-      </c>
-      <c r="S3" t="n">
-        <v>-0.98</v>
-      </c>
-      <c r="U3" t="n">
-        <v>-0.63</v>
-      </c>
-      <c r="V3" t="n">
-        <v>16.51</v>
-      </c>
-      <c r="W3" t="n">
-        <v>-24</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>20.5</v>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Hospitality</t>
+        </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>MONITOR</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/hunger-pangs-limited-drhp_105347.html</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Draft%20Abridged%20prospectus%20of%20Hunger%20Pangs%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INTELLIUS RECODE LIMITED - Notice to Investors</t>
+          <t>Integris Medtech Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Unclassified</t>
@@ -905,7 +830,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -916,14 +841,14 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/intellius-recode-limited-notice-to-investors_105445.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oravel Stays Limited</t>
+          <t>Jio Platforms Ltd.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -933,22 +858,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Hospitality</t>
+          <t>Internet Platforms</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -958,7 +883,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -969,29 +894,63 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jio-platforms-ltd-prospectus_105427.html</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Jio Platforms Ltd.</t>
+        </is>
+      </c>
+      <c r="AJ5" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>66.43000000000001</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>21.46</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>67.68000000000001</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/jio-platforms-ltd</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Integris Medtech Limited</t>
+          <t>Tonbo Imaging India Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1006,7 +965,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -1017,205 +976,29 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Jio Platforms Ltd.</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Internet Platforms</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jio-platforms-ltd-prospectus_105427.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Jio Platforms Ltd</t>
-        </is>
-      </c>
-      <c r="AM7" t="n">
-        <v>21.46</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>67.68000000000001</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>13.99</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/reliance-jio-ipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Tonbo Imaging India Limited</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr">
-        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>Tonbo Imaging India Ltd.</t>
         </is>
       </c>
-      <c r="AI8" t="n">
-        <v>6948</v>
-      </c>
-      <c r="AJ8" t="n">
+      <c r="AI6" t="n">
+        <v>7377</v>
+      </c>
+      <c r="AJ6" t="n">
         <v>0</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="AK6" t="n">
         <v>0.26</v>
       </c>
-      <c r="AL8" t="n">
+      <c r="AL6" t="n">
         <v>14.56</v>
       </c>
-      <c r="AR8" t="inlineStr">
+      <c r="AR6" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/tonbo-imaging-india-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Tablespace Technologies Limited</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>IT Services</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tablespace-technologies-limited-addendum-to-drhp_105343.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-29)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -699,27 +699,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INTELLIUS RECODE LIMITED - Notice to Investors</t>
+          <t>Paras Healthcare Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Hospitals</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -740,24 +745,61 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/intellius-recode-limited-notice-to-investors_105445.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/paras-healthcare-limited-prospectus_105471.html</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Paras Healthcare Ltd.</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>7976</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/paras-healthcare-ltd</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Oravel Stays Limited</t>
+          <t>INTELLIUS RECODE LIMITED - Notice to Investors</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -767,12 +809,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Hospitality</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -782,7 +819,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -793,14 +830,14 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/intellius-recode-limited-notice-to-investors_105445.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Integris Medtech Limited</t>
+          <t>Oravel Stays Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -820,7 +857,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Hospitality</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -841,14 +883,14 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jio Platforms Ltd.</t>
+          <t>Integris Medtech Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -858,22 +900,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Internet Platforms</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -883,7 +920,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -894,53 +931,19 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jio-platforms-ltd-prospectus_105427.html</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>Jio Platforms Ltd.</t>
-        </is>
-      </c>
-      <c r="AJ5" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>66.43000000000001</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>21.46</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>67.68000000000001</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>13.99</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>21.36</v>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/jio-platforms-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tonbo Imaging India Limited</t>
+          <t>Jio Platforms Ltd.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -955,7 +958,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Internet Platforms</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -976,29 +984,44 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/tonbo-imaging-india-limited-prospectus_105341.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jio-platforms-ltd-prospectus_105427.html</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>Tonbo Imaging India Ltd.</t>
+          <t>Jio Platforms Ltd.</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>7377</v>
+        <v>1305242</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="AL6" t="n">
-        <v>14.56</v>
+        <v>64.48</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>21.46</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>67.68000000000001</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>21.36</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/tonbo-imaging-india-ltd</t>
+          <t>https://groww.in/stocks/jio-platforms-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-10-30)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR6"/>
+  <dimension ref="A1:AR8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Paras Healthcare Limited</t>
+          <t>BLS Polymers Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -719,12 +719,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Hospitals</t>
+          <t>Chemicals</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -745,72 +745,79 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/paras-healthcare-limited-prospectus_105471.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/bls-polymers-limited-prospectus_105357.html</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>Paras Healthcare Ltd.</t>
-        </is>
-      </c>
-      <c r="AI2" t="n">
-        <v>7976</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>3.53</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>63.95</v>
+          <t>BLS Polymers Ltd</t>
+        </is>
       </c>
       <c r="AM2" t="n">
-        <v>2.22</v>
+        <v>238.64</v>
       </c>
       <c r="AN2" t="n">
-        <v>3.09</v>
+        <v>200.25</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.64</v>
+        <v>558.05</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>3.9</v>
+        <v>123.68</v>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/paras-healthcare-ltd</t>
+          <t>https://groww.in/ipo/bls-polymers-ipo</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INTELLIUS RECODE LIMITED - Notice to Investors</t>
+          <t>Carlsberg India Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>UDRHP</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Beverages</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="T3" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="V3" t="n">
+        <v>22.06</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -819,50 +826,55 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/intellius-recode-limited-notice-to-investors_105445.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/carlsberg-india-limited-udrhp-1_105485.html</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/oct-2026/Carlsberg%20India%20Limited_DA_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oravel Stays Limited</t>
+          <t>Paras Healthcare Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Hospitality</t>
+          <t>Hospitals</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -872,7 +884,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -883,24 +895,61 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/paras-healthcare-limited-prospectus_105471.html</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Paras Healthcare Ltd.</t>
+        </is>
+      </c>
+      <c r="AI4" t="n">
+        <v>8380</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>63.95</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/paras-healthcare-ltd</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Integris Medtech Limited</t>
+          <t>INTELLIUS RECODE LIMITED - Notice to Investors</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -920,7 +969,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -931,14 +980,14 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/intellius-recode-limited-notice-to-investors_105445.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jio Platforms Ltd.</t>
+          <t>Oravel Stays Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -948,22 +997,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Internet Platforms</t>
+          <t>Hospitality</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -973,7 +1022,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -984,42 +1033,143 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/oravel-stays-limited-addendum-to-drhp_105418.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Integris Medtech Limited</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/integris-medtech-limited-addendum-to-drhp_105416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jio Platforms Ltd.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Internet Platforms</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
           <t>https://www.sebi.gov.in/filings/public-issues/oct-2026/jio-platforms-ltd-prospectus_105427.html</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AH8" t="inlineStr">
         <is>
           <t>Jio Platforms Ltd.</t>
         </is>
       </c>
-      <c r="AI6" t="n">
-        <v>1305242</v>
-      </c>
-      <c r="AJ6" t="n">
+      <c r="AI8" t="n">
+        <v>1310491</v>
+      </c>
+      <c r="AJ8" t="n">
         <v>8.949999999999999</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AK8" t="n">
         <v>0.25</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AL8" t="n">
         <v>64.48</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="AM8" t="n">
         <v>21.46</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="AN8" t="n">
         <v>67.68000000000001</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AO8" t="n">
         <v>13.99</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="AP8" t="n">
         <v>2.7</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="AQ8" t="n">
         <v>21.36</v>
       </c>
-      <c r="AR6" t="inlineStr">
+      <c r="AR8" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/jio-platforms-ltd</t>
         </is>

</xml_diff>